<commit_message>
Resultados actualizados - 06-10-mié 16:29
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\web poll\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E17BE2D-CB3C-4055-B074-9C853A5EED31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93159B57-0CEA-47C4-909A-E6E11524CA9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -3102,8 +3102,12 @@
       <c r="W6" s="2">
         <v>0</v>
       </c>
-      <c r="X6" s="2"/>
-      <c r="Y6" s="2"/>
+      <c r="X6" s="2">
+        <v>1</v>
+      </c>
+      <c r="Y6" s="2">
+        <v>1</v>
+      </c>
       <c r="Z6" s="2">
         <v>2</v>
       </c>
@@ -3189,8 +3193,12 @@
       <c r="W7" s="6">
         <v>0</v>
       </c>
-      <c r="X7" s="6"/>
-      <c r="Y7" s="6"/>
+      <c r="X7" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y7" s="6">
+        <v>1</v>
+      </c>
       <c r="Z7" s="6">
         <v>2</v>
       </c>
@@ -6216,6 +6224,7 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AD4:AE4"/>
     <mergeCell ref="AF4:AG4"/>
     <mergeCell ref="A1:AG1"/>
@@ -6232,7 +6241,6 @@
     <mergeCell ref="V4:W4"/>
     <mergeCell ref="X4:Y4"/>
     <mergeCell ref="Z4:AA4"/>
-    <mergeCell ref="AB4:AC4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Resultados actualizados - 06-10-mié 16:30
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93159B57-0CEA-47C4-909A-E6E11524CA9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9DAD269-72E7-424A-9C59-BB6C8FE79067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3102,12 +3102,8 @@
       <c r="W6" s="2">
         <v>0</v>
       </c>
-      <c r="X6" s="2">
-        <v>1</v>
-      </c>
-      <c r="Y6" s="2">
-        <v>1</v>
-      </c>
+      <c r="X6" s="2"/>
+      <c r="Y6" s="2"/>
       <c r="Z6" s="2">
         <v>2</v>
       </c>
@@ -3193,12 +3189,8 @@
       <c r="W7" s="6">
         <v>0</v>
       </c>
-      <c r="X7" s="6">
-        <v>1</v>
-      </c>
-      <c r="Y7" s="6">
-        <v>1</v>
-      </c>
+      <c r="X7" s="6"/>
+      <c r="Y7" s="6"/>
       <c r="Z7" s="6">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Resultados actualizados - 06-10-mié 20:32
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9DAD269-72E7-424A-9C59-BB6C8FE79067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5A3370C-90DD-4042-A6E0-16360CBDD010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3102,8 +3102,12 @@
       <c r="W6" s="2">
         <v>0</v>
       </c>
-      <c r="X6" s="2"/>
-      <c r="Y6" s="2"/>
+      <c r="X6" s="2">
+        <v>2</v>
+      </c>
+      <c r="Y6" s="2">
+        <v>0</v>
+      </c>
       <c r="Z6" s="2">
         <v>2</v>
       </c>
@@ -3189,8 +3193,12 @@
       <c r="W7" s="6">
         <v>0</v>
       </c>
-      <c r="X7" s="6"/>
-      <c r="Y7" s="6"/>
+      <c r="X7" s="6">
+        <v>2</v>
+      </c>
+      <c r="Y7" s="6">
+        <v>1</v>
+      </c>
       <c r="Z7" s="6">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Resultados actualizados - 06-11-jue  9:59
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5A3370C-90DD-4042-A6E0-16360CBDD010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A761C5BE-AB74-428A-AF04-77F0EB629B1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -773,6 +773,9 @@
     <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -780,9 +783,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1058,20 +1058,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
     </row>
     <row r="2" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
     </row>
     <row r="3" spans="1:4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1338,26 +1338,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
     </row>
     <row r="3" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2773,78 +2773,78 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="44"/>
-      <c r="R1" s="44"/>
-      <c r="S1" s="44"/>
-      <c r="T1" s="44"/>
-      <c r="U1" s="44"/>
-      <c r="V1" s="44"/>
-      <c r="W1" s="44"/>
-      <c r="X1" s="44"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="44"/>
-      <c r="AA1" s="44"/>
-      <c r="AB1" s="44"/>
-      <c r="AC1" s="44"/>
-      <c r="AD1" s="44"/>
-      <c r="AE1" s="44"/>
-      <c r="AF1" s="44"/>
-      <c r="AG1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="45"/>
+      <c r="O1" s="45"/>
+      <c r="P1" s="45"/>
+      <c r="Q1" s="45"/>
+      <c r="R1" s="45"/>
+      <c r="S1" s="45"/>
+      <c r="T1" s="45"/>
+      <c r="U1" s="45"/>
+      <c r="V1" s="45"/>
+      <c r="W1" s="45"/>
+      <c r="X1" s="45"/>
+      <c r="Y1" s="45"/>
+      <c r="Z1" s="45"/>
+      <c r="AA1" s="45"/>
+      <c r="AB1" s="45"/>
+      <c r="AC1" s="45"/>
+      <c r="AD1" s="45"/>
+      <c r="AE1" s="45"/>
+      <c r="AF1" s="45"/>
+      <c r="AG1" s="45"/>
     </row>
     <row r="2" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="46" t="s">
         <v>95</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
-      <c r="P2" s="45"/>
-      <c r="Q2" s="45"/>
-      <c r="R2" s="45"/>
-      <c r="S2" s="45"/>
-      <c r="T2" s="45"/>
-      <c r="U2" s="45"/>
-      <c r="V2" s="45"/>
-      <c r="W2" s="45"/>
-      <c r="X2" s="45"/>
-      <c r="Y2" s="45"/>
-      <c r="Z2" s="45"/>
-      <c r="AA2" s="45"/>
-      <c r="AB2" s="45"/>
-      <c r="AC2" s="45"/>
-      <c r="AD2" s="45"/>
-      <c r="AE2" s="45"/>
-      <c r="AF2" s="45"/>
-      <c r="AG2" s="45"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+      <c r="J2" s="46"/>
+      <c r="K2" s="46"/>
+      <c r="L2" s="46"/>
+      <c r="M2" s="46"/>
+      <c r="N2" s="46"/>
+      <c r="O2" s="46"/>
+      <c r="P2" s="46"/>
+      <c r="Q2" s="46"/>
+      <c r="R2" s="46"/>
+      <c r="S2" s="46"/>
+      <c r="T2" s="46"/>
+      <c r="U2" s="46"/>
+      <c r="V2" s="46"/>
+      <c r="W2" s="46"/>
+      <c r="X2" s="46"/>
+      <c r="Y2" s="46"/>
+      <c r="Z2" s="46"/>
+      <c r="AA2" s="46"/>
+      <c r="AB2" s="46"/>
+      <c r="AC2" s="46"/>
+      <c r="AD2" s="46"/>
+      <c r="AE2" s="46"/>
+      <c r="AF2" s="46"/>
+      <c r="AG2" s="46"/>
     </row>
     <row r="3" spans="1:33" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2857,81 +2857,81 @@
       <c r="C4" s="39" t="s">
         <v>97</v>
       </c>
-      <c r="D4" s="47" t="str">
+      <c r="D4" s="44" t="str">
         <f>Participantes!B5</f>
         <v>Andres Jesús</v>
       </c>
-      <c r="E4" s="47"/>
-      <c r="F4" s="47" t="str">
+      <c r="E4" s="44"/>
+      <c r="F4" s="44" t="str">
         <f>Participantes!B6</f>
         <v>Leonardo Fabio</v>
       </c>
-      <c r="G4" s="47"/>
-      <c r="H4" s="47" t="str">
+      <c r="G4" s="44"/>
+      <c r="H4" s="44" t="str">
         <f>Participantes!B7</f>
         <v>Martha Cenidia</v>
       </c>
-      <c r="I4" s="47"/>
-      <c r="J4" s="47" t="str">
+      <c r="I4" s="44"/>
+      <c r="J4" s="44" t="str">
         <f>Participantes!B8</f>
         <v>Freddy Ramón</v>
       </c>
-      <c r="K4" s="47"/>
-      <c r="L4" s="47" t="str">
+      <c r="K4" s="44"/>
+      <c r="L4" s="44" t="str">
         <f>Participantes!B9</f>
         <v xml:space="preserve">Juan Camilo </v>
       </c>
-      <c r="M4" s="47"/>
-      <c r="N4" s="47" t="str">
+      <c r="M4" s="44"/>
+      <c r="N4" s="44" t="str">
         <f>Participantes!B10</f>
         <v xml:space="preserve">Juan David </v>
       </c>
-      <c r="O4" s="47"/>
-      <c r="P4" s="47" t="str">
+      <c r="O4" s="44"/>
+      <c r="P4" s="44" t="str">
         <f>Participantes!B11</f>
         <v>María Trinidad</v>
       </c>
-      <c r="Q4" s="47"/>
-      <c r="R4" s="47" t="str">
+      <c r="Q4" s="44"/>
+      <c r="R4" s="44" t="str">
         <f>Participantes!B12</f>
         <v xml:space="preserve">María Gabriela </v>
       </c>
-      <c r="S4" s="47"/>
-      <c r="T4" s="47" t="str">
+      <c r="S4" s="44"/>
+      <c r="T4" s="44" t="str">
         <f>Participantes!B13</f>
         <v>Laura Valentina</v>
       </c>
-      <c r="U4" s="47"/>
-      <c r="V4" s="47" t="str">
+      <c r="U4" s="44"/>
+      <c r="V4" s="44" t="str">
         <f>Participantes!B14</f>
         <v>Gloria Isabel</v>
       </c>
-      <c r="W4" s="47"/>
-      <c r="X4" s="47" t="str">
+      <c r="W4" s="44"/>
+      <c r="X4" s="44" t="str">
         <f>Participantes!B15</f>
         <v xml:space="preserve">María del Pilar </v>
       </c>
-      <c r="Y4" s="47"/>
-      <c r="Z4" s="47" t="str">
+      <c r="Y4" s="44"/>
+      <c r="Z4" s="44" t="str">
         <f>Participantes!B16</f>
         <v>Jaime Andres</v>
       </c>
-      <c r="AA4" s="47"/>
-      <c r="AB4" s="47" t="str">
+      <c r="AA4" s="44"/>
+      <c r="AB4" s="44" t="str">
         <f>Participantes!B17</f>
         <v>Participante 13</v>
       </c>
-      <c r="AC4" s="47"/>
-      <c r="AD4" s="47" t="str">
+      <c r="AC4" s="44"/>
+      <c r="AD4" s="44" t="str">
         <f>Participantes!B18</f>
         <v>Participante 14</v>
       </c>
-      <c r="AE4" s="47"/>
-      <c r="AF4" s="47" t="str">
+      <c r="AE4" s="44"/>
+      <c r="AF4" s="44" t="str">
         <f>Participantes!B19</f>
         <v>Participante 15</v>
       </c>
-      <c r="AG4" s="47"/>
+      <c r="AG4" s="44"/>
     </row>
     <row r="5" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="40"/>
@@ -3085,10 +3085,10 @@
         <v>1</v>
       </c>
       <c r="R6" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S6" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T6" s="2">
         <v>2</v>
@@ -6224,6 +6224,7 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="Z4:AA4"/>
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AD4:AE4"/>
     <mergeCell ref="AF4:AG4"/>
@@ -6240,7 +6241,6 @@
     <mergeCell ref="T4:U4"/>
     <mergeCell ref="V4:W4"/>
     <mergeCell ref="X4:Y4"/>
-    <mergeCell ref="Z4:AA4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Resultados actualizados - 06-11-jue 16:05
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A761C5BE-AB74-428A-AF04-77F0EB629B1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C8AAE68-9B20-411B-8EA3-9643B76457BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="113">
   <si>
     <t>🏆  QUINIELA MUNDIAL 2026</t>
   </si>
@@ -377,6 +377,9 @@
   </si>
   <si>
     <t>Jaime Andres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   </t>
   </si>
 </sst>
 </file>
@@ -1325,7 +1328,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:N76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -1393,8 +1396,12 @@
       <c r="C5" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
+      <c r="D5" s="13">
+        <v>2</v>
+      </c>
+      <c r="E5" s="13">
+        <v>0</v>
+      </c>
       <c r="F5" s="11" t="s">
         <v>19</v>
       </c>
@@ -1611,7 +1618,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11">
         <v>13</v>
       </c>
@@ -1629,8 +1636,11 @@
       <c r="G17" s="11" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N17" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14">
         <v>14</v>
       </c>
@@ -1649,7 +1659,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11">
         <v>15</v>
       </c>
@@ -1668,7 +1678,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14">
         <v>16</v>
       </c>
@@ -1687,7 +1697,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="11">
         <v>17</v>
       </c>
@@ -1706,7 +1716,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14">
         <v>18</v>
       </c>
@@ -1725,7 +1735,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
         <v>19</v>
       </c>
@@ -1744,7 +1754,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14">
         <v>20</v>
       </c>
@@ -1763,7 +1773,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
         <v>21</v>
       </c>
@@ -1782,7 +1792,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14">
         <v>22</v>
       </c>
@@ -1801,7 +1811,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
         <v>23</v>
       </c>
@@ -1820,7 +1830,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14">
         <v>24</v>
       </c>
@@ -1839,7 +1849,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
         <v>25</v>
       </c>
@@ -1858,7 +1868,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14">
         <v>26</v>
       </c>
@@ -1877,7 +1887,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
         <v>27</v>
       </c>
@@ -1896,7 +1906,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="14">
         <v>28</v>
       </c>
@@ -3040,7 +3050,7 @@
       </c>
       <c r="C6" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D5),Fixture!D5&amp;"-"&amp;Fixture!E5,"")</f>
-        <v/>
+        <v>2-0</v>
       </c>
       <c r="D6" s="2">
         <v>2</v>

</xml_diff>

<commit_message>
Resultados actualizados - 06-11-jue 17:37
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C8AAE68-9B20-411B-8EA3-9643B76457BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1613A4C1-1748-41B2-A2AB-F9F5283FB7BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -776,9 +776,6 @@
     <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -786,6 +783,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1061,20 +1061,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
     </row>
     <row r="2" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
     </row>
     <row r="3" spans="1:4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1341,26 +1341,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="44" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
     </row>
     <row r="3" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2783,78 +2783,78 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="44" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
-      <c r="K1" s="45"/>
-      <c r="L1" s="45"/>
-      <c r="M1" s="45"/>
-      <c r="N1" s="45"/>
-      <c r="O1" s="45"/>
-      <c r="P1" s="45"/>
-      <c r="Q1" s="45"/>
-      <c r="R1" s="45"/>
-      <c r="S1" s="45"/>
-      <c r="T1" s="45"/>
-      <c r="U1" s="45"/>
-      <c r="V1" s="45"/>
-      <c r="W1" s="45"/>
-      <c r="X1" s="45"/>
-      <c r="Y1" s="45"/>
-      <c r="Z1" s="45"/>
-      <c r="AA1" s="45"/>
-      <c r="AB1" s="45"/>
-      <c r="AC1" s="45"/>
-      <c r="AD1" s="45"/>
-      <c r="AE1" s="45"/>
-      <c r="AF1" s="45"/>
-      <c r="AG1" s="45"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
+      <c r="K1" s="44"/>
+      <c r="L1" s="44"/>
+      <c r="M1" s="44"/>
+      <c r="N1" s="44"/>
+      <c r="O1" s="44"/>
+      <c r="P1" s="44"/>
+      <c r="Q1" s="44"/>
+      <c r="R1" s="44"/>
+      <c r="S1" s="44"/>
+      <c r="T1" s="44"/>
+      <c r="U1" s="44"/>
+      <c r="V1" s="44"/>
+      <c r="W1" s="44"/>
+      <c r="X1" s="44"/>
+      <c r="Y1" s="44"/>
+      <c r="Z1" s="44"/>
+      <c r="AA1" s="44"/>
+      <c r="AB1" s="44"/>
+      <c r="AC1" s="44"/>
+      <c r="AD1" s="44"/>
+      <c r="AE1" s="44"/>
+      <c r="AF1" s="44"/>
+      <c r="AG1" s="44"/>
     </row>
     <row r="2" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="45" t="s">
         <v>95</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
-      <c r="N2" s="46"/>
-      <c r="O2" s="46"/>
-      <c r="P2" s="46"/>
-      <c r="Q2" s="46"/>
-      <c r="R2" s="46"/>
-      <c r="S2" s="46"/>
-      <c r="T2" s="46"/>
-      <c r="U2" s="46"/>
-      <c r="V2" s="46"/>
-      <c r="W2" s="46"/>
-      <c r="X2" s="46"/>
-      <c r="Y2" s="46"/>
-      <c r="Z2" s="46"/>
-      <c r="AA2" s="46"/>
-      <c r="AB2" s="46"/>
-      <c r="AC2" s="46"/>
-      <c r="AD2" s="46"/>
-      <c r="AE2" s="46"/>
-      <c r="AF2" s="46"/>
-      <c r="AG2" s="46"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="45"/>
+      <c r="P2" s="45"/>
+      <c r="Q2" s="45"/>
+      <c r="R2" s="45"/>
+      <c r="S2" s="45"/>
+      <c r="T2" s="45"/>
+      <c r="U2" s="45"/>
+      <c r="V2" s="45"/>
+      <c r="W2" s="45"/>
+      <c r="X2" s="45"/>
+      <c r="Y2" s="45"/>
+      <c r="Z2" s="45"/>
+      <c r="AA2" s="45"/>
+      <c r="AB2" s="45"/>
+      <c r="AC2" s="45"/>
+      <c r="AD2" s="45"/>
+      <c r="AE2" s="45"/>
+      <c r="AF2" s="45"/>
+      <c r="AG2" s="45"/>
     </row>
     <row r="3" spans="1:33" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2867,81 +2867,81 @@
       <c r="C4" s="39" t="s">
         <v>97</v>
       </c>
-      <c r="D4" s="44" t="str">
+      <c r="D4" s="47" t="str">
         <f>Participantes!B5</f>
         <v>Andres Jesús</v>
       </c>
-      <c r="E4" s="44"/>
-      <c r="F4" s="44" t="str">
+      <c r="E4" s="47"/>
+      <c r="F4" s="47" t="str">
         <f>Participantes!B6</f>
         <v>Leonardo Fabio</v>
       </c>
-      <c r="G4" s="44"/>
-      <c r="H4" s="44" t="str">
+      <c r="G4" s="47"/>
+      <c r="H4" s="47" t="str">
         <f>Participantes!B7</f>
         <v>Martha Cenidia</v>
       </c>
-      <c r="I4" s="44"/>
-      <c r="J4" s="44" t="str">
+      <c r="I4" s="47"/>
+      <c r="J4" s="47" t="str">
         <f>Participantes!B8</f>
         <v>Freddy Ramón</v>
       </c>
-      <c r="K4" s="44"/>
-      <c r="L4" s="44" t="str">
+      <c r="K4" s="47"/>
+      <c r="L4" s="47" t="str">
         <f>Participantes!B9</f>
         <v xml:space="preserve">Juan Camilo </v>
       </c>
-      <c r="M4" s="44"/>
-      <c r="N4" s="44" t="str">
+      <c r="M4" s="47"/>
+      <c r="N4" s="47" t="str">
         <f>Participantes!B10</f>
         <v xml:space="preserve">Juan David </v>
       </c>
-      <c r="O4" s="44"/>
-      <c r="P4" s="44" t="str">
+      <c r="O4" s="47"/>
+      <c r="P4" s="47" t="str">
         <f>Participantes!B11</f>
         <v>María Trinidad</v>
       </c>
-      <c r="Q4" s="44"/>
-      <c r="R4" s="44" t="str">
+      <c r="Q4" s="47"/>
+      <c r="R4" s="47" t="str">
         <f>Participantes!B12</f>
         <v xml:space="preserve">María Gabriela </v>
       </c>
-      <c r="S4" s="44"/>
-      <c r="T4" s="44" t="str">
+      <c r="S4" s="47"/>
+      <c r="T4" s="47" t="str">
         <f>Participantes!B13</f>
         <v>Laura Valentina</v>
       </c>
-      <c r="U4" s="44"/>
-      <c r="V4" s="44" t="str">
+      <c r="U4" s="47"/>
+      <c r="V4" s="47" t="str">
         <f>Participantes!B14</f>
         <v>Gloria Isabel</v>
       </c>
-      <c r="W4" s="44"/>
-      <c r="X4" s="44" t="str">
+      <c r="W4" s="47"/>
+      <c r="X4" s="47" t="str">
         <f>Participantes!B15</f>
         <v xml:space="preserve">María del Pilar </v>
       </c>
-      <c r="Y4" s="44"/>
-      <c r="Z4" s="44" t="str">
+      <c r="Y4" s="47"/>
+      <c r="Z4" s="47" t="str">
         <f>Participantes!B16</f>
         <v>Jaime Andres</v>
       </c>
-      <c r="AA4" s="44"/>
-      <c r="AB4" s="44" t="str">
+      <c r="AA4" s="47"/>
+      <c r="AB4" s="47" t="str">
         <f>Participantes!B17</f>
         <v>Participante 13</v>
       </c>
-      <c r="AC4" s="44"/>
-      <c r="AD4" s="44" t="str">
+      <c r="AC4" s="47"/>
+      <c r="AD4" s="47" t="str">
         <f>Participantes!B18</f>
         <v>Participante 14</v>
       </c>
-      <c r="AE4" s="44"/>
-      <c r="AF4" s="44" t="str">
+      <c r="AE4" s="47"/>
+      <c r="AF4" s="47" t="str">
         <f>Participantes!B19</f>
         <v>Participante 15</v>
       </c>
-      <c r="AG4" s="44"/>
+      <c r="AG4" s="47"/>
     </row>
     <row r="5" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="40"/>
@@ -3406,18 +3406,34 @@
         <f>IF(ISNUMBER(Fixture!D11),Fixture!D11&amp;"-"&amp;Fixture!E11,"")</f>
         <v/>
       </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
+      <c r="D12" s="2">
+        <v>0</v>
+      </c>
+      <c r="E12" s="2">
+        <v>2</v>
+      </c>
+      <c r="F12" s="2">
+        <v>2</v>
+      </c>
+      <c r="G12" s="2">
+        <v>0</v>
+      </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
+      <c r="J12" s="2">
+        <v>1</v>
+      </c>
+      <c r="K12" s="2">
+        <v>1</v>
+      </c>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
-      <c r="N12" s="2"/>
-      <c r="O12" s="2"/>
+      <c r="N12" s="2">
+        <v>1</v>
+      </c>
+      <c r="O12" s="2">
+        <v>1</v>
+      </c>
       <c r="P12" s="2"/>
       <c r="Q12" s="2"/>
       <c r="R12" s="2"/>
@@ -3922,18 +3938,34 @@
         <f>IF(ISNUMBER(Fixture!D23),Fixture!D23&amp;"-"&amp;Fixture!E23,"")</f>
         <v/>
       </c>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
+      <c r="D24" s="2">
+        <v>1</v>
+      </c>
+      <c r="E24" s="2">
+        <v>0</v>
+      </c>
+      <c r="F24" s="2">
+        <v>0</v>
+      </c>
+      <c r="G24" s="2">
+        <v>1</v>
+      </c>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
+      <c r="J24" s="2">
+        <v>3</v>
+      </c>
+      <c r="K24" s="2">
+        <v>1</v>
+      </c>
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2"/>
+      <c r="N24" s="2">
+        <v>1</v>
+      </c>
+      <c r="O24" s="2">
+        <v>2</v>
+      </c>
       <c r="P24" s="2"/>
       <c r="Q24" s="2"/>
       <c r="R24" s="2"/>
@@ -6234,6 +6266,7 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="X4:Y4"/>
     <mergeCell ref="Z4:AA4"/>
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AD4:AE4"/>
@@ -6250,7 +6283,6 @@
     <mergeCell ref="R4:S4"/>
     <mergeCell ref="T4:U4"/>
     <mergeCell ref="V4:W4"/>
-    <mergeCell ref="X4:Y4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Resultados actualizados - 06-11-jue 17:44
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1613A4C1-1748-41B2-A2AB-F9F5283FB7BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C558FEF-C70F-4369-915E-D603CB08D3DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3418,8 +3418,12 @@
       <c r="G12" s="2">
         <v>0</v>
       </c>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
+      <c r="H12" s="2">
+        <v>2</v>
+      </c>
+      <c r="I12" s="2">
+        <v>2</v>
+      </c>
       <c r="J12" s="2">
         <v>1</v>
       </c>
@@ -3438,14 +3442,22 @@
       <c r="Q12" s="2"/>
       <c r="R12" s="2"/>
       <c r="S12" s="2"/>
-      <c r="T12" s="2"/>
-      <c r="U12" s="2"/>
+      <c r="T12" s="2">
+        <v>1</v>
+      </c>
+      <c r="U12" s="2">
+        <v>0</v>
+      </c>
       <c r="V12" s="2"/>
       <c r="W12" s="2"/>
       <c r="X12" s="2"/>
       <c r="Y12" s="2"/>
-      <c r="Z12" s="2"/>
-      <c r="AA12" s="2"/>
+      <c r="Z12" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA12" s="2">
+        <v>0</v>
+      </c>
       <c r="AB12" s="2"/>
       <c r="AC12" s="2"/>
       <c r="AD12" s="2"/>
@@ -3939,7 +3951,7 @@
         <v/>
       </c>
       <c r="D24" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E24" s="2">
         <v>0</v>
@@ -3950,8 +3962,12 @@
       <c r="G24" s="2">
         <v>1</v>
       </c>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
+      <c r="H24" s="2">
+        <v>1</v>
+      </c>
+      <c r="I24" s="2">
+        <v>0</v>
+      </c>
       <c r="J24" s="2">
         <v>3</v>
       </c>
@@ -3970,14 +3986,22 @@
       <c r="Q24" s="2"/>
       <c r="R24" s="2"/>
       <c r="S24" s="2"/>
-      <c r="T24" s="2"/>
-      <c r="U24" s="2"/>
+      <c r="T24" s="2">
+        <v>2</v>
+      </c>
+      <c r="U24" s="2">
+        <v>1</v>
+      </c>
       <c r="V24" s="2"/>
       <c r="W24" s="2"/>
       <c r="X24" s="2"/>
       <c r="Y24" s="2"/>
-      <c r="Z24" s="2"/>
-      <c r="AA24" s="2"/>
+      <c r="Z24" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA24" s="2">
+        <v>1</v>
+      </c>
       <c r="AB24" s="2"/>
       <c r="AC24" s="2"/>
       <c r="AD24" s="2"/>

</xml_diff>

<commit_message>
Resultados actualizados - 06-11-jue 17:47
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C558FEF-C70F-4369-915E-D603CB08D3DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{635958BF-2B18-4599-B0C4-20358C93FDC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3440,8 +3440,12 @@
       </c>
       <c r="P12" s="2"/>
       <c r="Q12" s="2"/>
-      <c r="R12" s="2"/>
-      <c r="S12" s="2"/>
+      <c r="R12" s="2">
+        <v>1</v>
+      </c>
+      <c r="S12" s="2">
+        <v>0</v>
+      </c>
       <c r="T12" s="2">
         <v>1</v>
       </c>
@@ -3984,8 +3988,12 @@
       </c>
       <c r="P24" s="2"/>
       <c r="Q24" s="2"/>
-      <c r="R24" s="2"/>
-      <c r="S24" s="2"/>
+      <c r="R24" s="2">
+        <v>2</v>
+      </c>
+      <c r="S24" s="2">
+        <v>1</v>
+      </c>
       <c r="T24" s="2">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Actualizar - 06-11-jue 17:56
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{635958BF-2B18-4599-B0C4-20358C93FDC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E4F30A0-E2A9-42BF-8CFC-E4393C033696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3452,8 +3452,12 @@
       <c r="U12" s="2">
         <v>0</v>
       </c>
-      <c r="V12" s="2"/>
-      <c r="W12" s="2"/>
+      <c r="V12" s="2">
+        <v>1</v>
+      </c>
+      <c r="W12" s="2">
+        <v>1</v>
+      </c>
       <c r="X12" s="2"/>
       <c r="Y12" s="2"/>
       <c r="Z12" s="2">
@@ -4000,8 +4004,12 @@
       <c r="U24" s="2">
         <v>1</v>
       </c>
-      <c r="V24" s="2"/>
-      <c r="W24" s="2"/>
+      <c r="V24" s="2">
+        <v>1</v>
+      </c>
+      <c r="W24" s="2">
+        <v>1</v>
+      </c>
       <c r="X24" s="2"/>
       <c r="Y24" s="2"/>
       <c r="Z24" s="2">

</xml_diff>

<commit_message>
Actualizar - 06-11-jue 22:13
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E4F30A0-E2A9-42BF-8CFC-E4393C033696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9683E97-E8CF-4D22-AB3B-2F3ADC29CB21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3458,8 +3458,12 @@
       <c r="W12" s="2">
         <v>1</v>
       </c>
-      <c r="X12" s="2"/>
-      <c r="Y12" s="2"/>
+      <c r="X12" s="2">
+        <v>1</v>
+      </c>
+      <c r="Y12" s="2">
+        <v>1</v>
+      </c>
       <c r="Z12" s="2">
         <v>2</v>
       </c>
@@ -4010,8 +4014,12 @@
       <c r="W24" s="2">
         <v>1</v>
       </c>
-      <c r="X24" s="2"/>
-      <c r="Y24" s="2"/>
+      <c r="X24" s="2">
+        <v>2</v>
+      </c>
+      <c r="Y24" s="2">
+        <v>1</v>
+      </c>
       <c r="Z24" s="2">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Actualizar - 06-11-jue 22:57
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9683E97-E8CF-4D22-AB3B-2F3ADC29CB21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B23521AA-C360-43ED-A47C-B480EC485C5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1419,8 +1419,12 @@
       <c r="C6" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
+      <c r="D6" s="13">
+        <v>2</v>
+      </c>
+      <c r="E6" s="13">
+        <v>1</v>
+      </c>
       <c r="F6" s="14" t="s">
         <v>22</v>
       </c>
@@ -3141,7 +3145,7 @@
       </c>
       <c r="C7" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D6),Fixture!D6&amp;"-"&amp;Fixture!E6,"")</f>
-        <v/>
+        <v>2-1</v>
       </c>
       <c r="D7" s="6">
         <v>1</v>

</xml_diff>

<commit_message>
Actualizar - 06-12-vie  9:13
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B23521AA-C360-43ED-A47C-B480EC485C5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21BF9623-2270-4099-BB78-7BF198518D2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3442,8 +3442,12 @@
       <c r="O12" s="2">
         <v>1</v>
       </c>
-      <c r="P12" s="2"/>
-      <c r="Q12" s="2"/>
+      <c r="P12" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>0</v>
+      </c>
       <c r="R12" s="2">
         <v>1</v>
       </c>
@@ -3998,8 +4002,12 @@
       <c r="O24" s="2">
         <v>2</v>
       </c>
-      <c r="P24" s="2"/>
-      <c r="Q24" s="2"/>
+      <c r="P24" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q24" s="2">
+        <v>1</v>
+      </c>
       <c r="R24" s="2">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Actualizar - 06-12-vie 10:43
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21BF9623-2270-4099-BB78-7BF198518D2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB34F21E-96A0-45D0-BA89-A223D1F07CE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3434,8 +3434,12 @@
       <c r="K12" s="2">
         <v>1</v>
       </c>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
+      <c r="L12" s="2">
+        <v>2</v>
+      </c>
+      <c r="M12" s="2">
+        <v>0</v>
+      </c>
       <c r="N12" s="2">
         <v>1</v>
       </c>
@@ -3994,8 +3998,12 @@
       <c r="K24" s="2">
         <v>1</v>
       </c>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
+      <c r="L24" s="2">
+        <v>1</v>
+      </c>
+      <c r="M24" s="2">
+        <v>2</v>
+      </c>
       <c r="N24" s="2">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Actualizar - 06-12-vie 16:03
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB34F21E-96A0-45D0-BA89-A223D1F07CE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA7B7EA0-C22A-4CF9-923F-206A6A50E1C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -1442,8 +1442,12 @@
       <c r="C7" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
+      <c r="D7" s="13">
+        <v>1</v>
+      </c>
+      <c r="E7" s="13">
+        <v>1</v>
+      </c>
       <c r="F7" s="11" t="s">
         <v>19</v>
       </c>
@@ -3236,7 +3240,7 @@
       </c>
       <c r="C8" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D7),Fixture!D7&amp;"-"&amp;Fixture!E7,"")</f>
-        <v/>
+        <v>1-1</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>

</xml_diff>

<commit_message>
Actualizar - 06-12-vie 16:21
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B26497EF-04BB-4547-8956-F2726FFBD0E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8306F1D-F97D-4817-9A85-62786DAE26D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -3505,14 +3505,22 @@
         <f>IF(ISNUMBER(Fixture!D12),Fixture!D12&amp;"-"&amp;Fixture!E12,"")</f>
         <v/>
       </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
+      <c r="D13" s="6">
+        <v>0</v>
+      </c>
+      <c r="E13" s="6">
+        <v>2</v>
+      </c>
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
+      <c r="J13" s="6">
+        <v>2</v>
+      </c>
+      <c r="K13" s="6">
+        <v>1</v>
+      </c>
       <c r="L13" s="6"/>
       <c r="M13" s="6"/>
       <c r="N13" s="6"/>
@@ -3720,14 +3728,22 @@
         <f>IF(ISNUMBER(Fixture!D17),Fixture!D17&amp;"-"&amp;Fixture!E17,"")</f>
         <v/>
       </c>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
+      <c r="D18" s="2">
+        <v>1</v>
+      </c>
+      <c r="E18" s="2">
+        <v>1</v>
+      </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
+      <c r="J18" s="2">
+        <v>2</v>
+      </c>
+      <c r="K18" s="2">
+        <v>2</v>
+      </c>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
       <c r="N18" s="2"/>
@@ -3763,14 +3779,22 @@
         <f>IF(ISNUMBER(Fixture!D18),Fixture!D18&amp;"-"&amp;Fixture!E18,"")</f>
         <v/>
       </c>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
+      <c r="D19" s="6">
+        <v>0</v>
+      </c>
+      <c r="E19" s="6">
+        <v>2</v>
+      </c>
       <c r="F19" s="6"/>
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
       <c r="I19" s="6"/>
-      <c r="J19" s="6"/>
-      <c r="K19" s="6"/>
+      <c r="J19" s="6">
+        <v>0</v>
+      </c>
+      <c r="K19" s="6">
+        <v>4</v>
+      </c>
       <c r="L19" s="6"/>
       <c r="M19" s="6"/>
       <c r="N19" s="6"/>
@@ -4069,14 +4093,22 @@
         <f>IF(ISNUMBER(Fixture!D24),Fixture!D24&amp;"-"&amp;Fixture!E24,"")</f>
         <v/>
       </c>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
+      <c r="D25" s="6">
+        <v>1</v>
+      </c>
+      <c r="E25" s="6">
+        <v>2</v>
+      </c>
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
       <c r="H25" s="6"/>
       <c r="I25" s="6"/>
-      <c r="J25" s="6"/>
-      <c r="K25" s="6"/>
+      <c r="J25" s="6">
+        <v>0</v>
+      </c>
+      <c r="K25" s="6">
+        <v>2</v>
+      </c>
       <c r="L25" s="6"/>
       <c r="M25" s="6"/>
       <c r="N25" s="6"/>

</xml_diff>

<commit_message>
Actualizar - 06-12-vie 16:32
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8306F1D-F97D-4817-9A85-62786DAE26D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{863AAF41-C570-47CB-8DB1-9F1037418D56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3513,8 +3513,12 @@
       </c>
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
+      <c r="H13" s="6">
+        <v>0</v>
+      </c>
+      <c r="I13" s="6">
+        <v>2</v>
+      </c>
       <c r="J13" s="6">
         <v>2</v>
       </c>
@@ -3523,16 +3527,24 @@
       </c>
       <c r="L13" s="6"/>
       <c r="M13" s="6"/>
-      <c r="N13" s="6"/>
-      <c r="O13" s="6"/>
+      <c r="N13" s="6">
+        <v>0</v>
+      </c>
+      <c r="O13" s="6">
+        <v>2</v>
+      </c>
       <c r="P13" s="6"/>
       <c r="Q13" s="6"/>
       <c r="R13" s="6"/>
       <c r="S13" s="6"/>
       <c r="T13" s="6"/>
       <c r="U13" s="6"/>
-      <c r="V13" s="6"/>
-      <c r="W13" s="6"/>
+      <c r="V13" s="6">
+        <v>1</v>
+      </c>
+      <c r="W13" s="6">
+        <v>2</v>
+      </c>
       <c r="X13" s="6"/>
       <c r="Y13" s="6"/>
       <c r="Z13" s="6"/>
@@ -3736,8 +3748,12 @@
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
+      <c r="H18" s="2">
+        <v>2</v>
+      </c>
+      <c r="I18" s="2">
+        <v>1</v>
+      </c>
       <c r="J18" s="2">
         <v>2</v>
       </c>
@@ -3746,16 +3762,24 @@
       </c>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2"/>
+      <c r="N18" s="2">
+        <v>2</v>
+      </c>
+      <c r="O18" s="2">
+        <v>1</v>
+      </c>
       <c r="P18" s="2"/>
       <c r="Q18" s="2"/>
       <c r="R18" s="2"/>
       <c r="S18" s="2"/>
       <c r="T18" s="2"/>
       <c r="U18" s="2"/>
-      <c r="V18" s="2"/>
-      <c r="W18" s="2"/>
+      <c r="V18" s="2">
+        <v>2</v>
+      </c>
+      <c r="W18" s="2">
+        <v>2</v>
+      </c>
       <c r="X18" s="2"/>
       <c r="Y18" s="2"/>
       <c r="Z18" s="2"/>
@@ -3787,8 +3811,12 @@
       </c>
       <c r="F19" s="6"/>
       <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="6"/>
+      <c r="H19" s="6">
+        <v>0</v>
+      </c>
+      <c r="I19" s="6">
+        <v>2</v>
+      </c>
       <c r="J19" s="6">
         <v>0</v>
       </c>
@@ -3797,16 +3825,24 @@
       </c>
       <c r="L19" s="6"/>
       <c r="M19" s="6"/>
-      <c r="N19" s="6"/>
-      <c r="O19" s="6"/>
+      <c r="N19" s="6">
+        <v>0</v>
+      </c>
+      <c r="O19" s="6">
+        <v>3</v>
+      </c>
       <c r="P19" s="6"/>
       <c r="Q19" s="6"/>
       <c r="R19" s="6"/>
       <c r="S19" s="6"/>
       <c r="T19" s="6"/>
       <c r="U19" s="6"/>
-      <c r="V19" s="6"/>
-      <c r="W19" s="6"/>
+      <c r="V19" s="6">
+        <v>0</v>
+      </c>
+      <c r="W19" s="6">
+        <v>2</v>
+      </c>
       <c r="X19" s="6"/>
       <c r="Y19" s="6"/>
       <c r="Z19" s="6"/>
@@ -4101,8 +4137,12 @@
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
-      <c r="H25" s="6"/>
-      <c r="I25" s="6"/>
+      <c r="H25" s="6">
+        <v>1</v>
+      </c>
+      <c r="I25" s="6">
+        <v>1</v>
+      </c>
       <c r="J25" s="6">
         <v>0</v>
       </c>
@@ -4111,16 +4151,24 @@
       </c>
       <c r="L25" s="6"/>
       <c r="M25" s="6"/>
-      <c r="N25" s="6"/>
-      <c r="O25" s="6"/>
+      <c r="N25" s="6">
+        <v>1</v>
+      </c>
+      <c r="O25" s="6">
+        <v>3</v>
+      </c>
       <c r="P25" s="6"/>
       <c r="Q25" s="6"/>
       <c r="R25" s="6"/>
       <c r="S25" s="6"/>
       <c r="T25" s="6"/>
       <c r="U25" s="6"/>
-      <c r="V25" s="6"/>
-      <c r="W25" s="6"/>
+      <c r="V25" s="6">
+        <v>1</v>
+      </c>
+      <c r="W25" s="6">
+        <v>2</v>
+      </c>
       <c r="X25" s="6"/>
       <c r="Y25" s="6"/>
       <c r="Z25" s="6"/>

</xml_diff>

<commit_message>
Actualizar - 06-12-vie 16:52
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{863AAF41-C570-47CB-8DB1-9F1037418D56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19C3EF6F-8B77-4BF7-BB1B-54D8EA7834E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3537,8 +3537,12 @@
       <c r="Q13" s="6"/>
       <c r="R13" s="6"/>
       <c r="S13" s="6"/>
-      <c r="T13" s="6"/>
-      <c r="U13" s="6"/>
+      <c r="T13" s="6">
+        <v>0</v>
+      </c>
+      <c r="U13" s="6">
+        <v>2</v>
+      </c>
       <c r="V13" s="6">
         <v>1</v>
       </c>
@@ -3772,8 +3776,12 @@
       <c r="Q18" s="2"/>
       <c r="R18" s="2"/>
       <c r="S18" s="2"/>
-      <c r="T18" s="2"/>
-      <c r="U18" s="2"/>
+      <c r="T18" s="2">
+        <v>2</v>
+      </c>
+      <c r="U18" s="2">
+        <v>1</v>
+      </c>
       <c r="V18" s="2">
         <v>2</v>
       </c>
@@ -3835,8 +3843,12 @@
       <c r="Q19" s="6"/>
       <c r="R19" s="6"/>
       <c r="S19" s="6"/>
-      <c r="T19" s="6"/>
-      <c r="U19" s="6"/>
+      <c r="T19" s="6">
+        <v>0</v>
+      </c>
+      <c r="U19" s="6">
+        <v>2</v>
+      </c>
       <c r="V19" s="6">
         <v>0</v>
       </c>
@@ -4161,8 +4173,12 @@
       <c r="Q25" s="6"/>
       <c r="R25" s="6"/>
       <c r="S25" s="6"/>
-      <c r="T25" s="6"/>
-      <c r="U25" s="6"/>
+      <c r="T25" s="6">
+        <v>1</v>
+      </c>
+      <c r="U25" s="6">
+        <v>2</v>
+      </c>
       <c r="V25" s="6">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Actualizar - 06-12-vie 18:44
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19C3EF6F-8B77-4BF7-BB1B-54D8EA7834E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED5B3137-37AE-4064-94A6-BCEEA5A080FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -3549,8 +3549,12 @@
       <c r="W13" s="6">
         <v>2</v>
       </c>
-      <c r="X13" s="6"/>
-      <c r="Y13" s="6"/>
+      <c r="X13" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="6">
+        <v>3</v>
+      </c>
       <c r="Z13" s="6"/>
       <c r="AA13" s="6"/>
       <c r="AB13" s="6"/>
@@ -3788,8 +3792,12 @@
       <c r="W18" s="2">
         <v>2</v>
       </c>
-      <c r="X18" s="2"/>
-      <c r="Y18" s="2"/>
+      <c r="X18" s="2">
+        <v>2</v>
+      </c>
+      <c r="Y18" s="2">
+        <v>1</v>
+      </c>
       <c r="Z18" s="2"/>
       <c r="AA18" s="2"/>
       <c r="AB18" s="2"/>
@@ -3855,8 +3863,12 @@
       <c r="W19" s="6">
         <v>2</v>
       </c>
-      <c r="X19" s="6"/>
-      <c r="Y19" s="6"/>
+      <c r="X19" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y19" s="6">
+        <v>3</v>
+      </c>
       <c r="Z19" s="6"/>
       <c r="AA19" s="6"/>
       <c r="AB19" s="6"/>
@@ -4185,8 +4197,12 @@
       <c r="W25" s="6">
         <v>2</v>
       </c>
-      <c r="X25" s="6"/>
-      <c r="Y25" s="6"/>
+      <c r="X25" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y25" s="6">
+        <v>1</v>
+      </c>
       <c r="Z25" s="6"/>
       <c r="AA25" s="6"/>
       <c r="AB25" s="6"/>

</xml_diff>

<commit_message>
Actualizar - 06-12-vie 22:08
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED5B3137-37AE-4064-94A6-BCEEA5A080FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E58426A-980F-4C11-A098-3F932AC659B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -1753,8 +1753,12 @@
       <c r="C23" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
+      <c r="D23" s="13">
+        <v>4</v>
+      </c>
+      <c r="E23" s="13">
+        <v>1</v>
+      </c>
       <c r="F23" s="11" t="s">
         <v>40</v>
       </c>
@@ -4060,7 +4064,7 @@
       </c>
       <c r="C24" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D23),Fixture!D23&amp;"-"&amp;Fixture!E23,"")</f>
-        <v/>
+        <v>4-1</v>
       </c>
       <c r="D24" s="2">
         <v>2</v>

</xml_diff>

<commit_message>
Actualizar - 06-13-sáb 14:11
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E58426A-980F-4C11-A098-3F932AC659B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FADCF7FC-4A43-4339-9981-0AE6864EFEB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -3515,8 +3515,12 @@
       <c r="E13" s="6">
         <v>2</v>
       </c>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
+      <c r="F13" s="6">
+        <v>0</v>
+      </c>
+      <c r="G13" s="6">
+        <v>2</v>
+      </c>
       <c r="H13" s="6">
         <v>0</v>
       </c>
@@ -3529,8 +3533,12 @@
       <c r="K13" s="6">
         <v>1</v>
       </c>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
+      <c r="L13" s="6">
+        <v>0</v>
+      </c>
+      <c r="M13" s="6">
+        <v>3</v>
+      </c>
       <c r="N13" s="6">
         <v>0</v>
       </c>
@@ -3758,8 +3766,12 @@
       <c r="E18" s="2">
         <v>1</v>
       </c>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
+      <c r="F18" s="2">
+        <v>1</v>
+      </c>
+      <c r="G18" s="2">
+        <v>0</v>
+      </c>
       <c r="H18" s="2">
         <v>2</v>
       </c>
@@ -3772,8 +3784,12 @@
       <c r="K18" s="2">
         <v>2</v>
       </c>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2"/>
+      <c r="L18" s="2">
+        <v>2</v>
+      </c>
+      <c r="M18" s="2">
+        <v>1</v>
+      </c>
       <c r="N18" s="2">
         <v>2</v>
       </c>
@@ -3802,8 +3818,12 @@
       <c r="Y18" s="2">
         <v>1</v>
       </c>
-      <c r="Z18" s="2"/>
-      <c r="AA18" s="2"/>
+      <c r="Z18" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA18" s="2">
+        <v>0</v>
+      </c>
       <c r="AB18" s="2"/>
       <c r="AC18" s="2"/>
       <c r="AD18" s="2"/>
@@ -3829,8 +3849,12 @@
       <c r="E19" s="6">
         <v>2</v>
       </c>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
+      <c r="F19" s="6">
+        <v>1</v>
+      </c>
+      <c r="G19" s="6">
+        <v>2</v>
+      </c>
       <c r="H19" s="6">
         <v>0</v>
       </c>
@@ -3843,8 +3867,12 @@
       <c r="K19" s="6">
         <v>4</v>
       </c>
-      <c r="L19" s="6"/>
-      <c r="M19" s="6"/>
+      <c r="L19" s="6">
+        <v>0</v>
+      </c>
+      <c r="M19" s="6">
+        <v>2</v>
+      </c>
       <c r="N19" s="6">
         <v>0</v>
       </c>
@@ -3873,8 +3901,12 @@
       <c r="Y19" s="6">
         <v>3</v>
       </c>
-      <c r="Z19" s="6"/>
-      <c r="AA19" s="6"/>
+      <c r="Z19" s="6">
+        <v>1</v>
+      </c>
+      <c r="AA19" s="6">
+        <v>1</v>
+      </c>
       <c r="AB19" s="6"/>
       <c r="AC19" s="6"/>
       <c r="AD19" s="6"/>
@@ -4163,8 +4195,12 @@
       <c r="E25" s="6">
         <v>2</v>
       </c>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
+      <c r="F25" s="6">
+        <v>1</v>
+      </c>
+      <c r="G25" s="6">
+        <v>1</v>
+      </c>
       <c r="H25" s="6">
         <v>1</v>
       </c>
@@ -4177,8 +4213,12 @@
       <c r="K25" s="6">
         <v>2</v>
       </c>
-      <c r="L25" s="6"/>
-      <c r="M25" s="6"/>
+      <c r="L25" s="6">
+        <v>1</v>
+      </c>
+      <c r="M25" s="6">
+        <v>1</v>
+      </c>
       <c r="N25" s="6">
         <v>1</v>
       </c>
@@ -4207,8 +4247,12 @@
       <c r="Y25" s="6">
         <v>1</v>
       </c>
-      <c r="Z25" s="6"/>
-      <c r="AA25" s="6"/>
+      <c r="Z25" s="6">
+        <v>2</v>
+      </c>
+      <c r="AA25" s="6">
+        <v>1</v>
+      </c>
       <c r="AB25" s="6"/>
       <c r="AC25" s="6"/>
       <c r="AD25" s="6"/>
@@ -6454,11 +6498,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="X4:Y4"/>
-    <mergeCell ref="Z4:AA4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AD4:AE4"/>
-    <mergeCell ref="AF4:AG4"/>
     <mergeCell ref="A1:AG1"/>
     <mergeCell ref="A2:AG2"/>
     <mergeCell ref="D4:E4"/>
@@ -6471,6 +6510,11 @@
     <mergeCell ref="R4:S4"/>
     <mergeCell ref="T4:U4"/>
     <mergeCell ref="V4:W4"/>
+    <mergeCell ref="X4:Y4"/>
+    <mergeCell ref="Z4:AA4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AD4:AE4"/>
+    <mergeCell ref="AF4:AG4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Actualizar - 06-13-sáb 14:19
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FADCF7FC-4A43-4339-9981-0AE6864EFEB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{359422AC-2F5D-48C8-AF70-F45E8A1B7DD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4247,12 +4247,8 @@
       <c r="Y25" s="6">
         <v>1</v>
       </c>
-      <c r="Z25" s="6">
-        <v>2</v>
-      </c>
-      <c r="AA25" s="6">
-        <v>1</v>
-      </c>
+      <c r="Z25" s="6"/>
+      <c r="AA25" s="6"/>
       <c r="AB25" s="6"/>
       <c r="AC25" s="6"/>
       <c r="AD25" s="6"/>
@@ -4444,8 +4440,12 @@
         <f>IF(ISNUMBER(Fixture!D29),Fixture!D29&amp;"-"&amp;Fixture!E29,"")</f>
         <v/>
       </c>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
+      <c r="D30" s="2">
+        <v>5</v>
+      </c>
+      <c r="E30" s="2">
+        <v>0</v>
+      </c>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
@@ -4454,8 +4454,12 @@
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
       <c r="M30" s="2"/>
-      <c r="N30" s="2"/>
-      <c r="O30" s="2"/>
+      <c r="N30" s="2">
+        <v>6</v>
+      </c>
+      <c r="O30" s="2">
+        <v>0</v>
+      </c>
       <c r="P30" s="2"/>
       <c r="Q30" s="2"/>
       <c r="R30" s="2"/>
@@ -4487,8 +4491,12 @@
         <f>IF(ISNUMBER(Fixture!D30),Fixture!D30&amp;"-"&amp;Fixture!E30,"")</f>
         <v/>
       </c>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
+      <c r="D31" s="6">
+        <v>1</v>
+      </c>
+      <c r="E31" s="6">
+        <v>1</v>
+      </c>
       <c r="F31" s="6"/>
       <c r="G31" s="6"/>
       <c r="H31" s="6"/>
@@ -4497,8 +4505,12 @@
       <c r="K31" s="6"/>
       <c r="L31" s="6"/>
       <c r="M31" s="6"/>
-      <c r="N31" s="6"/>
-      <c r="O31" s="6"/>
+      <c r="N31" s="6">
+        <v>0</v>
+      </c>
+      <c r="O31" s="6">
+        <v>1</v>
+      </c>
       <c r="P31" s="6"/>
       <c r="Q31" s="6"/>
       <c r="R31" s="6"/>
@@ -4702,8 +4714,12 @@
         <f>IF(ISNUMBER(Fixture!D35),Fixture!D35&amp;"-"&amp;Fixture!E35,"")</f>
         <v/>
       </c>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
+      <c r="D36" s="2">
+        <v>2</v>
+      </c>
+      <c r="E36" s="2">
+        <v>2</v>
+      </c>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
@@ -4712,8 +4728,12 @@
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
       <c r="M36" s="2"/>
-      <c r="N36" s="2"/>
-      <c r="O36" s="2"/>
+      <c r="N36" s="2">
+        <v>2</v>
+      </c>
+      <c r="O36" s="2">
+        <v>1</v>
+      </c>
       <c r="P36" s="2"/>
       <c r="Q36" s="2"/>
       <c r="R36" s="2"/>
@@ -4745,8 +4765,12 @@
         <f>IF(ISNUMBER(Fixture!D36),Fixture!D36&amp;"-"&amp;Fixture!E36,"")</f>
         <v/>
       </c>
-      <c r="D37" s="6"/>
-      <c r="E37" s="6"/>
+      <c r="D37" s="6">
+        <v>2</v>
+      </c>
+      <c r="E37" s="6">
+        <v>0</v>
+      </c>
       <c r="F37" s="6"/>
       <c r="G37" s="6"/>
       <c r="H37" s="6"/>
@@ -4755,8 +4779,12 @@
       <c r="K37" s="6"/>
       <c r="L37" s="6"/>
       <c r="M37" s="6"/>
-      <c r="N37" s="6"/>
-      <c r="O37" s="6"/>
+      <c r="N37" s="6">
+        <v>2</v>
+      </c>
+      <c r="O37" s="6">
+        <v>0</v>
+      </c>
       <c r="P37" s="6"/>
       <c r="Q37" s="6"/>
       <c r="R37" s="6"/>

</xml_diff>

<commit_message>
Actualizar - 06-13-sáb 16:06
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{359422AC-2F5D-48C8-AF70-F45E8A1B7DD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6088B18E-C197-4FB4-8132-E12A4BEDDEC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -1541,8 +1541,12 @@
       <c r="C12" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
+      <c r="D12" s="13">
+        <v>1</v>
+      </c>
+      <c r="E12" s="13">
+        <v>1</v>
+      </c>
       <c r="F12" s="14" t="s">
         <v>30</v>
       </c>
@@ -3507,7 +3511,7 @@
       </c>
       <c r="C13" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D12),Fixture!D12&amp;"-"&amp;Fixture!E12,"")</f>
-        <v/>
+        <v>1-1</v>
       </c>
       <c r="D13" s="6">
         <v>0</v>

</xml_diff>

<commit_message>
Actualizar - 06-13-sáb 19:06
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6088B18E-C197-4FB4-8132-E12A4BEDDEC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D15F377E-1421-4A8F-9E36-69080AC14CCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -555,7 +555,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -604,6 +604,18 @@
         <bgColor rgb="FF1A6B5C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -645,7 +657,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -786,6 +798,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1640,8 +1658,12 @@
       <c r="C17" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
+      <c r="D17" s="13">
+        <v>1</v>
+      </c>
+      <c r="E17" s="13">
+        <v>1</v>
+      </c>
       <c r="F17" s="11" t="s">
         <v>34</v>
       </c>
@@ -3060,7 +3082,7 @@
       <c r="A6" s="12">
         <v>1</v>
       </c>
-      <c r="B6" s="11" t="str">
+      <c r="B6" s="48" t="str">
         <f>Fixture!C5&amp;" vs "&amp;Fixture!F5</f>
         <v>México vs Sudáfrica</v>
       </c>
@@ -3151,7 +3173,7 @@
       <c r="A7" s="15">
         <v>2</v>
       </c>
-      <c r="B7" s="14" t="str">
+      <c r="B7" s="49" t="str">
         <f>Fixture!C6&amp;" vs "&amp;Fixture!F6</f>
         <v>Corea del Sur vs Chequia</v>
       </c>
@@ -3414,7 +3436,7 @@
       <c r="A12" s="12">
         <v>7</v>
       </c>
-      <c r="B12" s="11" t="str">
+      <c r="B12" s="48" t="str">
         <f>Fixture!C11&amp;" vs "&amp;Fixture!F11</f>
         <v>Canadá vs Bosnia-Herzegovina</v>
       </c>
@@ -3505,7 +3527,7 @@
       <c r="A13" s="15">
         <v>8</v>
       </c>
-      <c r="B13" s="14" t="str">
+      <c r="B13" s="49" t="str">
         <f>Fixture!C12&amp;" vs "&amp;Fixture!F12</f>
         <v>Qatar vs Suiza</v>
       </c>
@@ -3762,7 +3784,7 @@
       </c>
       <c r="C18" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D17),Fixture!D17&amp;"-"&amp;Fixture!E17,"")</f>
-        <v/>
+        <v>1-1</v>
       </c>
       <c r="D18" s="2">
         <v>1</v>
@@ -3800,8 +3822,12 @@
       <c r="O18" s="2">
         <v>1</v>
       </c>
-      <c r="P18" s="2"/>
-      <c r="Q18" s="2"/>
+      <c r="P18" s="2">
+        <v>3</v>
+      </c>
+      <c r="Q18" s="2">
+        <v>1</v>
+      </c>
       <c r="R18" s="2"/>
       <c r="S18" s="2"/>
       <c r="T18" s="2">
@@ -3883,8 +3909,12 @@
       <c r="O19" s="6">
         <v>3</v>
       </c>
-      <c r="P19" s="6"/>
-      <c r="Q19" s="6"/>
+      <c r="P19" s="6">
+        <v>1</v>
+      </c>
+      <c r="Q19" s="6">
+        <v>1</v>
+      </c>
       <c r="R19" s="6"/>
       <c r="S19" s="6"/>
       <c r="T19" s="6">
@@ -4094,7 +4124,7 @@
       <c r="A24" s="12">
         <v>19</v>
       </c>
-      <c r="B24" s="11" t="str">
+      <c r="B24" s="48" t="str">
         <f>Fixture!C23&amp;" vs "&amp;Fixture!F23</f>
         <v>Estados Unidos vs Paraguay</v>
       </c>
@@ -4229,8 +4259,12 @@
       <c r="O25" s="6">
         <v>3</v>
       </c>
-      <c r="P25" s="6"/>
-      <c r="Q25" s="6"/>
+      <c r="P25" s="6">
+        <v>1</v>
+      </c>
+      <c r="Q25" s="6">
+        <v>2</v>
+      </c>
       <c r="R25" s="6"/>
       <c r="S25" s="6"/>
       <c r="T25" s="6">
@@ -4454,8 +4488,12 @@
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
-      <c r="J30" s="2"/>
-      <c r="K30" s="2"/>
+      <c r="J30" s="2">
+        <v>6</v>
+      </c>
+      <c r="K30" s="2">
+        <v>0</v>
+      </c>
       <c r="L30" s="2"/>
       <c r="M30" s="2"/>
       <c r="N30" s="2">
@@ -4470,8 +4508,12 @@
       <c r="S30" s="2"/>
       <c r="T30" s="2"/>
       <c r="U30" s="2"/>
-      <c r="V30" s="2"/>
-      <c r="W30" s="2"/>
+      <c r="V30" s="2">
+        <v>4</v>
+      </c>
+      <c r="W30" s="2">
+        <v>0</v>
+      </c>
       <c r="X30" s="2"/>
       <c r="Y30" s="2"/>
       <c r="Z30" s="2"/>
@@ -4505,8 +4547,12 @@
       <c r="G31" s="6"/>
       <c r="H31" s="6"/>
       <c r="I31" s="6"/>
-      <c r="J31" s="6"/>
-      <c r="K31" s="6"/>
+      <c r="J31" s="6">
+        <v>0</v>
+      </c>
+      <c r="K31" s="6">
+        <v>2</v>
+      </c>
       <c r="L31" s="6"/>
       <c r="M31" s="6"/>
       <c r="N31" s="6">
@@ -4521,8 +4567,12 @@
       <c r="S31" s="6"/>
       <c r="T31" s="6"/>
       <c r="U31" s="6"/>
-      <c r="V31" s="6"/>
-      <c r="W31" s="6"/>
+      <c r="V31" s="6">
+        <v>1</v>
+      </c>
+      <c r="W31" s="6">
+        <v>1</v>
+      </c>
       <c r="X31" s="6"/>
       <c r="Y31" s="6"/>
       <c r="Z31" s="6"/>
@@ -4728,8 +4778,12 @@
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
-      <c r="J36" s="2"/>
-      <c r="K36" s="2"/>
+      <c r="J36" s="2">
+        <v>3</v>
+      </c>
+      <c r="K36" s="2">
+        <v>2</v>
+      </c>
       <c r="L36" s="2"/>
       <c r="M36" s="2"/>
       <c r="N36" s="2">
@@ -4744,8 +4798,12 @@
       <c r="S36" s="2"/>
       <c r="T36" s="2"/>
       <c r="U36" s="2"/>
-      <c r="V36" s="2"/>
-      <c r="W36" s="2"/>
+      <c r="V36" s="2">
+        <v>2</v>
+      </c>
+      <c r="W36" s="2">
+        <v>2</v>
+      </c>
       <c r="X36" s="2"/>
       <c r="Y36" s="2"/>
       <c r="Z36" s="2"/>
@@ -4779,8 +4837,12 @@
       <c r="G37" s="6"/>
       <c r="H37" s="6"/>
       <c r="I37" s="6"/>
-      <c r="J37" s="6"/>
-      <c r="K37" s="6"/>
+      <c r="J37" s="6">
+        <v>1</v>
+      </c>
+      <c r="K37" s="6">
+        <v>0</v>
+      </c>
       <c r="L37" s="6"/>
       <c r="M37" s="6"/>
       <c r="N37" s="6">
@@ -4795,8 +4857,12 @@
       <c r="S37" s="6"/>
       <c r="T37" s="6"/>
       <c r="U37" s="6"/>
-      <c r="V37" s="6"/>
-      <c r="W37" s="6"/>
+      <c r="V37" s="6">
+        <v>2</v>
+      </c>
+      <c r="W37" s="6">
+        <v>0</v>
+      </c>
       <c r="X37" s="6"/>
       <c r="Y37" s="6"/>
       <c r="Z37" s="6"/>

</xml_diff>

<commit_message>
Actualizar - 06-14-dom 11:16
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D15F377E-1421-4A8F-9E36-69080AC14CCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9AF5642-AA5C-40A6-B02C-BD4E1E1E6CC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -1684,8 +1684,12 @@
       <c r="C18" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
+      <c r="D18" s="13">
+        <v>0</v>
+      </c>
+      <c r="E18" s="13">
+        <v>1</v>
+      </c>
       <c r="F18" s="14" t="s">
         <v>36</v>
       </c>
@@ -1802,8 +1806,12 @@
       <c r="C24" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
+      <c r="D24" s="13">
+        <v>2</v>
+      </c>
+      <c r="E24" s="13">
+        <v>0</v>
+      </c>
       <c r="F24" s="14" t="s">
         <v>42</v>
       </c>
@@ -3778,7 +3786,7 @@
       <c r="A18" s="12">
         <v>13</v>
       </c>
-      <c r="B18" s="11" t="str">
+      <c r="B18" s="48" t="str">
         <f>Fixture!C17&amp;" vs "&amp;Fixture!F17</f>
         <v>Brasil vs Marruecos</v>
       </c>
@@ -3865,13 +3873,13 @@
       <c r="A19" s="15">
         <v>14</v>
       </c>
-      <c r="B19" s="14" t="str">
+      <c r="B19" s="49" t="str">
         <f>Fixture!C18&amp;" vs "&amp;Fixture!F18</f>
         <v>Haití vs Escocia</v>
       </c>
       <c r="C19" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D18),Fixture!D18&amp;"-"&amp;Fixture!E18,"")</f>
-        <v/>
+        <v>0-1</v>
       </c>
       <c r="D19" s="6">
         <v>0</v>
@@ -4215,13 +4223,13 @@
       <c r="A25" s="15">
         <v>20</v>
       </c>
-      <c r="B25" s="14" t="str">
+      <c r="B25" s="49" t="str">
         <f>Fixture!C24&amp;" vs "&amp;Fixture!F24</f>
         <v>Australia vs Turquía</v>
       </c>
       <c r="C25" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D24),Fixture!D24&amp;"-"&amp;Fixture!E24,"")</f>
-        <v/>
+        <v>2-0</v>
       </c>
       <c r="D25" s="6">
         <v>1</v>

</xml_diff>

<commit_message>
Actualizar - 06-14-dom 11:23
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9AF5642-AA5C-40A6-B02C-BD4E1E1E6CC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{926F717B-385F-4714-BEA0-7C9E776B88C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4492,26 +4492,42 @@
       <c r="E30" s="2">
         <v>0</v>
       </c>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
+      <c r="F30" s="2">
+        <v>3</v>
+      </c>
+      <c r="G30" s="2">
+        <v>0</v>
+      </c>
+      <c r="H30" s="2">
+        <v>7</v>
+      </c>
+      <c r="I30" s="2">
+        <v>0</v>
+      </c>
       <c r="J30" s="2">
         <v>6</v>
       </c>
       <c r="K30" s="2">
         <v>0</v>
       </c>
-      <c r="L30" s="2"/>
-      <c r="M30" s="2"/>
+      <c r="L30" s="2">
+        <v>4</v>
+      </c>
+      <c r="M30" s="2">
+        <v>0</v>
+      </c>
       <c r="N30" s="2">
         <v>6</v>
       </c>
       <c r="O30" s="2">
         <v>0</v>
       </c>
-      <c r="P30" s="2"/>
-      <c r="Q30" s="2"/>
+      <c r="P30" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q30" s="2">
+        <v>0</v>
+      </c>
       <c r="R30" s="2"/>
       <c r="S30" s="2"/>
       <c r="T30" s="2"/>
@@ -4522,8 +4538,12 @@
       <c r="W30" s="2">
         <v>0</v>
       </c>
-      <c r="X30" s="2"/>
-      <c r="Y30" s="2"/>
+      <c r="X30" s="2">
+        <v>4</v>
+      </c>
+      <c r="Y30" s="2">
+        <v>0</v>
+      </c>
       <c r="Z30" s="2"/>
       <c r="AA30" s="2"/>
       <c r="AB30" s="2"/>
@@ -4551,10 +4571,18 @@
       <c r="E31" s="6">
         <v>1</v>
       </c>
-      <c r="F31" s="6"/>
-      <c r="G31" s="6"/>
-      <c r="H31" s="6"/>
-      <c r="I31" s="6"/>
+      <c r="F31" s="6">
+        <v>1</v>
+      </c>
+      <c r="G31" s="6">
+        <v>3</v>
+      </c>
+      <c r="H31" s="6">
+        <v>2</v>
+      </c>
+      <c r="I31" s="6">
+        <v>2</v>
+      </c>
       <c r="J31" s="6">
         <v>0</v>
       </c>
@@ -4569,8 +4597,12 @@
       <c r="O31" s="6">
         <v>1</v>
       </c>
-      <c r="P31" s="6"/>
-      <c r="Q31" s="6"/>
+      <c r="P31" s="6">
+        <v>1</v>
+      </c>
+      <c r="Q31" s="6">
+        <v>1</v>
+      </c>
       <c r="R31" s="6"/>
       <c r="S31" s="6"/>
       <c r="T31" s="6"/>
@@ -4581,8 +4613,12 @@
       <c r="W31" s="6">
         <v>1</v>
       </c>
-      <c r="X31" s="6"/>
-      <c r="Y31" s="6"/>
+      <c r="X31" s="6">
+        <v>2</v>
+      </c>
+      <c r="Y31" s="6">
+        <v>1</v>
+      </c>
       <c r="Z31" s="6"/>
       <c r="AA31" s="6"/>
       <c r="AB31" s="6"/>
@@ -4782,26 +4818,42 @@
       <c r="E36" s="2">
         <v>2</v>
       </c>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-      <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
+      <c r="F36" s="2">
+        <v>2</v>
+      </c>
+      <c r="G36" s="2">
+        <v>2</v>
+      </c>
+      <c r="H36" s="2">
+        <v>1</v>
+      </c>
+      <c r="I36" s="2">
+        <v>1</v>
+      </c>
       <c r="J36" s="2">
         <v>3</v>
       </c>
       <c r="K36" s="2">
         <v>2</v>
       </c>
-      <c r="L36" s="2"/>
-      <c r="M36" s="2"/>
+      <c r="L36" s="2">
+        <v>1</v>
+      </c>
+      <c r="M36" s="2">
+        <v>1</v>
+      </c>
       <c r="N36" s="2">
         <v>2</v>
       </c>
       <c r="O36" s="2">
         <v>1</v>
       </c>
-      <c r="P36" s="2"/>
-      <c r="Q36" s="2"/>
+      <c r="P36" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q36" s="2">
+        <v>2</v>
+      </c>
       <c r="R36" s="2"/>
       <c r="S36" s="2"/>
       <c r="T36" s="2"/>
@@ -4812,8 +4864,12 @@
       <c r="W36" s="2">
         <v>2</v>
       </c>
-      <c r="X36" s="2"/>
-      <c r="Y36" s="2"/>
+      <c r="X36" s="2">
+        <v>1</v>
+      </c>
+      <c r="Y36" s="2">
+        <v>1</v>
+      </c>
       <c r="Z36" s="2"/>
       <c r="AA36" s="2"/>
       <c r="AB36" s="2"/>
@@ -4841,10 +4897,18 @@
       <c r="E37" s="6">
         <v>0</v>
       </c>
-      <c r="F37" s="6"/>
-      <c r="G37" s="6"/>
-      <c r="H37" s="6"/>
-      <c r="I37" s="6"/>
+      <c r="F37" s="6">
+        <v>2</v>
+      </c>
+      <c r="G37" s="6">
+        <v>1</v>
+      </c>
+      <c r="H37" s="6">
+        <v>1</v>
+      </c>
+      <c r="I37" s="6">
+        <v>1</v>
+      </c>
       <c r="J37" s="6">
         <v>1</v>
       </c>
@@ -4859,8 +4923,12 @@
       <c r="O37" s="6">
         <v>0</v>
       </c>
-      <c r="P37" s="6"/>
-      <c r="Q37" s="6"/>
+      <c r="P37" s="6">
+        <v>2</v>
+      </c>
+      <c r="Q37" s="6">
+        <v>1</v>
+      </c>
       <c r="R37" s="6"/>
       <c r="S37" s="6"/>
       <c r="T37" s="6"/>
@@ -4871,8 +4939,12 @@
       <c r="W37" s="6">
         <v>0</v>
       </c>
-      <c r="X37" s="6"/>
-      <c r="Y37" s="6"/>
+      <c r="X37" s="6">
+        <v>2</v>
+      </c>
+      <c r="Y37" s="6">
+        <v>0</v>
+      </c>
       <c r="Z37" s="6"/>
       <c r="AA37" s="6"/>
       <c r="AB37" s="6"/>

</xml_diff>

<commit_message>
Actualizar - 06-14-dom 12:21
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{926F717B-385F-4714-BEA0-7C9E776B88C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C979AFB-09B6-4729-9779-8AB7D4B0E3F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4528,10 +4528,18 @@
       <c r="Q30" s="2">
         <v>0</v>
       </c>
-      <c r="R30" s="2"/>
-      <c r="S30" s="2"/>
-      <c r="T30" s="2"/>
-      <c r="U30" s="2"/>
+      <c r="R30" s="2">
+        <v>3</v>
+      </c>
+      <c r="S30" s="2">
+        <v>0</v>
+      </c>
+      <c r="T30" s="2">
+        <v>2</v>
+      </c>
+      <c r="U30" s="2">
+        <v>0</v>
+      </c>
       <c r="V30" s="2">
         <v>4</v>
       </c>
@@ -4544,8 +4552,12 @@
       <c r="Y30" s="2">
         <v>0</v>
       </c>
-      <c r="Z30" s="2"/>
-      <c r="AA30" s="2"/>
+      <c r="Z30" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA30" s="2">
+        <v>1</v>
+      </c>
       <c r="AB30" s="2"/>
       <c r="AC30" s="2"/>
       <c r="AD30" s="2"/>
@@ -4589,8 +4601,12 @@
       <c r="K31" s="6">
         <v>2</v>
       </c>
-      <c r="L31" s="6"/>
-      <c r="M31" s="6"/>
+      <c r="L31" s="6">
+        <v>2</v>
+      </c>
+      <c r="M31" s="6">
+        <v>1</v>
+      </c>
       <c r="N31" s="6">
         <v>0</v>
       </c>
@@ -4603,10 +4619,18 @@
       <c r="Q31" s="6">
         <v>1</v>
       </c>
-      <c r="R31" s="6"/>
-      <c r="S31" s="6"/>
-      <c r="T31" s="6"/>
-      <c r="U31" s="6"/>
+      <c r="R31" s="6">
+        <v>1</v>
+      </c>
+      <c r="S31" s="6">
+        <v>1</v>
+      </c>
+      <c r="T31" s="6">
+        <v>2</v>
+      </c>
+      <c r="U31" s="6">
+        <v>2</v>
+      </c>
       <c r="V31" s="6">
         <v>1</v>
       </c>
@@ -4619,8 +4643,12 @@
       <c r="Y31" s="6">
         <v>1</v>
       </c>
-      <c r="Z31" s="6"/>
-      <c r="AA31" s="6"/>
+      <c r="Z31" s="6">
+        <v>3</v>
+      </c>
+      <c r="AA31" s="6">
+        <v>0</v>
+      </c>
       <c r="AB31" s="6"/>
       <c r="AC31" s="6"/>
       <c r="AD31" s="6"/>
@@ -4854,10 +4882,18 @@
       <c r="Q36" s="2">
         <v>2</v>
       </c>
-      <c r="R36" s="2"/>
-      <c r="S36" s="2"/>
-      <c r="T36" s="2"/>
-      <c r="U36" s="2"/>
+      <c r="R36" s="2">
+        <v>2</v>
+      </c>
+      <c r="S36" s="2">
+        <v>1</v>
+      </c>
+      <c r="T36" s="2">
+        <v>0</v>
+      </c>
+      <c r="U36" s="2">
+        <v>1</v>
+      </c>
       <c r="V36" s="2">
         <v>2</v>
       </c>
@@ -4870,8 +4906,12 @@
       <c r="Y36" s="2">
         <v>1</v>
       </c>
-      <c r="Z36" s="2"/>
-      <c r="AA36" s="2"/>
+      <c r="Z36" s="2">
+        <v>0</v>
+      </c>
+      <c r="AA36" s="2">
+        <v>2</v>
+      </c>
       <c r="AB36" s="2"/>
       <c r="AC36" s="2"/>
       <c r="AD36" s="2"/>
@@ -4915,8 +4955,12 @@
       <c r="K37" s="6">
         <v>0</v>
       </c>
-      <c r="L37" s="6"/>
-      <c r="M37" s="6"/>
+      <c r="L37" s="6">
+        <v>1</v>
+      </c>
+      <c r="M37" s="6">
+        <v>0</v>
+      </c>
       <c r="N37" s="6">
         <v>2</v>
       </c>
@@ -4929,10 +4973,18 @@
       <c r="Q37" s="6">
         <v>1</v>
       </c>
-      <c r="R37" s="6"/>
-      <c r="S37" s="6"/>
-      <c r="T37" s="6"/>
-      <c r="U37" s="6"/>
+      <c r="R37" s="6">
+        <v>1</v>
+      </c>
+      <c r="S37" s="6">
+        <v>0</v>
+      </c>
+      <c r="T37" s="6">
+        <v>1</v>
+      </c>
+      <c r="U37" s="6">
+        <v>0</v>
+      </c>
       <c r="V37" s="6">
         <v>2</v>
       </c>
@@ -4945,8 +4997,12 @@
       <c r="Y37" s="6">
         <v>0</v>
       </c>
-      <c r="Z37" s="6"/>
-      <c r="AA37" s="6"/>
+      <c r="Z37" s="6">
+        <v>2</v>
+      </c>
+      <c r="AA37" s="6">
+        <v>0</v>
+      </c>
       <c r="AB37" s="6"/>
       <c r="AC37" s="6"/>
       <c r="AD37" s="6"/>

</xml_diff>

<commit_message>
Actualizar - 06-14-dom 12:23
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C979AFB-09B6-4729-9779-8AB7D4B0E3F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADD70408-75E2-479F-BA3D-CD7CCC16D8C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4535,7 +4535,7 @@
         <v>0</v>
       </c>
       <c r="T30" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U30" s="2">
         <v>0</v>
@@ -4626,10 +4626,10 @@
         <v>1</v>
       </c>
       <c r="T31" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U31" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V31" s="6">
         <v>1</v>
@@ -4889,7 +4889,7 @@
         <v>1</v>
       </c>
       <c r="T36" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U36" s="2">
         <v>1</v>

</xml_diff>

<commit_message>
Actualizar - 06-14-dom 22:27
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADD70408-75E2-479F-BA3D-CD7CCC16D8C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58C73E74-AD72-46EB-ABBB-62DB7CB0633C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -788,22 +788,22 @@
     <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="22" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1079,20 +1079,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="46" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
+      <c r="A1" s="49" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
     </row>
     <row r="2" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
+      <c r="A2" s="47" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
     </row>
     <row r="3" spans="1:4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1359,26 +1359,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
     </row>
     <row r="3" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1905,8 +1905,12 @@
       <c r="C29" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
+      <c r="D29" s="13">
+        <v>7</v>
+      </c>
+      <c r="E29" s="13">
+        <v>1</v>
+      </c>
       <c r="F29" s="11" t="s">
         <v>46</v>
       </c>
@@ -1924,8 +1928,12 @@
       <c r="C30" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
+      <c r="D30" s="13">
+        <v>1</v>
+      </c>
+      <c r="E30" s="13">
+        <v>0</v>
+      </c>
       <c r="F30" s="14" t="s">
         <v>49</v>
       </c>
@@ -2019,8 +2027,12 @@
       <c r="C35" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
+      <c r="D35" s="13">
+        <v>2</v>
+      </c>
+      <c r="E35" s="13">
+        <v>2</v>
+      </c>
       <c r="F35" s="11" t="s">
         <v>53</v>
       </c>
@@ -2829,78 +2841,78 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="46" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="44"/>
-      <c r="R1" s="44"/>
-      <c r="S1" s="44"/>
-      <c r="T1" s="44"/>
-      <c r="U1" s="44"/>
-      <c r="V1" s="44"/>
-      <c r="W1" s="44"/>
-      <c r="X1" s="44"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="44"/>
-      <c r="AA1" s="44"/>
-      <c r="AB1" s="44"/>
-      <c r="AC1" s="44"/>
-      <c r="AD1" s="44"/>
-      <c r="AE1" s="44"/>
-      <c r="AF1" s="44"/>
-      <c r="AG1" s="44"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
+      <c r="M1" s="46"/>
+      <c r="N1" s="46"/>
+      <c r="O1" s="46"/>
+      <c r="P1" s="46"/>
+      <c r="Q1" s="46"/>
+      <c r="R1" s="46"/>
+      <c r="S1" s="46"/>
+      <c r="T1" s="46"/>
+      <c r="U1" s="46"/>
+      <c r="V1" s="46"/>
+      <c r="W1" s="46"/>
+      <c r="X1" s="46"/>
+      <c r="Y1" s="46"/>
+      <c r="Z1" s="46"/>
+      <c r="AA1" s="46"/>
+      <c r="AB1" s="46"/>
+      <c r="AC1" s="46"/>
+      <c r="AD1" s="46"/>
+      <c r="AE1" s="46"/>
+      <c r="AF1" s="46"/>
+      <c r="AG1" s="46"/>
     </row>
     <row r="2" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="47" t="s">
         <v>95</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
-      <c r="P2" s="45"/>
-      <c r="Q2" s="45"/>
-      <c r="R2" s="45"/>
-      <c r="S2" s="45"/>
-      <c r="T2" s="45"/>
-      <c r="U2" s="45"/>
-      <c r="V2" s="45"/>
-      <c r="W2" s="45"/>
-      <c r="X2" s="45"/>
-      <c r="Y2" s="45"/>
-      <c r="Z2" s="45"/>
-      <c r="AA2" s="45"/>
-      <c r="AB2" s="45"/>
-      <c r="AC2" s="45"/>
-      <c r="AD2" s="45"/>
-      <c r="AE2" s="45"/>
-      <c r="AF2" s="45"/>
-      <c r="AG2" s="45"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47"/>
+      <c r="M2" s="47"/>
+      <c r="N2" s="47"/>
+      <c r="O2" s="47"/>
+      <c r="P2" s="47"/>
+      <c r="Q2" s="47"/>
+      <c r="R2" s="47"/>
+      <c r="S2" s="47"/>
+      <c r="T2" s="47"/>
+      <c r="U2" s="47"/>
+      <c r="V2" s="47"/>
+      <c r="W2" s="47"/>
+      <c r="X2" s="47"/>
+      <c r="Y2" s="47"/>
+      <c r="Z2" s="47"/>
+      <c r="AA2" s="47"/>
+      <c r="AB2" s="47"/>
+      <c r="AC2" s="47"/>
+      <c r="AD2" s="47"/>
+      <c r="AE2" s="47"/>
+      <c r="AF2" s="47"/>
+      <c r="AG2" s="47"/>
     </row>
     <row r="3" spans="1:33" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2913,81 +2925,81 @@
       <c r="C4" s="39" t="s">
         <v>97</v>
       </c>
-      <c r="D4" s="47" t="str">
+      <c r="D4" s="48" t="str">
         <f>Participantes!B5</f>
         <v>Andres Jesús</v>
       </c>
-      <c r="E4" s="47"/>
-      <c r="F4" s="47" t="str">
+      <c r="E4" s="48"/>
+      <c r="F4" s="48" t="str">
         <f>Participantes!B6</f>
         <v>Leonardo Fabio</v>
       </c>
-      <c r="G4" s="47"/>
-      <c r="H4" s="47" t="str">
+      <c r="G4" s="48"/>
+      <c r="H4" s="48" t="str">
         <f>Participantes!B7</f>
         <v>Martha Cenidia</v>
       </c>
-      <c r="I4" s="47"/>
-      <c r="J4" s="47" t="str">
+      <c r="I4" s="48"/>
+      <c r="J4" s="48" t="str">
         <f>Participantes!B8</f>
         <v>Freddy Ramón</v>
       </c>
-      <c r="K4" s="47"/>
-      <c r="L4" s="47" t="str">
+      <c r="K4" s="48"/>
+      <c r="L4" s="48" t="str">
         <f>Participantes!B9</f>
         <v xml:space="preserve">Juan Camilo </v>
       </c>
-      <c r="M4" s="47"/>
-      <c r="N4" s="47" t="str">
+      <c r="M4" s="48"/>
+      <c r="N4" s="48" t="str">
         <f>Participantes!B10</f>
         <v xml:space="preserve">Juan David </v>
       </c>
-      <c r="O4" s="47"/>
-      <c r="P4" s="47" t="str">
+      <c r="O4" s="48"/>
+      <c r="P4" s="48" t="str">
         <f>Participantes!B11</f>
         <v>María Trinidad</v>
       </c>
-      <c r="Q4" s="47"/>
-      <c r="R4" s="47" t="str">
+      <c r="Q4" s="48"/>
+      <c r="R4" s="48" t="str">
         <f>Participantes!B12</f>
         <v xml:space="preserve">María Gabriela </v>
       </c>
-      <c r="S4" s="47"/>
-      <c r="T4" s="47" t="str">
+      <c r="S4" s="48"/>
+      <c r="T4" s="48" t="str">
         <f>Participantes!B13</f>
         <v>Laura Valentina</v>
       </c>
-      <c r="U4" s="47"/>
-      <c r="V4" s="47" t="str">
+      <c r="U4" s="48"/>
+      <c r="V4" s="48" t="str">
         <f>Participantes!B14</f>
         <v>Gloria Isabel</v>
       </c>
-      <c r="W4" s="47"/>
-      <c r="X4" s="47" t="str">
+      <c r="W4" s="48"/>
+      <c r="X4" s="48" t="str">
         <f>Participantes!B15</f>
         <v xml:space="preserve">María del Pilar </v>
       </c>
-      <c r="Y4" s="47"/>
-      <c r="Z4" s="47" t="str">
+      <c r="Y4" s="48"/>
+      <c r="Z4" s="48" t="str">
         <f>Participantes!B16</f>
         <v>Jaime Andres</v>
       </c>
-      <c r="AA4" s="47"/>
-      <c r="AB4" s="47" t="str">
+      <c r="AA4" s="48"/>
+      <c r="AB4" s="48" t="str">
         <f>Participantes!B17</f>
         <v>Participante 13</v>
       </c>
-      <c r="AC4" s="47"/>
-      <c r="AD4" s="47" t="str">
+      <c r="AC4" s="48"/>
+      <c r="AD4" s="48" t="str">
         <f>Participantes!B18</f>
         <v>Participante 14</v>
       </c>
-      <c r="AE4" s="47"/>
-      <c r="AF4" s="47" t="str">
+      <c r="AE4" s="48"/>
+      <c r="AF4" s="48" t="str">
         <f>Participantes!B19</f>
         <v>Participante 15</v>
       </c>
-      <c r="AG4" s="47"/>
+      <c r="AG4" s="48"/>
     </row>
     <row r="5" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="40"/>
@@ -3090,7 +3102,7 @@
       <c r="A6" s="12">
         <v>1</v>
       </c>
-      <c r="B6" s="48" t="str">
+      <c r="B6" s="44" t="str">
         <f>Fixture!C5&amp;" vs "&amp;Fixture!F5</f>
         <v>México vs Sudáfrica</v>
       </c>
@@ -3181,7 +3193,7 @@
       <c r="A7" s="15">
         <v>2</v>
       </c>
-      <c r="B7" s="49" t="str">
+      <c r="B7" s="45" t="str">
         <f>Fixture!C6&amp;" vs "&amp;Fixture!F6</f>
         <v>Corea del Sur vs Chequia</v>
       </c>
@@ -3444,7 +3456,7 @@
       <c r="A12" s="12">
         <v>7</v>
       </c>
-      <c r="B12" s="48" t="str">
+      <c r="B12" s="44" t="str">
         <f>Fixture!C11&amp;" vs "&amp;Fixture!F11</f>
         <v>Canadá vs Bosnia-Herzegovina</v>
       </c>
@@ -3535,7 +3547,7 @@
       <c r="A13" s="15">
         <v>8</v>
       </c>
-      <c r="B13" s="49" t="str">
+      <c r="B13" s="45" t="str">
         <f>Fixture!C12&amp;" vs "&amp;Fixture!F12</f>
         <v>Qatar vs Suiza</v>
       </c>
@@ -3786,7 +3798,7 @@
       <c r="A18" s="12">
         <v>13</v>
       </c>
-      <c r="B18" s="48" t="str">
+      <c r="B18" s="44" t="str">
         <f>Fixture!C17&amp;" vs "&amp;Fixture!F17</f>
         <v>Brasil vs Marruecos</v>
       </c>
@@ -3873,7 +3885,7 @@
       <c r="A19" s="15">
         <v>14</v>
       </c>
-      <c r="B19" s="49" t="str">
+      <c r="B19" s="45" t="str">
         <f>Fixture!C18&amp;" vs "&amp;Fixture!F18</f>
         <v>Haití vs Escocia</v>
       </c>
@@ -4132,7 +4144,7 @@
       <c r="A24" s="12">
         <v>19</v>
       </c>
-      <c r="B24" s="48" t="str">
+      <c r="B24" s="44" t="str">
         <f>Fixture!C23&amp;" vs "&amp;Fixture!F23</f>
         <v>Estados Unidos vs Paraguay</v>
       </c>
@@ -4223,7 +4235,7 @@
       <c r="A25" s="15">
         <v>20</v>
       </c>
-      <c r="B25" s="49" t="str">
+      <c r="B25" s="45" t="str">
         <f>Fixture!C24&amp;" vs "&amp;Fixture!F24</f>
         <v>Australia vs Turquía</v>
       </c>
@@ -4484,7 +4496,7 @@
       </c>
       <c r="C30" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D29),Fixture!D29&amp;"-"&amp;Fixture!E29,"")</f>
-        <v/>
+        <v>7-1</v>
       </c>
       <c r="D30" s="2">
         <v>5</v>
@@ -4575,7 +4587,7 @@
       </c>
       <c r="C31" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D30),Fixture!D30&amp;"-"&amp;Fixture!E30,"")</f>
-        <v/>
+        <v>1-0</v>
       </c>
       <c r="D31" s="6">
         <v>1</v>
@@ -4838,7 +4850,7 @@
       </c>
       <c r="C36" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D35),Fixture!D35&amp;"-"&amp;Fixture!E35,"")</f>
-        <v/>
+        <v>2-2</v>
       </c>
       <c r="D36" s="2">
         <v>2</v>
@@ -6732,6 +6744,7 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="AF4:AG4"/>
     <mergeCell ref="A1:AG1"/>
     <mergeCell ref="A2:AG2"/>
     <mergeCell ref="D4:E4"/>
@@ -6748,7 +6761,6 @@
     <mergeCell ref="Z4:AA4"/>
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AD4:AE4"/>
-    <mergeCell ref="AF4:AG4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Actualizar - 06-14-dom 22:37
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58C73E74-AD72-46EB-ABBB-62DB7CB0633C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E147F1AB-9592-4FCD-9954-175C9D91C218}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -4490,7 +4490,7 @@
       <c r="A30" s="12">
         <v>25</v>
       </c>
-      <c r="B30" s="11" t="str">
+      <c r="B30" s="44" t="str">
         <f>Fixture!C29&amp;" vs "&amp;Fixture!F29</f>
         <v>Alemania vs Curazao</v>
       </c>
@@ -4581,7 +4581,7 @@
       <c r="A31" s="15">
         <v>26</v>
       </c>
-      <c r="B31" s="14" t="str">
+      <c r="B31" s="45" t="str">
         <f>Fixture!C30&amp;" vs "&amp;Fixture!F30</f>
         <v>Costa de Marfil vs Ecuador</v>
       </c>
@@ -4844,7 +4844,7 @@
       <c r="A36" s="12">
         <v>31</v>
       </c>
-      <c r="B36" s="11" t="str">
+      <c r="B36" s="44" t="str">
         <f>Fixture!C35&amp;" vs "&amp;Fixture!F35</f>
         <v>Países Bajos vs Japón</v>
       </c>
@@ -5206,26 +5206,46 @@
         <f>IF(ISNUMBER(Fixture!D41),Fixture!D41&amp;"-"&amp;Fixture!E41,"")</f>
         <v/>
       </c>
-      <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
+      <c r="D42" s="2">
+        <v>2</v>
+      </c>
+      <c r="E42" s="2">
+        <v>1</v>
+      </c>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
-      <c r="H42" s="2"/>
-      <c r="I42" s="2"/>
-      <c r="J42" s="2"/>
-      <c r="K42" s="2"/>
+      <c r="H42" s="2">
+        <v>2</v>
+      </c>
+      <c r="I42" s="2">
+        <v>2</v>
+      </c>
+      <c r="J42" s="2">
+        <v>1</v>
+      </c>
+      <c r="K42" s="2">
+        <v>1</v>
+      </c>
       <c r="L42" s="2"/>
       <c r="M42" s="2"/>
-      <c r="N42" s="2"/>
-      <c r="O42" s="2"/>
+      <c r="N42" s="2">
+        <v>1</v>
+      </c>
+      <c r="O42" s="2">
+        <v>1</v>
+      </c>
       <c r="P42" s="2"/>
       <c r="Q42" s="2"/>
       <c r="R42" s="2"/>
       <c r="S42" s="2"/>
       <c r="T42" s="2"/>
       <c r="U42" s="2"/>
-      <c r="V42" s="2"/>
-      <c r="W42" s="2"/>
+      <c r="V42" s="2">
+        <v>2</v>
+      </c>
+      <c r="W42" s="2">
+        <v>1</v>
+      </c>
       <c r="X42" s="2"/>
       <c r="Y42" s="2"/>
       <c r="Z42" s="2"/>
@@ -5249,26 +5269,46 @@
         <f>IF(ISNUMBER(Fixture!D42),Fixture!D42&amp;"-"&amp;Fixture!E42,"")</f>
         <v/>
       </c>
-      <c r="D43" s="6"/>
-      <c r="E43" s="6"/>
+      <c r="D43" s="6">
+        <v>1</v>
+      </c>
+      <c r="E43" s="6">
+        <v>1</v>
+      </c>
       <c r="F43" s="6"/>
       <c r="G43" s="6"/>
-      <c r="H43" s="6"/>
-      <c r="I43" s="6"/>
-      <c r="J43" s="6"/>
-      <c r="K43" s="6"/>
+      <c r="H43" s="6">
+        <v>2</v>
+      </c>
+      <c r="I43" s="6">
+        <v>0</v>
+      </c>
+      <c r="J43" s="6">
+        <v>2</v>
+      </c>
+      <c r="K43" s="6">
+        <v>1</v>
+      </c>
       <c r="L43" s="6"/>
       <c r="M43" s="6"/>
-      <c r="N43" s="6"/>
-      <c r="O43" s="6"/>
+      <c r="N43" s="6">
+        <v>3</v>
+      </c>
+      <c r="O43" s="6">
+        <v>1</v>
+      </c>
       <c r="P43" s="6"/>
       <c r="Q43" s="6"/>
       <c r="R43" s="6"/>
       <c r="S43" s="6"/>
       <c r="T43" s="6"/>
       <c r="U43" s="6"/>
-      <c r="V43" s="6"/>
-      <c r="W43" s="6"/>
+      <c r="V43" s="6">
+        <v>2</v>
+      </c>
+      <c r="W43" s="6">
+        <v>0</v>
+      </c>
       <c r="X43" s="6"/>
       <c r="Y43" s="6"/>
       <c r="Z43" s="6"/>
@@ -5464,26 +5504,46 @@
         <f>IF(ISNUMBER(Fixture!D47),Fixture!D47&amp;"-"&amp;Fixture!E47,"")</f>
         <v/>
       </c>
-      <c r="D48" s="2"/>
-      <c r="E48" s="2"/>
+      <c r="D48" s="2">
+        <v>4</v>
+      </c>
+      <c r="E48" s="2">
+        <v>1</v>
+      </c>
       <c r="F48" s="2"/>
       <c r="G48" s="2"/>
-      <c r="H48" s="2"/>
-      <c r="I48" s="2"/>
-      <c r="J48" s="2"/>
-      <c r="K48" s="2"/>
+      <c r="H48" s="2">
+        <v>3</v>
+      </c>
+      <c r="I48" s="2">
+        <v>1</v>
+      </c>
+      <c r="J48" s="2">
+        <v>3</v>
+      </c>
+      <c r="K48" s="2">
+        <v>1</v>
+      </c>
       <c r="L48" s="2"/>
       <c r="M48" s="2"/>
-      <c r="N48" s="2"/>
-      <c r="O48" s="2"/>
+      <c r="N48" s="2">
+        <v>4</v>
+      </c>
+      <c r="O48" s="2">
+        <v>1</v>
+      </c>
       <c r="P48" s="2"/>
       <c r="Q48" s="2"/>
       <c r="R48" s="2"/>
       <c r="S48" s="2"/>
       <c r="T48" s="2"/>
       <c r="U48" s="2"/>
-      <c r="V48" s="2"/>
-      <c r="W48" s="2"/>
+      <c r="V48" s="2">
+        <v>3</v>
+      </c>
+      <c r="W48" s="2">
+        <v>0</v>
+      </c>
       <c r="X48" s="2"/>
       <c r="Y48" s="2"/>
       <c r="Z48" s="2"/>
@@ -5507,26 +5567,46 @@
         <f>IF(ISNUMBER(Fixture!D48),Fixture!D48&amp;"-"&amp;Fixture!E48,"")</f>
         <v/>
       </c>
-      <c r="D49" s="6"/>
-      <c r="E49" s="6"/>
+      <c r="D49" s="6">
+        <v>1</v>
+      </c>
+      <c r="E49" s="6">
+        <v>3</v>
+      </c>
       <c r="F49" s="6"/>
       <c r="G49" s="6"/>
-      <c r="H49" s="6"/>
-      <c r="I49" s="6"/>
-      <c r="J49" s="6"/>
-      <c r="K49" s="6"/>
+      <c r="H49" s="6">
+        <v>2</v>
+      </c>
+      <c r="I49" s="6">
+        <v>3</v>
+      </c>
+      <c r="J49" s="6">
+        <v>0</v>
+      </c>
+      <c r="K49" s="6">
+        <v>2</v>
+      </c>
       <c r="L49" s="6"/>
       <c r="M49" s="6"/>
-      <c r="N49" s="6"/>
-      <c r="O49" s="6"/>
+      <c r="N49" s="6">
+        <v>1</v>
+      </c>
+      <c r="O49" s="6">
+        <v>2</v>
+      </c>
       <c r="P49" s="6"/>
       <c r="Q49" s="6"/>
       <c r="R49" s="6"/>
       <c r="S49" s="6"/>
       <c r="T49" s="6"/>
       <c r="U49" s="6"/>
-      <c r="V49" s="6"/>
-      <c r="W49" s="6"/>
+      <c r="V49" s="6">
+        <v>0</v>
+      </c>
+      <c r="W49" s="6">
+        <v>2</v>
+      </c>
       <c r="X49" s="6"/>
       <c r="Y49" s="6"/>
       <c r="Z49" s="6"/>

</xml_diff>

<commit_message>
Actualizar - 06-15-lun 10:01
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E147F1AB-9592-4FCD-9954-175C9D91C218}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F0AB40-4ED8-4B2D-98E9-BDBBF5F92FA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2050,8 +2050,12 @@
       <c r="C36" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
+      <c r="D36" s="13">
+        <v>5</v>
+      </c>
+      <c r="E36" s="13">
+        <v>1</v>
+      </c>
       <c r="F36" s="14" t="s">
         <v>55</v>
       </c>
@@ -4941,7 +4945,7 @@
       </c>
       <c r="C37" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D36),Fixture!D36&amp;"-"&amp;Fixture!E36,"")</f>
-        <v/>
+        <v>5-1</v>
       </c>
       <c r="D37" s="6">
         <v>2</v>
@@ -5212,8 +5216,12 @@
       <c r="E42" s="2">
         <v>1</v>
       </c>
-      <c r="F42" s="2"/>
-      <c r="G42" s="2"/>
+      <c r="F42" s="2">
+        <v>2</v>
+      </c>
+      <c r="G42" s="2">
+        <v>1</v>
+      </c>
       <c r="H42" s="2">
         <v>2</v>
       </c>
@@ -5234,22 +5242,38 @@
       <c r="O42" s="2">
         <v>1</v>
       </c>
-      <c r="P42" s="2"/>
-      <c r="Q42" s="2"/>
+      <c r="P42" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q42" s="2">
+        <v>2</v>
+      </c>
       <c r="R42" s="2"/>
       <c r="S42" s="2"/>
-      <c r="T42" s="2"/>
-      <c r="U42" s="2"/>
+      <c r="T42" s="2">
+        <v>2</v>
+      </c>
+      <c r="U42" s="2">
+        <v>1</v>
+      </c>
       <c r="V42" s="2">
         <v>2</v>
       </c>
       <c r="W42" s="2">
         <v>1</v>
       </c>
-      <c r="X42" s="2"/>
-      <c r="Y42" s="2"/>
-      <c r="Z42" s="2"/>
-      <c r="AA42" s="2"/>
+      <c r="X42" s="2">
+        <v>2</v>
+      </c>
+      <c r="Y42" s="2">
+        <v>1</v>
+      </c>
+      <c r="Z42" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA42" s="2">
+        <v>0</v>
+      </c>
       <c r="AB42" s="2"/>
       <c r="AC42" s="2"/>
       <c r="AD42" s="2"/>
@@ -5275,8 +5299,12 @@
       <c r="E43" s="6">
         <v>1</v>
       </c>
-      <c r="F43" s="6"/>
-      <c r="G43" s="6"/>
+      <c r="F43" s="6">
+        <v>3</v>
+      </c>
+      <c r="G43" s="6">
+        <v>0</v>
+      </c>
       <c r="H43" s="6">
         <v>2</v>
       </c>
@@ -5297,22 +5325,38 @@
       <c r="O43" s="6">
         <v>1</v>
       </c>
-      <c r="P43" s="6"/>
-      <c r="Q43" s="6"/>
+      <c r="P43" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q43" s="6">
+        <v>2</v>
+      </c>
       <c r="R43" s="6"/>
       <c r="S43" s="6"/>
-      <c r="T43" s="6"/>
-      <c r="U43" s="6"/>
+      <c r="T43" s="6">
+        <v>1</v>
+      </c>
+      <c r="U43" s="6">
+        <v>0</v>
+      </c>
       <c r="V43" s="6">
         <v>2</v>
       </c>
       <c r="W43" s="6">
         <v>0</v>
       </c>
-      <c r="X43" s="6"/>
-      <c r="Y43" s="6"/>
-      <c r="Z43" s="6"/>
-      <c r="AA43" s="6"/>
+      <c r="X43" s="6">
+        <v>2</v>
+      </c>
+      <c r="Y43" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z43" s="6">
+        <v>1</v>
+      </c>
+      <c r="AA43" s="6">
+        <v>0</v>
+      </c>
       <c r="AB43" s="6"/>
       <c r="AC43" s="6"/>
       <c r="AD43" s="6"/>
@@ -5510,8 +5554,12 @@
       <c r="E48" s="2">
         <v>1</v>
       </c>
-      <c r="F48" s="2"/>
-      <c r="G48" s="2"/>
+      <c r="F48" s="2">
+        <v>4</v>
+      </c>
+      <c r="G48" s="2">
+        <v>1</v>
+      </c>
       <c r="H48" s="2">
         <v>3</v>
       </c>
@@ -5532,22 +5580,38 @@
       <c r="O48" s="2">
         <v>1</v>
       </c>
-      <c r="P48" s="2"/>
-      <c r="Q48" s="2"/>
+      <c r="P48" s="2">
+        <v>4</v>
+      </c>
+      <c r="Q48" s="2">
+        <v>0</v>
+      </c>
       <c r="R48" s="2"/>
       <c r="S48" s="2"/>
-      <c r="T48" s="2"/>
-      <c r="U48" s="2"/>
+      <c r="T48" s="2">
+        <v>3</v>
+      </c>
+      <c r="U48" s="2">
+        <v>0</v>
+      </c>
       <c r="V48" s="2">
         <v>3</v>
       </c>
       <c r="W48" s="2">
         <v>0</v>
       </c>
-      <c r="X48" s="2"/>
-      <c r="Y48" s="2"/>
-      <c r="Z48" s="2"/>
-      <c r="AA48" s="2"/>
+      <c r="X48" s="2">
+        <v>3</v>
+      </c>
+      <c r="Y48" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z48" s="2">
+        <v>4</v>
+      </c>
+      <c r="AA48" s="2">
+        <v>0</v>
+      </c>
       <c r="AB48" s="2"/>
       <c r="AC48" s="2"/>
       <c r="AD48" s="2"/>
@@ -5573,8 +5637,12 @@
       <c r="E49" s="6">
         <v>3</v>
       </c>
-      <c r="F49" s="6"/>
-      <c r="G49" s="6"/>
+      <c r="F49" s="6">
+        <v>1</v>
+      </c>
+      <c r="G49" s="6">
+        <v>3</v>
+      </c>
       <c r="H49" s="6">
         <v>2</v>
       </c>
@@ -5595,22 +5663,38 @@
       <c r="O49" s="6">
         <v>2</v>
       </c>
-      <c r="P49" s="6"/>
-      <c r="Q49" s="6"/>
+      <c r="P49" s="6">
+        <v>1</v>
+      </c>
+      <c r="Q49" s="6">
+        <v>2</v>
+      </c>
       <c r="R49" s="6"/>
       <c r="S49" s="6"/>
-      <c r="T49" s="6"/>
-      <c r="U49" s="6"/>
+      <c r="T49" s="6">
+        <v>1</v>
+      </c>
+      <c r="U49" s="6">
+        <v>2</v>
+      </c>
       <c r="V49" s="6">
         <v>0</v>
       </c>
       <c r="W49" s="6">
         <v>2</v>
       </c>
-      <c r="X49" s="6"/>
-      <c r="Y49" s="6"/>
-      <c r="Z49" s="6"/>
-      <c r="AA49" s="6"/>
+      <c r="X49" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y49" s="6">
+        <v>2</v>
+      </c>
+      <c r="Z49" s="6">
+        <v>1</v>
+      </c>
+      <c r="AA49" s="6">
+        <v>2</v>
+      </c>
       <c r="AB49" s="6"/>
       <c r="AC49" s="6"/>
       <c r="AD49" s="6"/>

</xml_diff>

<commit_message>
Actualizar - 06-15-lun 10:04
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F0AB40-4ED8-4B2D-98E9-BDBBF5F92FA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04C47AF6-0DE6-4956-B55A-BC042AE80E58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5248,8 +5248,12 @@
       <c r="Q42" s="2">
         <v>2</v>
       </c>
-      <c r="R42" s="2"/>
-      <c r="S42" s="2"/>
+      <c r="R42" s="2">
+        <v>2</v>
+      </c>
+      <c r="S42" s="2">
+        <v>2</v>
+      </c>
       <c r="T42" s="2">
         <v>2</v>
       </c>
@@ -5331,8 +5335,12 @@
       <c r="Q43" s="6">
         <v>2</v>
       </c>
-      <c r="R43" s="6"/>
-      <c r="S43" s="6"/>
+      <c r="R43" s="6">
+        <v>0</v>
+      </c>
+      <c r="S43" s="6">
+        <v>2</v>
+      </c>
       <c r="T43" s="6">
         <v>1</v>
       </c>
@@ -5586,8 +5594,12 @@
       <c r="Q48" s="2">
         <v>0</v>
       </c>
-      <c r="R48" s="2"/>
-      <c r="S48" s="2"/>
+      <c r="R48" s="2">
+        <v>5</v>
+      </c>
+      <c r="S48" s="2">
+        <v>1</v>
+      </c>
       <c r="T48" s="2">
         <v>3</v>
       </c>
@@ -5669,8 +5681,12 @@
       <c r="Q49" s="6">
         <v>2</v>
       </c>
-      <c r="R49" s="6"/>
-      <c r="S49" s="6"/>
+      <c r="R49" s="6">
+        <v>1</v>
+      </c>
+      <c r="S49" s="6">
+        <v>2</v>
+      </c>
       <c r="T49" s="6">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Actualizar - 06-15-lun 13:23
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71425F46-5AE7-475F-B1E7-AB00E29E8770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CE7D78F-93DB-4657-9E4B-C993BFD5B035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2263,8 +2263,12 @@
       <c r="C47" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="D47" s="13"/>
-      <c r="E47" s="13"/>
+      <c r="D47" s="13">
+        <v>0</v>
+      </c>
+      <c r="E47" s="13">
+        <v>0</v>
+      </c>
       <c r="F47" s="11" t="s">
         <v>66</v>
       </c>
@@ -5234,8 +5238,12 @@
       <c r="K42" s="2">
         <v>1</v>
       </c>
-      <c r="L42" s="2"/>
-      <c r="M42" s="2"/>
+      <c r="L42" s="2">
+        <v>2</v>
+      </c>
+      <c r="M42" s="2">
+        <v>0</v>
+      </c>
       <c r="N42" s="2">
         <v>1</v>
       </c>
@@ -5321,8 +5329,12 @@
       <c r="K43" s="6">
         <v>1</v>
       </c>
-      <c r="L43" s="6"/>
-      <c r="M43" s="6"/>
+      <c r="L43" s="6">
+        <v>0</v>
+      </c>
+      <c r="M43" s="6">
+        <v>2</v>
+      </c>
       <c r="N43" s="6">
         <v>3</v>
       </c>
@@ -5554,7 +5566,7 @@
       </c>
       <c r="C48" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D47),Fixture!D47&amp;"-"&amp;Fixture!E47,"")</f>
-        <v/>
+        <v>0-0</v>
       </c>
       <c r="D48" s="2">
         <v>4</v>
@@ -5580,8 +5592,12 @@
       <c r="K48" s="2">
         <v>1</v>
       </c>
-      <c r="L48" s="2"/>
-      <c r="M48" s="2"/>
+      <c r="L48" s="2">
+        <v>4</v>
+      </c>
+      <c r="M48" s="2">
+        <v>1</v>
+      </c>
       <c r="N48" s="2">
         <v>4</v>
       </c>
@@ -5667,8 +5683,12 @@
       <c r="K49" s="6">
         <v>2</v>
       </c>
-      <c r="L49" s="6"/>
-      <c r="M49" s="6"/>
+      <c r="L49" s="6">
+        <v>1</v>
+      </c>
+      <c r="M49" s="6">
+        <v>3</v>
+      </c>
       <c r="N49" s="6">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Actualizar - 06-15-lun 15:58
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CE7D78F-93DB-4657-9E4B-C993BFD5B035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A29CD60-B9A0-45EA-A3C5-3329C6EA722D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -2149,8 +2149,12 @@
       <c r="C41" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="D41" s="13"/>
-      <c r="E41" s="13"/>
+      <c r="D41" s="13">
+        <v>1</v>
+      </c>
+      <c r="E41" s="13">
+        <v>1</v>
+      </c>
       <c r="F41" s="11" t="s">
         <v>58</v>
       </c>
@@ -5212,7 +5216,7 @@
       </c>
       <c r="C42" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D41),Fixture!D41&amp;"-"&amp;Fixture!E41,"")</f>
-        <v/>
+        <v>1-1</v>
       </c>
       <c r="D42" s="2">
         <v>2</v>

</xml_diff>

<commit_message>
Actualizar - 06-15-lun 21:02
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A29CD60-B9A0-45EA-A3C5-3329C6EA722D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{959644F5-F8FB-4D57-B7AE-56C5211D9C75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -2290,8 +2290,12 @@
       <c r="C48" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="D48" s="13"/>
-      <c r="E48" s="13"/>
+      <c r="D48" s="13">
+        <v>1</v>
+      </c>
+      <c r="E48" s="13">
+        <v>1</v>
+      </c>
       <c r="F48" s="14" t="s">
         <v>68</v>
       </c>
@@ -5210,7 +5214,7 @@
       <c r="A42" s="12">
         <v>37</v>
       </c>
-      <c r="B42" s="11" t="str">
+      <c r="B42" s="44" t="str">
         <f>Fixture!C41&amp;" vs "&amp;Fixture!F41</f>
         <v>Bélgica vs Egipto</v>
       </c>
@@ -5564,7 +5568,7 @@
       <c r="A48" s="12">
         <v>43</v>
       </c>
-      <c r="B48" s="11" t="str">
+      <c r="B48" s="44" t="str">
         <f>Fixture!C47&amp;" vs "&amp;Fixture!F47</f>
         <v>España vs Cabo Verde</v>
       </c>
@@ -5655,13 +5659,13 @@
       <c r="A49" s="15">
         <v>44</v>
       </c>
-      <c r="B49" s="14" t="str">
+      <c r="B49" s="45" t="str">
         <f>Fixture!C48&amp;" vs "&amp;Fixture!F48</f>
         <v>Arabia Saudita vs Uruguay</v>
       </c>
       <c r="C49" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D48),Fixture!D48&amp;"-"&amp;Fixture!E48,"")</f>
-        <v/>
+        <v>1-1</v>
       </c>
       <c r="D49" s="6">
         <v>1</v>
@@ -5926,26 +5930,50 @@
         <f>IF(ISNUMBER(Fixture!D53),Fixture!D53&amp;"-"&amp;Fixture!E53,"")</f>
         <v/>
       </c>
-      <c r="D54" s="2"/>
-      <c r="E54" s="2"/>
-      <c r="F54" s="2"/>
-      <c r="G54" s="2"/>
-      <c r="H54" s="2"/>
-      <c r="I54" s="2"/>
-      <c r="J54" s="2"/>
-      <c r="K54" s="2"/>
+      <c r="D54" s="2">
+        <v>2</v>
+      </c>
+      <c r="E54" s="2">
+        <v>0</v>
+      </c>
+      <c r="F54" s="2">
+        <v>3</v>
+      </c>
+      <c r="G54" s="2">
+        <v>1</v>
+      </c>
+      <c r="H54" s="2">
+        <v>3</v>
+      </c>
+      <c r="I54" s="2">
+        <v>0</v>
+      </c>
+      <c r="J54" s="2">
+        <v>1</v>
+      </c>
+      <c r="K54" s="2">
+        <v>1</v>
+      </c>
       <c r="L54" s="2"/>
       <c r="M54" s="2"/>
-      <c r="N54" s="2"/>
-      <c r="O54" s="2"/>
+      <c r="N54" s="2">
+        <v>3</v>
+      </c>
+      <c r="O54" s="2">
+        <v>1</v>
+      </c>
       <c r="P54" s="2"/>
       <c r="Q54" s="2"/>
       <c r="R54" s="2"/>
       <c r="S54" s="2"/>
       <c r="T54" s="2"/>
       <c r="U54" s="2"/>
-      <c r="V54" s="2"/>
-      <c r="W54" s="2"/>
+      <c r="V54" s="2">
+        <v>2</v>
+      </c>
+      <c r="W54" s="2">
+        <v>1</v>
+      </c>
       <c r="X54" s="2"/>
       <c r="Y54" s="2"/>
       <c r="Z54" s="2"/>
@@ -5969,26 +5997,50 @@
         <f>IF(ISNUMBER(Fixture!D54),Fixture!D54&amp;"-"&amp;Fixture!E54,"")</f>
         <v/>
       </c>
-      <c r="D55" s="6"/>
-      <c r="E55" s="6"/>
-      <c r="F55" s="6"/>
-      <c r="G55" s="6"/>
-      <c r="H55" s="6"/>
-      <c r="I55" s="6"/>
-      <c r="J55" s="6"/>
-      <c r="K55" s="6"/>
+      <c r="D55" s="6">
+        <v>0</v>
+      </c>
+      <c r="E55" s="6">
+        <v>6</v>
+      </c>
+      <c r="F55" s="6">
+        <v>1</v>
+      </c>
+      <c r="G55" s="6">
+        <v>2</v>
+      </c>
+      <c r="H55" s="6">
+        <v>0</v>
+      </c>
+      <c r="I55" s="6">
+        <v>5</v>
+      </c>
+      <c r="J55" s="6">
+        <v>2</v>
+      </c>
+      <c r="K55" s="6">
+        <v>1</v>
+      </c>
       <c r="L55" s="6"/>
       <c r="M55" s="6"/>
-      <c r="N55" s="6"/>
-      <c r="O55" s="6"/>
+      <c r="N55" s="6">
+        <v>0</v>
+      </c>
+      <c r="O55" s="6">
+        <v>4</v>
+      </c>
       <c r="P55" s="6"/>
       <c r="Q55" s="6"/>
       <c r="R55" s="6"/>
       <c r="S55" s="6"/>
       <c r="T55" s="6"/>
       <c r="U55" s="6"/>
-      <c r="V55" s="6"/>
-      <c r="W55" s="6"/>
+      <c r="V55" s="6">
+        <v>0</v>
+      </c>
+      <c r="W55" s="6">
+        <v>2</v>
+      </c>
       <c r="X55" s="6"/>
       <c r="Y55" s="6"/>
       <c r="Z55" s="6"/>
@@ -6184,26 +6236,50 @@
         <f>IF(ISNUMBER(Fixture!D59),Fixture!D59&amp;"-"&amp;Fixture!E59,"")</f>
         <v/>
       </c>
-      <c r="D60" s="2"/>
-      <c r="E60" s="2"/>
-      <c r="F60" s="2"/>
-      <c r="G60" s="2"/>
-      <c r="H60" s="2"/>
-      <c r="I60" s="2"/>
-      <c r="J60" s="2"/>
-      <c r="K60" s="2"/>
+      <c r="D60" s="2">
+        <v>2</v>
+      </c>
+      <c r="E60" s="2">
+        <v>0</v>
+      </c>
+      <c r="F60" s="2">
+        <v>3</v>
+      </c>
+      <c r="G60" s="2">
+        <v>2</v>
+      </c>
+      <c r="H60" s="2">
+        <v>3</v>
+      </c>
+      <c r="I60" s="2">
+        <v>1</v>
+      </c>
+      <c r="J60" s="2">
+        <v>2</v>
+      </c>
+      <c r="K60" s="2">
+        <v>2</v>
+      </c>
       <c r="L60" s="2"/>
       <c r="M60" s="2"/>
-      <c r="N60" s="2"/>
-      <c r="O60" s="2"/>
+      <c r="N60" s="2">
+        <v>2</v>
+      </c>
+      <c r="O60" s="2">
+        <v>1</v>
+      </c>
       <c r="P60" s="2"/>
       <c r="Q60" s="2"/>
       <c r="R60" s="2"/>
       <c r="S60" s="2"/>
       <c r="T60" s="2"/>
       <c r="U60" s="2"/>
-      <c r="V60" s="2"/>
-      <c r="W60" s="2"/>
+      <c r="V60" s="2">
+        <v>3</v>
+      </c>
+      <c r="W60" s="2">
+        <v>1</v>
+      </c>
       <c r="X60" s="2"/>
       <c r="Y60" s="2"/>
       <c r="Z60" s="2"/>
@@ -6227,26 +6303,50 @@
         <f>IF(ISNUMBER(Fixture!D60),Fixture!D60&amp;"-"&amp;Fixture!E60,"")</f>
         <v/>
       </c>
-      <c r="D61" s="6"/>
-      <c r="E61" s="6"/>
-      <c r="F61" s="6"/>
-      <c r="G61" s="6"/>
-      <c r="H61" s="6"/>
-      <c r="I61" s="6"/>
-      <c r="J61" s="6"/>
-      <c r="K61" s="6"/>
+      <c r="D61" s="6">
+        <v>1</v>
+      </c>
+      <c r="E61" s="6">
+        <v>0</v>
+      </c>
+      <c r="F61" s="6">
+        <v>2</v>
+      </c>
+      <c r="G61" s="6">
+        <v>1</v>
+      </c>
+      <c r="H61" s="6">
+        <v>1</v>
+      </c>
+      <c r="I61" s="6">
+        <v>0</v>
+      </c>
+      <c r="J61" s="6">
+        <v>3</v>
+      </c>
+      <c r="K61" s="6">
+        <v>0</v>
+      </c>
       <c r="L61" s="6"/>
       <c r="M61" s="6"/>
-      <c r="N61" s="6"/>
-      <c r="O61" s="6"/>
+      <c r="N61" s="6">
+        <v>2</v>
+      </c>
+      <c r="O61" s="6">
+        <v>0</v>
+      </c>
       <c r="P61" s="6"/>
       <c r="Q61" s="6"/>
       <c r="R61" s="6"/>
       <c r="S61" s="6"/>
       <c r="T61" s="6"/>
       <c r="U61" s="6"/>
-      <c r="V61" s="6"/>
-      <c r="W61" s="6"/>
+      <c r="V61" s="6">
+        <v>2</v>
+      </c>
+      <c r="W61" s="6">
+        <v>0</v>
+      </c>
       <c r="X61" s="6"/>
       <c r="Y61" s="6"/>
       <c r="Z61" s="6"/>

</xml_diff>

<commit_message>
Actualizar - 06-16-mar 13:26
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{959644F5-F8FB-4D57-B7AE-56C5211D9C75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35D1CBC3-AADA-4A22-B4CC-B9D59ADCF1EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5954,28 +5954,48 @@
       <c r="K54" s="2">
         <v>1</v>
       </c>
-      <c r="L54" s="2"/>
-      <c r="M54" s="2"/>
+      <c r="L54" s="2">
+        <v>3</v>
+      </c>
+      <c r="M54" s="2">
+        <v>1</v>
+      </c>
       <c r="N54" s="2">
         <v>3</v>
       </c>
       <c r="O54" s="2">
         <v>1</v>
       </c>
-      <c r="P54" s="2"/>
-      <c r="Q54" s="2"/>
-      <c r="R54" s="2"/>
-      <c r="S54" s="2"/>
-      <c r="T54" s="2"/>
-      <c r="U54" s="2"/>
+      <c r="P54" s="2">
+        <v>3</v>
+      </c>
+      <c r="Q54" s="2">
+        <v>1</v>
+      </c>
+      <c r="R54" s="2">
+        <v>2</v>
+      </c>
+      <c r="S54" s="2">
+        <v>1</v>
+      </c>
+      <c r="T54" s="2">
+        <v>2</v>
+      </c>
+      <c r="U54" s="2">
+        <v>1</v>
+      </c>
       <c r="V54" s="2">
         <v>2</v>
       </c>
       <c r="W54" s="2">
         <v>1</v>
       </c>
-      <c r="X54" s="2"/>
-      <c r="Y54" s="2"/>
+      <c r="X54" s="2">
+        <v>2</v>
+      </c>
+      <c r="Y54" s="2">
+        <v>1</v>
+      </c>
       <c r="Z54" s="2"/>
       <c r="AA54" s="2"/>
       <c r="AB54" s="2"/>
@@ -6021,28 +6041,48 @@
       <c r="K55" s="6">
         <v>1</v>
       </c>
-      <c r="L55" s="6"/>
-      <c r="M55" s="6"/>
+      <c r="L55" s="6">
+        <v>0</v>
+      </c>
+      <c r="M55" s="6">
+        <v>2</v>
+      </c>
       <c r="N55" s="6">
         <v>0</v>
       </c>
       <c r="O55" s="6">
         <v>4</v>
       </c>
-      <c r="P55" s="6"/>
-      <c r="Q55" s="6"/>
-      <c r="R55" s="6"/>
-      <c r="S55" s="6"/>
-      <c r="T55" s="6"/>
-      <c r="U55" s="6"/>
+      <c r="P55" s="6">
+        <v>1</v>
+      </c>
+      <c r="Q55" s="6">
+        <v>3</v>
+      </c>
+      <c r="R55" s="6">
+        <v>1</v>
+      </c>
+      <c r="S55" s="6">
+        <v>2</v>
+      </c>
+      <c r="T55" s="6">
+        <v>0</v>
+      </c>
+      <c r="U55" s="6">
+        <v>1</v>
+      </c>
       <c r="V55" s="6">
         <v>0</v>
       </c>
       <c r="W55" s="6">
         <v>2</v>
       </c>
-      <c r="X55" s="6"/>
-      <c r="Y55" s="6"/>
+      <c r="X55" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y55" s="6">
+        <v>2</v>
+      </c>
       <c r="Z55" s="6"/>
       <c r="AA55" s="6"/>
       <c r="AB55" s="6"/>
@@ -6260,28 +6300,48 @@
       <c r="K60" s="2">
         <v>2</v>
       </c>
-      <c r="L60" s="2"/>
-      <c r="M60" s="2"/>
+      <c r="L60" s="2">
+        <v>2</v>
+      </c>
+      <c r="M60" s="2">
+        <v>1</v>
+      </c>
       <c r="N60" s="2">
         <v>2</v>
       </c>
       <c r="O60" s="2">
         <v>1</v>
       </c>
-      <c r="P60" s="2"/>
-      <c r="Q60" s="2"/>
-      <c r="R60" s="2"/>
-      <c r="S60" s="2"/>
-      <c r="T60" s="2"/>
-      <c r="U60" s="2"/>
+      <c r="P60" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q60" s="2">
+        <v>1</v>
+      </c>
+      <c r="R60" s="2">
+        <v>2</v>
+      </c>
+      <c r="S60" s="2">
+        <v>0</v>
+      </c>
+      <c r="T60" s="2">
+        <v>2</v>
+      </c>
+      <c r="U60" s="2">
+        <v>0</v>
+      </c>
       <c r="V60" s="2">
         <v>3</v>
       </c>
       <c r="W60" s="2">
         <v>1</v>
       </c>
-      <c r="X60" s="2"/>
-      <c r="Y60" s="2"/>
+      <c r="X60" s="2">
+        <v>2</v>
+      </c>
+      <c r="Y60" s="2">
+        <v>1</v>
+      </c>
       <c r="Z60" s="2"/>
       <c r="AA60" s="2"/>
       <c r="AB60" s="2"/>
@@ -6327,28 +6387,48 @@
       <c r="K61" s="6">
         <v>0</v>
       </c>
-      <c r="L61" s="6"/>
-      <c r="M61" s="6"/>
+      <c r="L61" s="6">
+        <v>1</v>
+      </c>
+      <c r="M61" s="6">
+        <v>1</v>
+      </c>
       <c r="N61" s="6">
         <v>2</v>
       </c>
       <c r="O61" s="6">
         <v>0</v>
       </c>
-      <c r="P61" s="6"/>
-      <c r="Q61" s="6"/>
-      <c r="R61" s="6"/>
-      <c r="S61" s="6"/>
-      <c r="T61" s="6"/>
-      <c r="U61" s="6"/>
+      <c r="P61" s="6">
+        <v>2</v>
+      </c>
+      <c r="Q61" s="6">
+        <v>1</v>
+      </c>
+      <c r="R61" s="6">
+        <v>2</v>
+      </c>
+      <c r="S61" s="6">
+        <v>1</v>
+      </c>
+      <c r="T61" s="6">
+        <v>1</v>
+      </c>
+      <c r="U61" s="6">
+        <v>0</v>
+      </c>
       <c r="V61" s="6">
         <v>2</v>
       </c>
       <c r="W61" s="6">
         <v>0</v>
       </c>
-      <c r="X61" s="6"/>
-      <c r="Y61" s="6"/>
+      <c r="X61" s="6">
+        <v>2</v>
+      </c>
+      <c r="Y61" s="6">
+        <v>0</v>
+      </c>
       <c r="Z61" s="6"/>
       <c r="AA61" s="6"/>
       <c r="AB61" s="6"/>
@@ -6550,8 +6630,12 @@
       <c r="I66" s="2"/>
       <c r="J66" s="2"/>
       <c r="K66" s="2"/>
-      <c r="L66" s="2"/>
-      <c r="M66" s="2"/>
+      <c r="L66" s="2">
+        <v>2</v>
+      </c>
+      <c r="M66" s="2">
+        <v>1</v>
+      </c>
       <c r="N66" s="2"/>
       <c r="O66" s="2"/>
       <c r="P66" s="2"/>
@@ -6808,8 +6892,12 @@
       <c r="I72" s="2"/>
       <c r="J72" s="2"/>
       <c r="K72" s="2"/>
-      <c r="L72" s="2"/>
-      <c r="M72" s="2"/>
+      <c r="L72" s="2">
+        <v>1</v>
+      </c>
+      <c r="M72" s="2">
+        <v>2</v>
+      </c>
       <c r="N72" s="2"/>
       <c r="O72" s="2"/>
       <c r="P72" s="2"/>

</xml_diff>

<commit_message>
Actualizar - 06-16-mar 13:27
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35D1CBC3-AADA-4A22-B4CC-B9D59ADCF1EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D654AD3-506C-4A84-8809-848D6F685841}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6018,7 +6018,7 @@
         <v/>
       </c>
       <c r="D55" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E55" s="6">
         <v>6</v>

</xml_diff>

<commit_message>
Actualizar - 06-16-mar 13:33
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D654AD3-506C-4A84-8809-848D6F685841}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6051901A-9FF3-4B83-849B-08265085B260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2172,8 +2172,12 @@
       <c r="C42" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="D42" s="13"/>
-      <c r="E42" s="13"/>
+      <c r="D42" s="13">
+        <v>2</v>
+      </c>
+      <c r="E42" s="13">
+        <v>2</v>
+      </c>
       <c r="F42" s="14" t="s">
         <v>61</v>
       </c>
@@ -4951,7 +4955,7 @@
       <c r="A37" s="15">
         <v>32</v>
       </c>
-      <c r="B37" s="14" t="str">
+      <c r="B37" s="45" t="str">
         <f>Fixture!C36&amp;" vs "&amp;Fixture!F36</f>
         <v>Suecia vs Túnez</v>
       </c>
@@ -5305,13 +5309,13 @@
       <c r="A43" s="15">
         <v>38</v>
       </c>
-      <c r="B43" s="14" t="str">
+      <c r="B43" s="45" t="str">
         <f>Fixture!C42&amp;" vs "&amp;Fixture!F42</f>
         <v>Irán vs Nueva Zelanda</v>
       </c>
       <c r="C43" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D42),Fixture!D42&amp;"-"&amp;Fixture!E42,"")</f>
-        <v/>
+        <v>2-2</v>
       </c>
       <c r="D43" s="6">
         <v>1</v>
@@ -5996,8 +6000,12 @@
       <c r="Y54" s="2">
         <v>1</v>
       </c>
-      <c r="Z54" s="2"/>
-      <c r="AA54" s="2"/>
+      <c r="Z54" s="2">
+        <v>3</v>
+      </c>
+      <c r="AA54" s="2">
+        <v>1</v>
+      </c>
       <c r="AB54" s="2"/>
       <c r="AC54" s="2"/>
       <c r="AD54" s="2"/>
@@ -6083,8 +6091,12 @@
       <c r="Y55" s="6">
         <v>2</v>
       </c>
-      <c r="Z55" s="6"/>
-      <c r="AA55" s="6"/>
+      <c r="Z55" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA55" s="6">
+        <v>2</v>
+      </c>
       <c r="AB55" s="6"/>
       <c r="AC55" s="6"/>
       <c r="AD55" s="6"/>
@@ -6342,8 +6354,12 @@
       <c r="Y60" s="2">
         <v>1</v>
       </c>
-      <c r="Z60" s="2"/>
-      <c r="AA60" s="2"/>
+      <c r="Z60" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA60" s="2">
+        <v>0</v>
+      </c>
       <c r="AB60" s="2"/>
       <c r="AC60" s="2"/>
       <c r="AD60" s="2"/>
@@ -6429,8 +6445,12 @@
       <c r="Y61" s="6">
         <v>0</v>
       </c>
-      <c r="Z61" s="6"/>
-      <c r="AA61" s="6"/>
+      <c r="Z61" s="6">
+        <v>2</v>
+      </c>
+      <c r="AA61" s="6">
+        <v>1</v>
+      </c>
       <c r="AB61" s="6"/>
       <c r="AC61" s="6"/>
       <c r="AD61" s="6"/>
@@ -6622,8 +6642,12 @@
         <f>IF(ISNUMBER(Fixture!D65),Fixture!D65&amp;"-"&amp;Fixture!E65,"")</f>
         <v/>
       </c>
-      <c r="D66" s="2"/>
-      <c r="E66" s="2"/>
+      <c r="D66" s="2">
+        <v>4</v>
+      </c>
+      <c r="E66" s="2">
+        <v>1</v>
+      </c>
       <c r="F66" s="2"/>
       <c r="G66" s="2"/>
       <c r="H66" s="2"/>
@@ -6648,8 +6672,12 @@
       <c r="W66" s="2"/>
       <c r="X66" s="2"/>
       <c r="Y66" s="2"/>
-      <c r="Z66" s="2"/>
-      <c r="AA66" s="2"/>
+      <c r="Z66" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA66" s="2">
+        <v>0</v>
+      </c>
       <c r="AB66" s="2"/>
       <c r="AC66" s="2"/>
       <c r="AD66" s="2"/>
@@ -6669,8 +6697,12 @@
         <f>IF(ISNUMBER(Fixture!D66),Fixture!D66&amp;"-"&amp;Fixture!E66,"")</f>
         <v/>
       </c>
-      <c r="D67" s="6"/>
-      <c r="E67" s="6"/>
+      <c r="D67" s="6">
+        <v>0</v>
+      </c>
+      <c r="E67" s="6">
+        <v>3</v>
+      </c>
       <c r="F67" s="6"/>
       <c r="G67" s="6"/>
       <c r="H67" s="6"/>
@@ -6691,8 +6723,12 @@
       <c r="W67" s="6"/>
       <c r="X67" s="6"/>
       <c r="Y67" s="6"/>
-      <c r="Z67" s="6"/>
-      <c r="AA67" s="6"/>
+      <c r="Z67" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA67" s="6">
+        <v>2</v>
+      </c>
       <c r="AB67" s="6"/>
       <c r="AC67" s="6"/>
       <c r="AD67" s="6"/>
@@ -6884,8 +6920,12 @@
         <f>IF(ISNUMBER(Fixture!D71),Fixture!D71&amp;"-"&amp;Fixture!E71,"")</f>
         <v/>
       </c>
-      <c r="D72" s="2"/>
-      <c r="E72" s="2"/>
+      <c r="D72" s="2">
+        <v>2</v>
+      </c>
+      <c r="E72" s="2">
+        <v>3</v>
+      </c>
       <c r="F72" s="2"/>
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
@@ -6910,8 +6950,12 @@
       <c r="W72" s="2"/>
       <c r="X72" s="2"/>
       <c r="Y72" s="2"/>
-      <c r="Z72" s="2"/>
-      <c r="AA72" s="2"/>
+      <c r="Z72" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA72" s="2">
+        <v>1</v>
+      </c>
       <c r="AB72" s="2"/>
       <c r="AC72" s="2"/>
       <c r="AD72" s="2"/>
@@ -6931,8 +6975,12 @@
         <f>IF(ISNUMBER(Fixture!D72),Fixture!D72&amp;"-"&amp;Fixture!E72,"")</f>
         <v/>
       </c>
-      <c r="D73" s="6"/>
-      <c r="E73" s="6"/>
+      <c r="D73" s="6">
+        <v>3</v>
+      </c>
+      <c r="E73" s="6">
+        <v>1</v>
+      </c>
       <c r="F73" s="6"/>
       <c r="G73" s="6"/>
       <c r="H73" s="6"/>
@@ -6953,8 +7001,12 @@
       <c r="W73" s="6"/>
       <c r="X73" s="6"/>
       <c r="Y73" s="6"/>
-      <c r="Z73" s="6"/>
-      <c r="AA73" s="6"/>
+      <c r="Z73" s="6">
+        <v>1</v>
+      </c>
+      <c r="AA73" s="6">
+        <v>1</v>
+      </c>
       <c r="AB73" s="6"/>
       <c r="AC73" s="6"/>
       <c r="AD73" s="6"/>

</xml_diff>

<commit_message>
Actualizar - 06-16-mar 13:34
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6051901A-9FF3-4B83-849B-08265085B260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1564FEBA-4E68-4217-BBC6-53772A402F25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6650,8 +6650,12 @@
       </c>
       <c r="F66" s="2"/>
       <c r="G66" s="2"/>
-      <c r="H66" s="2"/>
-      <c r="I66" s="2"/>
+      <c r="H66" s="2">
+        <v>3</v>
+      </c>
+      <c r="I66" s="2">
+        <v>1</v>
+      </c>
       <c r="J66" s="2"/>
       <c r="K66" s="2"/>
       <c r="L66" s="2">
@@ -6705,8 +6709,12 @@
       </c>
       <c r="F67" s="6"/>
       <c r="G67" s="6"/>
-      <c r="H67" s="6"/>
-      <c r="I67" s="6"/>
+      <c r="H67" s="6">
+        <v>1</v>
+      </c>
+      <c r="I67" s="6">
+        <v>3</v>
+      </c>
       <c r="J67" s="6"/>
       <c r="K67" s="6"/>
       <c r="L67" s="6"/>
@@ -6928,8 +6936,12 @@
       </c>
       <c r="F72" s="2"/>
       <c r="G72" s="2"/>
-      <c r="H72" s="2"/>
-      <c r="I72" s="2"/>
+      <c r="H72" s="2">
+        <v>2</v>
+      </c>
+      <c r="I72" s="2">
+        <v>2</v>
+      </c>
       <c r="J72" s="2"/>
       <c r="K72" s="2"/>
       <c r="L72" s="2">
@@ -6983,8 +6995,12 @@
       </c>
       <c r="F73" s="6"/>
       <c r="G73" s="6"/>
-      <c r="H73" s="6"/>
-      <c r="I73" s="6"/>
+      <c r="H73" s="6">
+        <v>2</v>
+      </c>
+      <c r="I73" s="6">
+        <v>1</v>
+      </c>
       <c r="J73" s="6"/>
       <c r="K73" s="6"/>
       <c r="L73" s="6"/>

</xml_diff>

<commit_message>
Actualizar - 06-16-mar 13:35
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1564FEBA-4E68-4217-BBC6-53772A402F25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD031A95-611E-4711-8298-4E8EE4593B5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="114">
   <si>
     <t>🏆  QUINIELA MUNDIAL 2026</t>
   </si>
@@ -380,6 +380,9 @@
   </si>
   <si>
     <t xml:space="preserve">   </t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
 </sst>
 </file>
@@ -3611,10 +3614,18 @@
       <c r="O13" s="6">
         <v>2</v>
       </c>
-      <c r="P13" s="6"/>
-      <c r="Q13" s="6"/>
-      <c r="R13" s="6"/>
-      <c r="S13" s="6"/>
+      <c r="P13" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q13" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="R13" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="S13" s="6" t="s">
+        <v>113</v>
+      </c>
       <c r="T13" s="6">
         <v>0</v>
       </c>
@@ -3633,8 +3644,12 @@
       <c r="Y13" s="6">
         <v>3</v>
       </c>
-      <c r="Z13" s="6"/>
-      <c r="AA13" s="6"/>
+      <c r="Z13" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="AA13" s="6" t="s">
+        <v>113</v>
+      </c>
       <c r="AB13" s="6"/>
       <c r="AC13" s="6"/>
       <c r="AD13" s="6"/>
@@ -3868,8 +3883,12 @@
       <c r="Q18" s="2">
         <v>1</v>
       </c>
-      <c r="R18" s="2"/>
-      <c r="S18" s="2"/>
+      <c r="R18" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="S18" s="2" t="s">
+        <v>113</v>
+      </c>
       <c r="T18" s="2">
         <v>2</v>
       </c>
@@ -3955,8 +3974,12 @@
       <c r="Q19" s="6">
         <v>1</v>
       </c>
-      <c r="R19" s="6"/>
-      <c r="S19" s="6"/>
+      <c r="R19" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="S19" s="6" t="s">
+        <v>113</v>
+      </c>
       <c r="T19" s="6">
         <v>0</v>
       </c>
@@ -4305,8 +4328,12 @@
       <c r="Q25" s="6">
         <v>2</v>
       </c>
-      <c r="R25" s="6"/>
-      <c r="S25" s="6"/>
+      <c r="R25" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="S25" s="6" t="s">
+        <v>113</v>
+      </c>
       <c r="T25" s="6">
         <v>1</v>
       </c>
@@ -4325,8 +4352,12 @@
       <c r="Y25" s="6">
         <v>1</v>
       </c>
-      <c r="Z25" s="6"/>
-      <c r="AA25" s="6"/>
+      <c r="Z25" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="AA25" s="6" t="s">
+        <v>113</v>
+      </c>
       <c r="AB25" s="6"/>
       <c r="AC25" s="6"/>
       <c r="AD25" s="6"/>

</xml_diff>

<commit_message>
Actualizar - 06-16-mar 22:56
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD031A95-611E-4711-8298-4E8EE4593B5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52C09FE5-7676-42BD-B0C1-52E874F7579E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2396,8 +2396,12 @@
       <c r="C53" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="D53" s="13"/>
-      <c r="E53" s="13"/>
+      <c r="D53" s="13">
+        <v>3</v>
+      </c>
+      <c r="E53" s="13">
+        <v>1</v>
+      </c>
       <c r="F53" s="11" t="s">
         <v>71</v>
       </c>
@@ -2415,8 +2419,12 @@
       <c r="C54" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="D54" s="13"/>
-      <c r="E54" s="13"/>
+      <c r="D54" s="13">
+        <v>1</v>
+      </c>
+      <c r="E54" s="13">
+        <v>4</v>
+      </c>
       <c r="F54" s="14" t="s">
         <v>74</v>
       </c>
@@ -2510,8 +2518,12 @@
       <c r="C59" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="D59" s="13"/>
-      <c r="E59" s="13"/>
+      <c r="D59" s="13">
+        <v>3</v>
+      </c>
+      <c r="E59" s="13">
+        <v>0</v>
+      </c>
       <c r="F59" s="11" t="s">
         <v>78</v>
       </c>
@@ -5957,13 +5969,13 @@
       <c r="A54" s="12">
         <v>49</v>
       </c>
-      <c r="B54" s="11" t="str">
+      <c r="B54" s="44" t="str">
         <f>Fixture!C53&amp;" vs "&amp;Fixture!F53</f>
         <v>Francia vs Senegal</v>
       </c>
       <c r="C54" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D53),Fixture!D53&amp;"-"&amp;Fixture!E53,"")</f>
-        <v/>
+        <v>3-1</v>
       </c>
       <c r="D54" s="2">
         <v>2</v>
@@ -6048,13 +6060,13 @@
       <c r="A55" s="15">
         <v>50</v>
       </c>
-      <c r="B55" s="14" t="str">
+      <c r="B55" s="45" t="str">
         <f>Fixture!C54&amp;" vs "&amp;Fixture!F54</f>
         <v>Irak vs Noruega</v>
       </c>
       <c r="C55" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D54),Fixture!D54&amp;"-"&amp;Fixture!E54,"")</f>
-        <v/>
+        <v>1-4</v>
       </c>
       <c r="D55" s="6">
         <v>1</v>
@@ -6311,13 +6323,13 @@
       <c r="A60" s="12">
         <v>55</v>
       </c>
-      <c r="B60" s="11" t="str">
+      <c r="B60" s="44" t="str">
         <f>Fixture!C59&amp;" vs "&amp;Fixture!F59</f>
         <v>Argentina vs Argelia</v>
       </c>
       <c r="C60" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D59),Fixture!D59&amp;"-"&amp;Fixture!E59,"")</f>
-        <v/>
+        <v>3-0</v>
       </c>
       <c r="D60" s="2">
         <v>2</v>
@@ -6679,32 +6691,48 @@
       <c r="E66" s="2">
         <v>1</v>
       </c>
-      <c r="F66" s="2"/>
-      <c r="G66" s="2"/>
+      <c r="F66" s="2">
+        <v>3</v>
+      </c>
+      <c r="G66" s="2">
+        <v>0</v>
+      </c>
       <c r="H66" s="2">
+        <v>1</v>
+      </c>
+      <c r="I66" s="2">
+        <v>0</v>
+      </c>
+      <c r="J66" s="2">
         <v>3</v>
       </c>
-      <c r="I66" s="2">
-        <v>1</v>
-      </c>
-      <c r="J66" s="2"/>
-      <c r="K66" s="2"/>
+      <c r="K66" s="2">
+        <v>0</v>
+      </c>
       <c r="L66" s="2">
         <v>2</v>
       </c>
       <c r="M66" s="2">
         <v>1</v>
       </c>
-      <c r="N66" s="2"/>
-      <c r="O66" s="2"/>
+      <c r="N66" s="2">
+        <v>2</v>
+      </c>
+      <c r="O66" s="2">
+        <v>1</v>
+      </c>
       <c r="P66" s="2"/>
       <c r="Q66" s="2"/>
       <c r="R66" s="2"/>
       <c r="S66" s="2"/>
       <c r="T66" s="2"/>
       <c r="U66" s="2"/>
-      <c r="V66" s="2"/>
-      <c r="W66" s="2"/>
+      <c r="V66" s="2">
+        <v>2</v>
+      </c>
+      <c r="W66" s="2">
+        <v>0</v>
+      </c>
       <c r="X66" s="2"/>
       <c r="Y66" s="2"/>
       <c r="Z66" s="2">
@@ -6738,28 +6766,44 @@
       <c r="E67" s="6">
         <v>3</v>
       </c>
-      <c r="F67" s="6"/>
-      <c r="G67" s="6"/>
+      <c r="F67" s="6">
+        <v>1</v>
+      </c>
+      <c r="G67" s="6">
+        <v>2</v>
+      </c>
       <c r="H67" s="6">
         <v>1</v>
       </c>
       <c r="I67" s="6">
-        <v>3</v>
-      </c>
-      <c r="J67" s="6"/>
-      <c r="K67" s="6"/>
+        <v>2</v>
+      </c>
+      <c r="J67" s="6">
+        <v>0</v>
+      </c>
+      <c r="K67" s="6">
+        <v>2</v>
+      </c>
       <c r="L67" s="6"/>
       <c r="M67" s="6"/>
-      <c r="N67" s="6"/>
-      <c r="O67" s="6"/>
+      <c r="N67" s="6">
+        <v>1</v>
+      </c>
+      <c r="O67" s="6">
+        <v>2</v>
+      </c>
       <c r="P67" s="6"/>
       <c r="Q67" s="6"/>
       <c r="R67" s="6"/>
       <c r="S67" s="6"/>
       <c r="T67" s="6"/>
       <c r="U67" s="6"/>
-      <c r="V67" s="6"/>
-      <c r="W67" s="6"/>
+      <c r="V67" s="6">
+        <v>1</v>
+      </c>
+      <c r="W67" s="6">
+        <v>2</v>
+      </c>
       <c r="X67" s="6"/>
       <c r="Y67" s="6"/>
       <c r="Z67" s="6">
@@ -6965,32 +7009,48 @@
       <c r="E72" s="2">
         <v>3</v>
       </c>
-      <c r="F72" s="2"/>
-      <c r="G72" s="2"/>
+      <c r="F72" s="2">
+        <v>2</v>
+      </c>
+      <c r="G72" s="2">
+        <v>2</v>
+      </c>
       <c r="H72" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I72" s="2">
         <v>2</v>
       </c>
-      <c r="J72" s="2"/>
-      <c r="K72" s="2"/>
+      <c r="J72" s="2">
+        <v>1</v>
+      </c>
+      <c r="K72" s="2">
+        <v>0</v>
+      </c>
       <c r="L72" s="2">
         <v>1</v>
       </c>
       <c r="M72" s="2">
         <v>2</v>
       </c>
-      <c r="N72" s="2"/>
-      <c r="O72" s="2"/>
+      <c r="N72" s="2">
+        <v>2</v>
+      </c>
+      <c r="O72" s="2">
+        <v>2</v>
+      </c>
       <c r="P72" s="2"/>
       <c r="Q72" s="2"/>
       <c r="R72" s="2"/>
       <c r="S72" s="2"/>
       <c r="T72" s="2"/>
       <c r="U72" s="2"/>
-      <c r="V72" s="2"/>
-      <c r="W72" s="2"/>
+      <c r="V72" s="2">
+        <v>1</v>
+      </c>
+      <c r="W72" s="2">
+        <v>1</v>
+      </c>
       <c r="X72" s="2"/>
       <c r="Y72" s="2"/>
       <c r="Z72" s="2">
@@ -7024,28 +7084,44 @@
       <c r="E73" s="6">
         <v>1</v>
       </c>
-      <c r="F73" s="6"/>
-      <c r="G73" s="6"/>
+      <c r="F73" s="6">
+        <v>1</v>
+      </c>
+      <c r="G73" s="6">
+        <v>1</v>
+      </c>
       <c r="H73" s="6">
         <v>2</v>
       </c>
       <c r="I73" s="6">
         <v>1</v>
       </c>
-      <c r="J73" s="6"/>
-      <c r="K73" s="6"/>
+      <c r="J73" s="6">
+        <v>3</v>
+      </c>
+      <c r="K73" s="6">
+        <v>1</v>
+      </c>
       <c r="L73" s="6"/>
       <c r="M73" s="6"/>
-      <c r="N73" s="6"/>
-      <c r="O73" s="6"/>
+      <c r="N73" s="6">
+        <v>3</v>
+      </c>
+      <c r="O73" s="6">
+        <v>1</v>
+      </c>
       <c r="P73" s="6"/>
       <c r="Q73" s="6"/>
       <c r="R73" s="6"/>
       <c r="S73" s="6"/>
       <c r="T73" s="6"/>
       <c r="U73" s="6"/>
-      <c r="V73" s="6"/>
-      <c r="W73" s="6"/>
+      <c r="V73" s="6">
+        <v>2</v>
+      </c>
+      <c r="W73" s="6">
+        <v>1</v>
+      </c>
       <c r="X73" s="6"/>
       <c r="Y73" s="6"/>
       <c r="Z73" s="6">

</xml_diff>

<commit_message>
Actualizar - 06-23-mar 12:21
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52C09FE5-7676-42BD-B0C1-52E874F7579E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A783477-66DB-4663-92E7-47D3E7AB7A2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -58,9 +58,6 @@
     <t>Posición</t>
   </si>
   <si>
-    <t>Participante 13</t>
-  </si>
-  <si>
     <t>Participante 14</t>
   </si>
   <si>
@@ -383,6 +380,9 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>Cesar Lindarte</t>
   </si>
 </sst>
 </file>
@@ -797,13 +797,13 @@
     <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1090,12 +1090,12 @@
       <c r="D1" s="49"/>
     </row>
     <row r="2" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="47" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
+      <c r="A2" s="48" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
     </row>
     <row r="3" spans="1:4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1117,7 +1117,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C5" s="4">
         <v>0</v>
@@ -1132,7 +1132,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C6" s="8">
         <v>0</v>
@@ -1147,7 +1147,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C7" s="4">
         <v>0</v>
@@ -1162,7 +1162,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C8" s="8">
         <v>0</v>
@@ -1177,7 +1177,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C9" s="4">
         <v>0</v>
@@ -1192,7 +1192,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C10" s="8">
         <v>0</v>
@@ -1207,7 +1207,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C11" s="4">
         <v>0</v>
@@ -1222,7 +1222,7 @@
         <v>8</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C12" s="8">
         <v>0</v>
@@ -1237,7 +1237,7 @@
         <v>9</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C13" s="4">
         <v>0</v>
@@ -1252,7 +1252,7 @@
         <v>10</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C14" s="8">
         <v>0</v>
@@ -1267,7 +1267,7 @@
         <v>11</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C15" s="4">
         <v>0</v>
@@ -1282,7 +1282,7 @@
         <v>12</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C16" s="8">
         <v>0</v>
@@ -1297,7 +1297,7 @@
         <v>13</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>6</v>
+        <v>113</v>
       </c>
       <c r="C17" s="4">
         <v>0</v>
@@ -1312,7 +1312,7 @@
         <v>14</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C18" s="8">
         <v>0</v>
@@ -1327,7 +1327,7 @@
         <v>15</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C19" s="4">
         <v>0</v>
@@ -1362,26 +1362,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="47" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+    </row>
+    <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-    </row>
-    <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="47" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
     </row>
     <row r="3" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1389,22 +1389,22 @@
         <v>2</v>
       </c>
       <c r="B4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="D4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="E4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="F4" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="G4" s="10" t="s">
         <v>15</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1412,22 +1412,22 @@
         <v>1</v>
       </c>
       <c r="B5" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="D5" s="13">
+        <v>2</v>
+      </c>
+      <c r="E5" s="13">
+        <v>0</v>
+      </c>
+      <c r="F5" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="13">
-        <v>2</v>
-      </c>
-      <c r="E5" s="13">
-        <v>0</v>
-      </c>
-      <c r="F5" s="11" t="s">
+      <c r="G5" s="11" t="s">
         <v>19</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1435,22 +1435,22 @@
         <v>2</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C6" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="13">
+        <v>2</v>
+      </c>
+      <c r="E6" s="13">
+        <v>1</v>
+      </c>
+      <c r="F6" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="13">
-        <v>2</v>
-      </c>
-      <c r="E6" s="13">
-        <v>1</v>
-      </c>
-      <c r="F6" s="14" t="s">
-        <v>22</v>
-      </c>
       <c r="G6" s="14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1458,18 +1458,18 @@
         <v>3</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D7" s="13"/>
       <c r="E7" s="13"/>
       <c r="F7" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1477,18 +1477,18 @@
         <v>4</v>
       </c>
       <c r="B8" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="14" t="s">
         <v>17</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>18</v>
       </c>
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
       <c r="F8" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1496,18 +1496,18 @@
         <v>5</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D9" s="13"/>
       <c r="E9" s="13"/>
       <c r="F9" s="11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1515,18 +1515,18 @@
         <v>6</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D10" s="13"/>
       <c r="E10" s="13"/>
       <c r="F10" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1534,22 +1534,22 @@
         <v>7</v>
       </c>
       <c r="B11" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="D11" s="13">
+        <v>1</v>
+      </c>
+      <c r="E11" s="13">
+        <v>1</v>
+      </c>
+      <c r="F11" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="13">
-        <v>1</v>
-      </c>
-      <c r="E11" s="13">
-        <v>1</v>
-      </c>
-      <c r="F11" s="11" t="s">
+      <c r="G11" s="11" t="s">
         <v>27</v>
-      </c>
-      <c r="G11" s="11" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1557,22 +1557,22 @@
         <v>8</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C12" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="13">
+        <v>1</v>
+      </c>
+      <c r="E12" s="13">
+        <v>1</v>
+      </c>
+      <c r="F12" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="13">
-        <v>1</v>
-      </c>
-      <c r="E12" s="13">
-        <v>1</v>
-      </c>
-      <c r="F12" s="14" t="s">
+      <c r="G12" s="14" t="s">
         <v>30</v>
-      </c>
-      <c r="G12" s="14" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1580,18 +1580,18 @@
         <v>9</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D13" s="13"/>
       <c r="E13" s="13"/>
       <c r="F13" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1599,18 +1599,18 @@
         <v>10</v>
       </c>
       <c r="B14" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="14" t="s">
         <v>25</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>26</v>
       </c>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
       <c r="F14" s="14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1618,18 +1618,18 @@
         <v>11</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D15" s="13"/>
       <c r="E15" s="13"/>
       <c r="F15" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1637,18 +1637,18 @@
         <v>12</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D16" s="13"/>
       <c r="E16" s="13"/>
       <c r="F16" s="14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G16" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1656,25 +1656,25 @@
         <v>13</v>
       </c>
       <c r="B17" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="D17" s="13">
+        <v>1</v>
+      </c>
+      <c r="E17" s="13">
+        <v>1</v>
+      </c>
+      <c r="F17" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="D17" s="13">
-        <v>1</v>
-      </c>
-      <c r="E17" s="13">
-        <v>1</v>
-      </c>
-      <c r="F17" s="11" t="s">
-        <v>34</v>
-      </c>
       <c r="G17" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N17" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1682,22 +1682,22 @@
         <v>14</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C18" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D18" s="13">
+        <v>0</v>
+      </c>
+      <c r="E18" s="13">
+        <v>1</v>
+      </c>
+      <c r="F18" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="D18" s="13">
-        <v>0</v>
-      </c>
-      <c r="E18" s="13">
-        <v>1</v>
-      </c>
-      <c r="F18" s="14" t="s">
-        <v>36</v>
-      </c>
       <c r="G18" s="14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1705,18 +1705,18 @@
         <v>15</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D19" s="13"/>
       <c r="E19" s="13"/>
       <c r="F19" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1724,18 +1724,18 @@
         <v>16</v>
       </c>
       <c r="B20" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="C20" s="14" t="s">
         <v>32</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>33</v>
       </c>
       <c r="D20" s="13"/>
       <c r="E20" s="13"/>
       <c r="F20" s="14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G20" s="14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1743,18 +1743,18 @@
         <v>17</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D21" s="13"/>
       <c r="E21" s="13"/>
       <c r="F21" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="22" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1762,18 +1762,18 @@
         <v>18</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D22" s="13"/>
       <c r="E22" s="13"/>
       <c r="F22" s="14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G22" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1781,10 +1781,10 @@
         <v>19</v>
       </c>
       <c r="B23" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="C23" s="11" t="s">
         <v>38</v>
-      </c>
-      <c r="C23" s="11" t="s">
-        <v>39</v>
       </c>
       <c r="D23" s="13">
         <v>4</v>
@@ -1793,10 +1793,10 @@
         <v>1</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1804,22 +1804,22 @@
         <v>20</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C24" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D24" s="13">
+        <v>2</v>
+      </c>
+      <c r="E24" s="13">
+        <v>0</v>
+      </c>
+      <c r="F24" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="D24" s="13">
-        <v>2</v>
-      </c>
-      <c r="E24" s="13">
-        <v>0</v>
-      </c>
-      <c r="F24" s="14" t="s">
-        <v>42</v>
-      </c>
       <c r="G24" s="14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1827,18 +1827,18 @@
         <v>21</v>
       </c>
       <c r="B25" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" s="11" t="s">
         <v>38</v>
-      </c>
-      <c r="C25" s="11" t="s">
-        <v>39</v>
       </c>
       <c r="D25" s="13"/>
       <c r="E25" s="13"/>
       <c r="F25" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1846,18 +1846,18 @@
         <v>22</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D26" s="13"/>
       <c r="E26" s="13"/>
       <c r="F26" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G26" s="14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1865,18 +1865,18 @@
         <v>23</v>
       </c>
       <c r="B27" s="20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D27" s="13"/>
       <c r="E27" s="13"/>
       <c r="F27" s="11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="28" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1884,18 +1884,18 @@
         <v>24</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D28" s="13"/>
       <c r="E28" s="13"/>
       <c r="F28" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G28" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="29" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1903,10 +1903,10 @@
         <v>25</v>
       </c>
       <c r="B29" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" s="11" t="s">
         <v>44</v>
-      </c>
-      <c r="C29" s="11" t="s">
-        <v>45</v>
       </c>
       <c r="D29" s="13">
         <v>7</v>
@@ -1915,10 +1915,10 @@
         <v>1</v>
       </c>
       <c r="F29" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="G29" s="11" t="s">
         <v>46</v>
-      </c>
-      <c r="G29" s="11" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="30" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1926,22 +1926,22 @@
         <v>26</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C30" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="D30" s="13">
+        <v>1</v>
+      </c>
+      <c r="E30" s="13">
+        <v>0</v>
+      </c>
+      <c r="F30" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="D30" s="13">
-        <v>1</v>
-      </c>
-      <c r="E30" s="13">
-        <v>0</v>
-      </c>
-      <c r="F30" s="14" t="s">
-        <v>49</v>
-      </c>
       <c r="G30" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="31" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1949,18 +1949,18 @@
         <v>27</v>
       </c>
       <c r="B31" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="C31" s="11" t="s">
         <v>44</v>
-      </c>
-      <c r="C31" s="11" t="s">
-        <v>45</v>
       </c>
       <c r="D31" s="13"/>
       <c r="E31" s="13"/>
       <c r="F31" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="32" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1968,18 +1968,18 @@
         <v>28</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D32" s="13"/>
       <c r="E32" s="13"/>
       <c r="F32" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G32" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1987,18 +1987,18 @@
         <v>29</v>
       </c>
       <c r="B33" s="22" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D33" s="13"/>
       <c r="E33" s="13"/>
       <c r="F33" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2006,18 +2006,18 @@
         <v>30</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D34" s="13"/>
       <c r="E34" s="13"/>
       <c r="F34" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G34" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2025,22 +2025,22 @@
         <v>31</v>
       </c>
       <c r="B35" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="C35" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="C35" s="11" t="s">
+      <c r="D35" s="13">
+        <v>2</v>
+      </c>
+      <c r="E35" s="13">
+        <v>2</v>
+      </c>
+      <c r="F35" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="D35" s="13">
-        <v>2</v>
-      </c>
-      <c r="E35" s="13">
-        <v>2</v>
-      </c>
-      <c r="F35" s="11" t="s">
-        <v>53</v>
-      </c>
       <c r="G35" s="11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2048,10 +2048,10 @@
         <v>32</v>
       </c>
       <c r="B36" s="25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D36" s="13">
         <v>5</v>
@@ -2060,10 +2060,10 @@
         <v>1</v>
       </c>
       <c r="F36" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G36" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2071,18 +2071,18 @@
         <v>33</v>
       </c>
       <c r="B37" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="C37" s="11" t="s">
         <v>51</v>
-      </c>
-      <c r="C37" s="11" t="s">
-        <v>52</v>
       </c>
       <c r="D37" s="13"/>
       <c r="E37" s="13"/>
       <c r="F37" s="11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2090,18 +2090,18 @@
         <v>34</v>
       </c>
       <c r="B38" s="25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D38" s="13"/>
       <c r="E38" s="13"/>
       <c r="F38" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G38" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2109,18 +2109,18 @@
         <v>35</v>
       </c>
       <c r="B39" s="24" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D39" s="13"/>
       <c r="E39" s="13"/>
       <c r="F39" s="11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2128,18 +2128,18 @@
         <v>36</v>
       </c>
       <c r="B40" s="25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D40" s="13"/>
       <c r="E40" s="13"/>
       <c r="F40" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2147,22 +2147,22 @@
         <v>37</v>
       </c>
       <c r="B41" s="26" t="s">
+        <v>55</v>
+      </c>
+      <c r="C41" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="C41" s="11" t="s">
+      <c r="D41" s="13">
+        <v>1</v>
+      </c>
+      <c r="E41" s="13">
+        <v>1</v>
+      </c>
+      <c r="F41" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="D41" s="13">
-        <v>1</v>
-      </c>
-      <c r="E41" s="13">
-        <v>1</v>
-      </c>
-      <c r="F41" s="11" t="s">
+      <c r="G41" s="11" t="s">
         <v>58</v>
-      </c>
-      <c r="G41" s="11" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2170,22 +2170,22 @@
         <v>38</v>
       </c>
       <c r="B42" s="27" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C42" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="D42" s="13">
+        <v>2</v>
+      </c>
+      <c r="E42" s="13">
+        <v>2</v>
+      </c>
+      <c r="F42" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="D42" s="13">
-        <v>2</v>
-      </c>
-      <c r="E42" s="13">
-        <v>2</v>
-      </c>
-      <c r="F42" s="14" t="s">
-        <v>61</v>
-      </c>
       <c r="G42" s="14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2193,18 +2193,18 @@
         <v>39</v>
       </c>
       <c r="B43" s="26" t="s">
+        <v>55</v>
+      </c>
+      <c r="C43" s="11" t="s">
         <v>56</v>
-      </c>
-      <c r="C43" s="11" t="s">
-        <v>57</v>
       </c>
       <c r="D43" s="13"/>
       <c r="E43" s="13"/>
       <c r="F43" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G43" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2212,18 +2212,18 @@
         <v>40</v>
       </c>
       <c r="B44" s="27" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D44" s="13"/>
       <c r="E44" s="13"/>
       <c r="F44" s="14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G44" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2231,18 +2231,18 @@
         <v>41</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D45" s="13"/>
       <c r="E45" s="13"/>
       <c r="F45" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G45" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2250,18 +2250,18 @@
         <v>42</v>
       </c>
       <c r="B46" s="27" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D46" s="13"/>
       <c r="E46" s="13"/>
       <c r="F46" s="14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G46" s="14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2269,22 +2269,22 @@
         <v>43</v>
       </c>
       <c r="B47" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="C47" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="C47" s="11" t="s">
+      <c r="D47" s="13">
+        <v>0</v>
+      </c>
+      <c r="E47" s="13">
+        <v>0</v>
+      </c>
+      <c r="F47" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="D47" s="13">
-        <v>0</v>
-      </c>
-      <c r="E47" s="13">
-        <v>0</v>
-      </c>
-      <c r="F47" s="11" t="s">
-        <v>66</v>
-      </c>
       <c r="G47" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2292,22 +2292,22 @@
         <v>44</v>
       </c>
       <c r="B48" s="29" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C48" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D48" s="13">
+        <v>1</v>
+      </c>
+      <c r="E48" s="13">
+        <v>1</v>
+      </c>
+      <c r="F48" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="D48" s="13">
-        <v>1</v>
-      </c>
-      <c r="E48" s="13">
-        <v>1</v>
-      </c>
-      <c r="F48" s="14" t="s">
-        <v>68</v>
-      </c>
       <c r="G48" s="14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2315,18 +2315,18 @@
         <v>45</v>
       </c>
       <c r="B49" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="C49" s="11" t="s">
         <v>64</v>
-      </c>
-      <c r="C49" s="11" t="s">
-        <v>65</v>
       </c>
       <c r="D49" s="13"/>
       <c r="E49" s="13"/>
       <c r="F49" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G49" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2334,18 +2334,18 @@
         <v>46</v>
       </c>
       <c r="B50" s="29" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D50" s="13"/>
       <c r="E50" s="13"/>
       <c r="F50" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G50" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2353,18 +2353,18 @@
         <v>47</v>
       </c>
       <c r="B51" s="28" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D51" s="13"/>
       <c r="E51" s="13"/>
       <c r="F51" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G51" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2372,18 +2372,18 @@
         <v>48</v>
       </c>
       <c r="B52" s="29" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D52" s="13"/>
       <c r="E52" s="13"/>
       <c r="F52" s="14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G52" s="14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2391,10 +2391,10 @@
         <v>49</v>
       </c>
       <c r="B53" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="C53" s="11" t="s">
         <v>69</v>
-      </c>
-      <c r="C53" s="11" t="s">
-        <v>70</v>
       </c>
       <c r="D53" s="13">
         <v>3</v>
@@ -2403,10 +2403,10 @@
         <v>1</v>
       </c>
       <c r="F53" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="G53" s="11" t="s">
         <v>71</v>
-      </c>
-      <c r="G53" s="11" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2414,10 +2414,10 @@
         <v>50</v>
       </c>
       <c r="B54" s="31" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D54" s="13">
         <v>1</v>
@@ -2426,10 +2426,10 @@
         <v>4</v>
       </c>
       <c r="F54" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G54" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2437,18 +2437,18 @@
         <v>51</v>
       </c>
       <c r="B55" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="C55" s="11" t="s">
         <v>69</v>
-      </c>
-      <c r="C55" s="11" t="s">
-        <v>70</v>
       </c>
       <c r="D55" s="13"/>
       <c r="E55" s="13"/>
       <c r="F55" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G55" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2456,18 +2456,18 @@
         <v>52</v>
       </c>
       <c r="B56" s="31" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D56" s="13"/>
       <c r="E56" s="13"/>
       <c r="F56" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G56" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2475,18 +2475,18 @@
         <v>53</v>
       </c>
       <c r="B57" s="30" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C57" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D57" s="13"/>
       <c r="E57" s="13"/>
       <c r="F57" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G57" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2494,18 +2494,18 @@
         <v>54</v>
       </c>
       <c r="B58" s="31" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D58" s="13"/>
       <c r="E58" s="13"/>
       <c r="F58" s="14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G58" s="14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2513,10 +2513,10 @@
         <v>55</v>
       </c>
       <c r="B59" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="C59" s="11" t="s">
         <v>76</v>
-      </c>
-      <c r="C59" s="11" t="s">
-        <v>77</v>
       </c>
       <c r="D59" s="13">
         <v>3</v>
@@ -2525,10 +2525,10 @@
         <v>0</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G59" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2536,18 +2536,18 @@
         <v>56</v>
       </c>
       <c r="B60" s="33" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C60" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D60" s="13"/>
       <c r="E60" s="13"/>
       <c r="F60" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G60" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2555,18 +2555,18 @@
         <v>57</v>
       </c>
       <c r="B61" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="C61" s="11" t="s">
         <v>76</v>
-      </c>
-      <c r="C61" s="11" t="s">
-        <v>77</v>
       </c>
       <c r="D61" s="13"/>
       <c r="E61" s="13"/>
       <c r="F61" s="11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G61" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2574,18 +2574,18 @@
         <v>58</v>
       </c>
       <c r="B62" s="33" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C62" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D62" s="13"/>
       <c r="E62" s="13"/>
       <c r="F62" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G62" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2593,18 +2593,18 @@
         <v>59</v>
       </c>
       <c r="B63" s="32" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C63" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D63" s="13"/>
       <c r="E63" s="13"/>
       <c r="F63" s="11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G63" s="11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2612,18 +2612,18 @@
         <v>60</v>
       </c>
       <c r="B64" s="33" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C64" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D64" s="13"/>
       <c r="E64" s="13"/>
       <c r="F64" s="14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G64" s="14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2631,18 +2631,18 @@
         <v>61</v>
       </c>
       <c r="B65" s="34" t="s">
+        <v>81</v>
+      </c>
+      <c r="C65" s="11" t="s">
         <v>82</v>
-      </c>
-      <c r="C65" s="11" t="s">
-        <v>83</v>
       </c>
       <c r="D65" s="13"/>
       <c r="E65" s="13"/>
       <c r="F65" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="G65" s="11" t="s">
         <v>84</v>
-      </c>
-      <c r="G65" s="11" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2650,18 +2650,18 @@
         <v>62</v>
       </c>
       <c r="B66" s="35" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D66" s="13"/>
       <c r="E66" s="13"/>
       <c r="F66" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G66" s="14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2669,18 +2669,18 @@
         <v>63</v>
       </c>
       <c r="B67" s="34" t="s">
+        <v>81</v>
+      </c>
+      <c r="C67" s="11" t="s">
         <v>82</v>
-      </c>
-      <c r="C67" s="11" t="s">
-        <v>83</v>
       </c>
       <c r="D67" s="13"/>
       <c r="E67" s="13"/>
       <c r="F67" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G67" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2688,18 +2688,18 @@
         <v>64</v>
       </c>
       <c r="B68" s="35" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C68" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D68" s="13"/>
       <c r="E68" s="13"/>
       <c r="F68" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G68" s="14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2707,18 +2707,18 @@
         <v>65</v>
       </c>
       <c r="B69" s="34" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C69" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D69" s="13"/>
       <c r="E69" s="13"/>
       <c r="F69" s="11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G69" s="11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2726,18 +2726,18 @@
         <v>66</v>
       </c>
       <c r="B70" s="35" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C70" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D70" s="13"/>
       <c r="E70" s="13"/>
       <c r="F70" s="14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G70" s="14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2745,18 +2745,18 @@
         <v>67</v>
       </c>
       <c r="B71" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="C71" s="11" t="s">
         <v>89</v>
-      </c>
-      <c r="C71" s="11" t="s">
-        <v>90</v>
       </c>
       <c r="D71" s="13"/>
       <c r="E71" s="13"/>
       <c r="F71" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G71" s="11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2764,18 +2764,18 @@
         <v>68</v>
       </c>
       <c r="B72" s="37" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C72" s="14" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D72" s="13"/>
       <c r="E72" s="13"/>
       <c r="F72" s="14" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G72" s="14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="73" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2783,18 +2783,18 @@
         <v>69</v>
       </c>
       <c r="B73" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="C73" s="11" t="s">
         <v>89</v>
-      </c>
-      <c r="C73" s="11" t="s">
-        <v>90</v>
       </c>
       <c r="D73" s="13"/>
       <c r="E73" s="13"/>
       <c r="F73" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G73" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="74" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2802,18 +2802,18 @@
         <v>70</v>
       </c>
       <c r="B74" s="37" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C74" s="14" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D74" s="13"/>
       <c r="E74" s="13"/>
       <c r="F74" s="14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G74" s="14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2821,18 +2821,18 @@
         <v>71</v>
       </c>
       <c r="B75" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="C75" s="11" t="s">
         <v>89</v>
-      </c>
-      <c r="C75" s="11" t="s">
-        <v>90</v>
       </c>
       <c r="D75" s="13"/>
       <c r="E75" s="13"/>
       <c r="F75" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G75" s="11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2840,18 +2840,18 @@
         <v>72</v>
       </c>
       <c r="B76" s="37" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C76" s="14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D76" s="13"/>
       <c r="E76" s="13"/>
       <c r="F76" s="14" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G76" s="14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -2876,78 +2876,78 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="47" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
+      <c r="L1" s="47"/>
+      <c r="M1" s="47"/>
+      <c r="N1" s="47"/>
+      <c r="O1" s="47"/>
+      <c r="P1" s="47"/>
+      <c r="Q1" s="47"/>
+      <c r="R1" s="47"/>
+      <c r="S1" s="47"/>
+      <c r="T1" s="47"/>
+      <c r="U1" s="47"/>
+      <c r="V1" s="47"/>
+      <c r="W1" s="47"/>
+      <c r="X1" s="47"/>
+      <c r="Y1" s="47"/>
+      <c r="Z1" s="47"/>
+      <c r="AA1" s="47"/>
+      <c r="AB1" s="47"/>
+      <c r="AC1" s="47"/>
+      <c r="AD1" s="47"/>
+      <c r="AE1" s="47"/>
+      <c r="AF1" s="47"/>
+      <c r="AG1" s="47"/>
+    </row>
+    <row r="2" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="48" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
-      <c r="M1" s="46"/>
-      <c r="N1" s="46"/>
-      <c r="O1" s="46"/>
-      <c r="P1" s="46"/>
-      <c r="Q1" s="46"/>
-      <c r="R1" s="46"/>
-      <c r="S1" s="46"/>
-      <c r="T1" s="46"/>
-      <c r="U1" s="46"/>
-      <c r="V1" s="46"/>
-      <c r="W1" s="46"/>
-      <c r="X1" s="46"/>
-      <c r="Y1" s="46"/>
-      <c r="Z1" s="46"/>
-      <c r="AA1" s="46"/>
-      <c r="AB1" s="46"/>
-      <c r="AC1" s="46"/>
-      <c r="AD1" s="46"/>
-      <c r="AE1" s="46"/>
-      <c r="AF1" s="46"/>
-      <c r="AG1" s="46"/>
-    </row>
-    <row r="2" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="47" t="s">
-        <v>95</v>
-      </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
-      <c r="K2" s="47"/>
-      <c r="L2" s="47"/>
-      <c r="M2" s="47"/>
-      <c r="N2" s="47"/>
-      <c r="O2" s="47"/>
-      <c r="P2" s="47"/>
-      <c r="Q2" s="47"/>
-      <c r="R2" s="47"/>
-      <c r="S2" s="47"/>
-      <c r="T2" s="47"/>
-      <c r="U2" s="47"/>
-      <c r="V2" s="47"/>
-      <c r="W2" s="47"/>
-      <c r="X2" s="47"/>
-      <c r="Y2" s="47"/>
-      <c r="Z2" s="47"/>
-      <c r="AA2" s="47"/>
-      <c r="AB2" s="47"/>
-      <c r="AC2" s="47"/>
-      <c r="AD2" s="47"/>
-      <c r="AE2" s="47"/>
-      <c r="AF2" s="47"/>
-      <c r="AG2" s="47"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
+      <c r="I2" s="48"/>
+      <c r="J2" s="48"/>
+      <c r="K2" s="48"/>
+      <c r="L2" s="48"/>
+      <c r="M2" s="48"/>
+      <c r="N2" s="48"/>
+      <c r="O2" s="48"/>
+      <c r="P2" s="48"/>
+      <c r="Q2" s="48"/>
+      <c r="R2" s="48"/>
+      <c r="S2" s="48"/>
+      <c r="T2" s="48"/>
+      <c r="U2" s="48"/>
+      <c r="V2" s="48"/>
+      <c r="W2" s="48"/>
+      <c r="X2" s="48"/>
+      <c r="Y2" s="48"/>
+      <c r="Z2" s="48"/>
+      <c r="AA2" s="48"/>
+      <c r="AB2" s="48"/>
+      <c r="AC2" s="48"/>
+      <c r="AD2" s="48"/>
+      <c r="AE2" s="48"/>
+      <c r="AF2" s="48"/>
+      <c r="AG2" s="48"/>
     </row>
     <row r="3" spans="1:33" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2955,182 +2955,182 @@
         <v>2</v>
       </c>
       <c r="B4" s="38" t="s">
+        <v>95</v>
+      </c>
+      <c r="C4" s="39" t="s">
         <v>96</v>
       </c>
-      <c r="C4" s="39" t="s">
-        <v>97</v>
-      </c>
-      <c r="D4" s="48" t="str">
+      <c r="D4" s="46" t="str">
         <f>Participantes!B5</f>
         <v>Andres Jesús</v>
       </c>
-      <c r="E4" s="48"/>
-      <c r="F4" s="48" t="str">
+      <c r="E4" s="46"/>
+      <c r="F4" s="46" t="str">
         <f>Participantes!B6</f>
         <v>Leonardo Fabio</v>
       </c>
-      <c r="G4" s="48"/>
-      <c r="H4" s="48" t="str">
+      <c r="G4" s="46"/>
+      <c r="H4" s="46" t="str">
         <f>Participantes!B7</f>
         <v>Martha Cenidia</v>
       </c>
-      <c r="I4" s="48"/>
-      <c r="J4" s="48" t="str">
+      <c r="I4" s="46"/>
+      <c r="J4" s="46" t="str">
         <f>Participantes!B8</f>
         <v>Freddy Ramón</v>
       </c>
-      <c r="K4" s="48"/>
-      <c r="L4" s="48" t="str">
+      <c r="K4" s="46"/>
+      <c r="L4" s="46" t="str">
         <f>Participantes!B9</f>
         <v xml:space="preserve">Juan Camilo </v>
       </c>
-      <c r="M4" s="48"/>
-      <c r="N4" s="48" t="str">
+      <c r="M4" s="46"/>
+      <c r="N4" s="46" t="str">
         <f>Participantes!B10</f>
         <v xml:space="preserve">Juan David </v>
       </c>
-      <c r="O4" s="48"/>
-      <c r="P4" s="48" t="str">
+      <c r="O4" s="46"/>
+      <c r="P4" s="46" t="str">
         <f>Participantes!B11</f>
         <v>María Trinidad</v>
       </c>
-      <c r="Q4" s="48"/>
-      <c r="R4" s="48" t="str">
+      <c r="Q4" s="46"/>
+      <c r="R4" s="46" t="str">
         <f>Participantes!B12</f>
         <v xml:space="preserve">María Gabriela </v>
       </c>
-      <c r="S4" s="48"/>
-      <c r="T4" s="48" t="str">
+      <c r="S4" s="46"/>
+      <c r="T4" s="46" t="str">
         <f>Participantes!B13</f>
         <v>Laura Valentina</v>
       </c>
-      <c r="U4" s="48"/>
-      <c r="V4" s="48" t="str">
+      <c r="U4" s="46"/>
+      <c r="V4" s="46" t="str">
         <f>Participantes!B14</f>
         <v>Gloria Isabel</v>
       </c>
-      <c r="W4" s="48"/>
-      <c r="X4" s="48" t="str">
+      <c r="W4" s="46"/>
+      <c r="X4" s="46" t="str">
         <f>Participantes!B15</f>
         <v xml:space="preserve">María del Pilar </v>
       </c>
-      <c r="Y4" s="48"/>
-      <c r="Z4" s="48" t="str">
+      <c r="Y4" s="46"/>
+      <c r="Z4" s="46" t="str">
         <f>Participantes!B16</f>
         <v>Jaime Andres</v>
       </c>
-      <c r="AA4" s="48"/>
-      <c r="AB4" s="48" t="str">
+      <c r="AA4" s="46"/>
+      <c r="AB4" s="46" t="str">
         <f>Participantes!B17</f>
-        <v>Participante 13</v>
-      </c>
-      <c r="AC4" s="48"/>
-      <c r="AD4" s="48" t="str">
+        <v>Cesar Lindarte</v>
+      </c>
+      <c r="AC4" s="46"/>
+      <c r="AD4" s="46" t="str">
         <f>Participantes!B18</f>
         <v>Participante 14</v>
       </c>
-      <c r="AE4" s="48"/>
-      <c r="AF4" s="48" t="str">
+      <c r="AE4" s="46"/>
+      <c r="AF4" s="46" t="str">
         <f>Participantes!B19</f>
         <v>Participante 15</v>
       </c>
-      <c r="AG4" s="48"/>
+      <c r="AG4" s="46"/>
     </row>
     <row r="5" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="40"/>
       <c r="B5" s="40"/>
       <c r="C5" s="41" t="s">
+        <v>97</v>
+      </c>
+      <c r="D5" s="42" t="s">
+        <v>88</v>
+      </c>
+      <c r="E5" s="42" t="s">
         <v>98</v>
       </c>
-      <c r="D5" s="42" t="s">
-        <v>89</v>
-      </c>
-      <c r="E5" s="42" t="s">
-        <v>99</v>
-      </c>
       <c r="F5" s="42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G5" s="42" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H5" s="42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I5" s="42" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J5" s="42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="K5" s="42" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="L5" s="42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="M5" s="42" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N5" s="42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O5" s="42" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="P5" s="42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="Q5" s="42" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="R5" s="42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="S5" s="42" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="T5" s="42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="U5" s="42" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="V5" s="42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="W5" s="42" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="X5" s="42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="Y5" s="42" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="Z5" s="42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AA5" s="42" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="AB5" s="42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AC5" s="42" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="AD5" s="42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AE5" s="42" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="AF5" s="42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AG5" s="42" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:33" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3627,16 +3627,16 @@
         <v>2</v>
       </c>
       <c r="P13" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="Q13" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="R13" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="S13" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="T13" s="6">
         <v>0</v>
@@ -3657,10 +3657,10 @@
         <v>3</v>
       </c>
       <c r="Z13" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AA13" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AB13" s="6"/>
       <c r="AC13" s="6"/>
@@ -3896,10 +3896,10 @@
         <v>1</v>
       </c>
       <c r="R18" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="S18" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="T18" s="2">
         <v>2</v>
@@ -3987,10 +3987,10 @@
         <v>1</v>
       </c>
       <c r="R19" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="S19" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="T19" s="6">
         <v>0</v>
@@ -4341,10 +4341,10 @@
         <v>2</v>
       </c>
       <c r="R25" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="S25" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="T25" s="6">
         <v>1</v>
@@ -4365,10 +4365,10 @@
         <v>1</v>
       </c>
       <c r="Z25" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AA25" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AB25" s="6"/>
       <c r="AC25" s="6"/>
@@ -7311,6 +7311,7 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="AD4:AE4"/>
     <mergeCell ref="AF4:AG4"/>
     <mergeCell ref="A1:AG1"/>
     <mergeCell ref="A2:AG2"/>
@@ -7327,7 +7328,6 @@
     <mergeCell ref="X4:Y4"/>
     <mergeCell ref="Z4:AA4"/>
     <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AD4:AE4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Actualizar - 06-23-mar 12:32
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\web poll\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A783477-66DB-4663-92E7-47D3E7AB7A2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24785528-BABD-4781-934F-17A054BA5165}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="112">
   <si>
     <t>🏆  QUINIELA MUNDIAL 2026</t>
   </si>
@@ -374,12 +374,6 @@
   </si>
   <si>
     <t>Jaime Andres</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   </t>
-  </si>
-  <si>
-    <t>-</t>
   </si>
   <si>
     <t>Cesar Lindarte</t>
@@ -558,7 +552,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -607,18 +601,6 @@
         <bgColor rgb="FF1A6B5C"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
-        <bgColor rgb="FFE2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
-        <bgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -660,7 +642,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -789,12 +771,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1082,20 +1058,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
     </row>
     <row r="2" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
     </row>
     <row r="3" spans="1:4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1297,7 +1273,7 @@
         <v>13</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C17" s="4">
         <v>0</v>
@@ -1349,7 +1325,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:N76"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -1362,26 +1338,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="47"/>
-      <c r="G1" s="47"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
     </row>
     <row r="3" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1417,12 +1393,8 @@
       <c r="C5" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="13">
-        <v>2</v>
-      </c>
-      <c r="E5" s="13">
-        <v>0</v>
-      </c>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
       <c r="F5" s="11" t="s">
         <v>18</v>
       </c>
@@ -1440,12 +1412,8 @@
       <c r="C6" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="13">
-        <v>2</v>
-      </c>
-      <c r="E6" s="13">
-        <v>1</v>
-      </c>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
       <c r="F6" s="14" t="s">
         <v>21</v>
       </c>
@@ -1539,12 +1507,8 @@
       <c r="C11" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="13">
-        <v>1</v>
-      </c>
-      <c r="E11" s="13">
-        <v>1</v>
-      </c>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
       <c r="F11" s="11" t="s">
         <v>26</v>
       </c>
@@ -1562,12 +1526,8 @@
       <c r="C12" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="13">
-        <v>1</v>
-      </c>
-      <c r="E12" s="13">
-        <v>1</v>
-      </c>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
       <c r="F12" s="14" t="s">
         <v>29</v>
       </c>
@@ -1651,7 +1611,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11">
         <v>13</v>
       </c>
@@ -1661,23 +1621,16 @@
       <c r="C17" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="D17" s="13">
-        <v>1</v>
-      </c>
-      <c r="E17" s="13">
-        <v>1</v>
-      </c>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
       <c r="F17" s="11" t="s">
         <v>33</v>
       </c>
       <c r="G17" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="N17" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14">
         <v>14</v>
       </c>
@@ -1687,12 +1640,8 @@
       <c r="C18" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="D18" s="13">
-        <v>0</v>
-      </c>
-      <c r="E18" s="13">
-        <v>1</v>
-      </c>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
       <c r="F18" s="14" t="s">
         <v>35</v>
       </c>
@@ -1700,7 +1649,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11">
         <v>15</v>
       </c>
@@ -1719,7 +1668,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14">
         <v>16</v>
       </c>
@@ -1738,7 +1687,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="11">
         <v>17</v>
       </c>
@@ -1757,7 +1706,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14">
         <v>18</v>
       </c>
@@ -1776,7 +1725,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
         <v>19</v>
       </c>
@@ -1786,12 +1735,8 @@
       <c r="C23" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="D23" s="13">
-        <v>4</v>
-      </c>
-      <c r="E23" s="13">
-        <v>1</v>
-      </c>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
       <c r="F23" s="11" t="s">
         <v>39</v>
       </c>
@@ -1799,7 +1744,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14">
         <v>20</v>
       </c>
@@ -1809,12 +1754,8 @@
       <c r="C24" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="D24" s="13">
-        <v>2</v>
-      </c>
-      <c r="E24" s="13">
-        <v>0</v>
-      </c>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
       <c r="F24" s="14" t="s">
         <v>41</v>
       </c>
@@ -1822,7 +1763,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
         <v>21</v>
       </c>
@@ -1841,7 +1782,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14">
         <v>22</v>
       </c>
@@ -1860,7 +1801,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
         <v>23</v>
       </c>
@@ -1879,7 +1820,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14">
         <v>24</v>
       </c>
@@ -1898,7 +1839,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
         <v>25</v>
       </c>
@@ -1908,12 +1849,8 @@
       <c r="C29" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="D29" s="13">
-        <v>7</v>
-      </c>
-      <c r="E29" s="13">
-        <v>1</v>
-      </c>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
       <c r="F29" s="11" t="s">
         <v>45</v>
       </c>
@@ -1921,7 +1858,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14">
         <v>26</v>
       </c>
@@ -1931,12 +1868,8 @@
       <c r="C30" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="D30" s="13">
-        <v>1</v>
-      </c>
-      <c r="E30" s="13">
-        <v>0</v>
-      </c>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
       <c r="F30" s="14" t="s">
         <v>48</v>
       </c>
@@ -1944,7 +1877,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
         <v>27</v>
       </c>
@@ -1963,7 +1896,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="14">
         <v>28</v>
       </c>
@@ -2030,12 +1963,8 @@
       <c r="C35" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="D35" s="13">
-        <v>2</v>
-      </c>
-      <c r="E35" s="13">
-        <v>2</v>
-      </c>
+      <c r="D35" s="13"/>
+      <c r="E35" s="13"/>
       <c r="F35" s="11" t="s">
         <v>52</v>
       </c>
@@ -2053,12 +1982,8 @@
       <c r="C36" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="D36" s="13">
-        <v>5</v>
-      </c>
-      <c r="E36" s="13">
-        <v>1</v>
-      </c>
+      <c r="D36" s="13"/>
+      <c r="E36" s="13"/>
       <c r="F36" s="14" t="s">
         <v>54</v>
       </c>
@@ -2152,12 +2077,8 @@
       <c r="C41" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="D41" s="13">
-        <v>1</v>
-      </c>
-      <c r="E41" s="13">
-        <v>1</v>
-      </c>
+      <c r="D41" s="13"/>
+      <c r="E41" s="13"/>
       <c r="F41" s="11" t="s">
         <v>57</v>
       </c>
@@ -2175,12 +2096,8 @@
       <c r="C42" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="D42" s="13">
-        <v>2</v>
-      </c>
-      <c r="E42" s="13">
-        <v>2</v>
-      </c>
+      <c r="D42" s="13"/>
+      <c r="E42" s="13"/>
       <c r="F42" s="14" t="s">
         <v>60</v>
       </c>
@@ -2274,12 +2191,8 @@
       <c r="C47" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="D47" s="13">
-        <v>0</v>
-      </c>
-      <c r="E47" s="13">
-        <v>0</v>
-      </c>
+      <c r="D47" s="13"/>
+      <c r="E47" s="13"/>
       <c r="F47" s="11" t="s">
         <v>65</v>
       </c>
@@ -2297,12 +2210,8 @@
       <c r="C48" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="D48" s="13">
-        <v>1</v>
-      </c>
-      <c r="E48" s="13">
-        <v>1</v>
-      </c>
+      <c r="D48" s="13"/>
+      <c r="E48" s="13"/>
       <c r="F48" s="14" t="s">
         <v>67</v>
       </c>
@@ -2396,12 +2305,8 @@
       <c r="C53" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="D53" s="13">
-        <v>3</v>
-      </c>
-      <c r="E53" s="13">
-        <v>1</v>
-      </c>
+      <c r="D53" s="13"/>
+      <c r="E53" s="13"/>
       <c r="F53" s="11" t="s">
         <v>70</v>
       </c>
@@ -2419,12 +2324,8 @@
       <c r="C54" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="D54" s="13">
-        <v>1</v>
-      </c>
-      <c r="E54" s="13">
-        <v>4</v>
-      </c>
+      <c r="D54" s="13"/>
+      <c r="E54" s="13"/>
       <c r="F54" s="14" t="s">
         <v>73</v>
       </c>
@@ -2518,12 +2419,8 @@
       <c r="C59" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="D59" s="13">
-        <v>3</v>
-      </c>
-      <c r="E59" s="13">
-        <v>0</v>
-      </c>
+      <c r="D59" s="13"/>
+      <c r="E59" s="13"/>
       <c r="F59" s="11" t="s">
         <v>77</v>
       </c>
@@ -2876,78 +2773,78 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="45" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="47"/>
-      <c r="G1" s="47"/>
-      <c r="H1" s="47"/>
-      <c r="I1" s="47"/>
-      <c r="J1" s="47"/>
-      <c r="K1" s="47"/>
-      <c r="L1" s="47"/>
-      <c r="M1" s="47"/>
-      <c r="N1" s="47"/>
-      <c r="O1" s="47"/>
-      <c r="P1" s="47"/>
-      <c r="Q1" s="47"/>
-      <c r="R1" s="47"/>
-      <c r="S1" s="47"/>
-      <c r="T1" s="47"/>
-      <c r="U1" s="47"/>
-      <c r="V1" s="47"/>
-      <c r="W1" s="47"/>
-      <c r="X1" s="47"/>
-      <c r="Y1" s="47"/>
-      <c r="Z1" s="47"/>
-      <c r="AA1" s="47"/>
-      <c r="AB1" s="47"/>
-      <c r="AC1" s="47"/>
-      <c r="AD1" s="47"/>
-      <c r="AE1" s="47"/>
-      <c r="AF1" s="47"/>
-      <c r="AG1" s="47"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="45"/>
+      <c r="O1" s="45"/>
+      <c r="P1" s="45"/>
+      <c r="Q1" s="45"/>
+      <c r="R1" s="45"/>
+      <c r="S1" s="45"/>
+      <c r="T1" s="45"/>
+      <c r="U1" s="45"/>
+      <c r="V1" s="45"/>
+      <c r="W1" s="45"/>
+      <c r="X1" s="45"/>
+      <c r="Y1" s="45"/>
+      <c r="Z1" s="45"/>
+      <c r="AA1" s="45"/>
+      <c r="AB1" s="45"/>
+      <c r="AC1" s="45"/>
+      <c r="AD1" s="45"/>
+      <c r="AE1" s="45"/>
+      <c r="AF1" s="45"/>
+      <c r="AG1" s="45"/>
     </row>
     <row r="2" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="46" t="s">
         <v>94</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
-      <c r="I2" s="48"/>
-      <c r="J2" s="48"/>
-      <c r="K2" s="48"/>
-      <c r="L2" s="48"/>
-      <c r="M2" s="48"/>
-      <c r="N2" s="48"/>
-      <c r="O2" s="48"/>
-      <c r="P2" s="48"/>
-      <c r="Q2" s="48"/>
-      <c r="R2" s="48"/>
-      <c r="S2" s="48"/>
-      <c r="T2" s="48"/>
-      <c r="U2" s="48"/>
-      <c r="V2" s="48"/>
-      <c r="W2" s="48"/>
-      <c r="X2" s="48"/>
-      <c r="Y2" s="48"/>
-      <c r="Z2" s="48"/>
-      <c r="AA2" s="48"/>
-      <c r="AB2" s="48"/>
-      <c r="AC2" s="48"/>
-      <c r="AD2" s="48"/>
-      <c r="AE2" s="48"/>
-      <c r="AF2" s="48"/>
-      <c r="AG2" s="48"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+      <c r="J2" s="46"/>
+      <c r="K2" s="46"/>
+      <c r="L2" s="46"/>
+      <c r="M2" s="46"/>
+      <c r="N2" s="46"/>
+      <c r="O2" s="46"/>
+      <c r="P2" s="46"/>
+      <c r="Q2" s="46"/>
+      <c r="R2" s="46"/>
+      <c r="S2" s="46"/>
+      <c r="T2" s="46"/>
+      <c r="U2" s="46"/>
+      <c r="V2" s="46"/>
+      <c r="W2" s="46"/>
+      <c r="X2" s="46"/>
+      <c r="Y2" s="46"/>
+      <c r="Z2" s="46"/>
+      <c r="AA2" s="46"/>
+      <c r="AB2" s="46"/>
+      <c r="AC2" s="46"/>
+      <c r="AD2" s="46"/>
+      <c r="AE2" s="46"/>
+      <c r="AF2" s="46"/>
+      <c r="AG2" s="46"/>
     </row>
     <row r="3" spans="1:33" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2960,81 +2857,81 @@
       <c r="C4" s="39" t="s">
         <v>96</v>
       </c>
-      <c r="D4" s="46" t="str">
+      <c r="D4" s="44" t="str">
         <f>Participantes!B5</f>
         <v>Andres Jesús</v>
       </c>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46" t="str">
+      <c r="E4" s="44"/>
+      <c r="F4" s="44" t="str">
         <f>Participantes!B6</f>
         <v>Leonardo Fabio</v>
       </c>
-      <c r="G4" s="46"/>
-      <c r="H4" s="46" t="str">
+      <c r="G4" s="44"/>
+      <c r="H4" s="44" t="str">
         <f>Participantes!B7</f>
         <v>Martha Cenidia</v>
       </c>
-      <c r="I4" s="46"/>
-      <c r="J4" s="46" t="str">
+      <c r="I4" s="44"/>
+      <c r="J4" s="44" t="str">
         <f>Participantes!B8</f>
         <v>Freddy Ramón</v>
       </c>
-      <c r="K4" s="46"/>
-      <c r="L4" s="46" t="str">
+      <c r="K4" s="44"/>
+      <c r="L4" s="44" t="str">
         <f>Participantes!B9</f>
         <v xml:space="preserve">Juan Camilo </v>
       </c>
-      <c r="M4" s="46"/>
-      <c r="N4" s="46" t="str">
+      <c r="M4" s="44"/>
+      <c r="N4" s="44" t="str">
         <f>Participantes!B10</f>
         <v xml:space="preserve">Juan David </v>
       </c>
-      <c r="O4" s="46"/>
-      <c r="P4" s="46" t="str">
+      <c r="O4" s="44"/>
+      <c r="P4" s="44" t="str">
         <f>Participantes!B11</f>
         <v>María Trinidad</v>
       </c>
-      <c r="Q4" s="46"/>
-      <c r="R4" s="46" t="str">
+      <c r="Q4" s="44"/>
+      <c r="R4" s="44" t="str">
         <f>Participantes!B12</f>
         <v xml:space="preserve">María Gabriela </v>
       </c>
-      <c r="S4" s="46"/>
-      <c r="T4" s="46" t="str">
+      <c r="S4" s="44"/>
+      <c r="T4" s="44" t="str">
         <f>Participantes!B13</f>
         <v>Laura Valentina</v>
       </c>
-      <c r="U4" s="46"/>
-      <c r="V4" s="46" t="str">
+      <c r="U4" s="44"/>
+      <c r="V4" s="44" t="str">
         <f>Participantes!B14</f>
         <v>Gloria Isabel</v>
       </c>
-      <c r="W4" s="46"/>
-      <c r="X4" s="46" t="str">
+      <c r="W4" s="44"/>
+      <c r="X4" s="44" t="str">
         <f>Participantes!B15</f>
         <v xml:space="preserve">María del Pilar </v>
       </c>
-      <c r="Y4" s="46"/>
-      <c r="Z4" s="46" t="str">
+      <c r="Y4" s="44"/>
+      <c r="Z4" s="44" t="str">
         <f>Participantes!B16</f>
         <v>Jaime Andres</v>
       </c>
-      <c r="AA4" s="46"/>
-      <c r="AB4" s="46" t="str">
+      <c r="AA4" s="44"/>
+      <c r="AB4" s="44" t="str">
         <f>Participantes!B17</f>
         <v>Cesar Lindarte</v>
       </c>
-      <c r="AC4" s="46"/>
-      <c r="AD4" s="46" t="str">
+      <c r="AC4" s="44"/>
+      <c r="AD4" s="44" t="str">
         <f>Participantes!B18</f>
         <v>Participante 14</v>
       </c>
-      <c r="AE4" s="46"/>
-      <c r="AF4" s="46" t="str">
+      <c r="AE4" s="44"/>
+      <c r="AF4" s="44" t="str">
         <f>Participantes!B19</f>
         <v>Participante 15</v>
       </c>
-      <c r="AG4" s="46"/>
+      <c r="AG4" s="44"/>
     </row>
     <row r="5" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="40"/>
@@ -3137,13 +3034,13 @@
       <c r="A6" s="12">
         <v>1</v>
       </c>
-      <c r="B6" s="44" t="str">
+      <c r="B6" s="11" t="str">
         <f>Fixture!C5&amp;" vs "&amp;Fixture!F5</f>
         <v>México vs Sudáfrica</v>
       </c>
       <c r="C6" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D5),Fixture!D5&amp;"-"&amp;Fixture!E5,"")</f>
-        <v>2-0</v>
+        <v/>
       </c>
       <c r="D6" s="2">
         <v>2</v>
@@ -3188,10 +3085,10 @@
         <v>1</v>
       </c>
       <c r="R6" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S6" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T6" s="2">
         <v>2</v>
@@ -3206,10 +3103,10 @@
         <v>0</v>
       </c>
       <c r="X6" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y6" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z6" s="2">
         <v>2</v>
@@ -3228,13 +3125,13 @@
       <c r="A7" s="15">
         <v>2</v>
       </c>
-      <c r="B7" s="45" t="str">
+      <c r="B7" s="14" t="str">
         <f>Fixture!C6&amp;" vs "&amp;Fixture!F6</f>
         <v>Corea del Sur vs Chequia</v>
       </c>
       <c r="C7" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D6),Fixture!D6&amp;"-"&amp;Fixture!E6,"")</f>
-        <v>2-1</v>
+        <v/>
       </c>
       <c r="D7" s="6">
         <v>1</v>
@@ -3297,7 +3194,7 @@
         <v>0</v>
       </c>
       <c r="X7" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y7" s="6">
         <v>1</v>
@@ -3491,86 +3388,38 @@
       <c r="A12" s="12">
         <v>7</v>
       </c>
-      <c r="B12" s="44" t="str">
+      <c r="B12" s="11" t="str">
         <f>Fixture!C11&amp;" vs "&amp;Fixture!F11</f>
         <v>Canadá vs Bosnia-Herzegovina</v>
       </c>
       <c r="C12" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D11),Fixture!D11&amp;"-"&amp;Fixture!E11,"")</f>
-        <v>1-1</v>
-      </c>
-      <c r="D12" s="2">
-        <v>0</v>
-      </c>
-      <c r="E12" s="2">
-        <v>2</v>
-      </c>
-      <c r="F12" s="2">
-        <v>2</v>
-      </c>
-      <c r="G12" s="2">
-        <v>0</v>
-      </c>
-      <c r="H12" s="2">
-        <v>2</v>
-      </c>
-      <c r="I12" s="2">
-        <v>2</v>
-      </c>
-      <c r="J12" s="2">
-        <v>1</v>
-      </c>
-      <c r="K12" s="2">
-        <v>1</v>
-      </c>
-      <c r="L12" s="2">
-        <v>2</v>
-      </c>
-      <c r="M12" s="2">
-        <v>0</v>
-      </c>
-      <c r="N12" s="2">
-        <v>1</v>
-      </c>
-      <c r="O12" s="2">
-        <v>1</v>
-      </c>
-      <c r="P12" s="2">
-        <v>1</v>
-      </c>
-      <c r="Q12" s="2">
-        <v>0</v>
-      </c>
-      <c r="R12" s="2">
-        <v>1</v>
-      </c>
-      <c r="S12" s="2">
-        <v>0</v>
-      </c>
-      <c r="T12" s="2">
-        <v>1</v>
-      </c>
-      <c r="U12" s="2">
-        <v>0</v>
-      </c>
-      <c r="V12" s="2">
-        <v>1</v>
-      </c>
-      <c r="W12" s="2">
-        <v>1</v>
-      </c>
-      <c r="X12" s="2">
-        <v>1</v>
-      </c>
-      <c r="Y12" s="2">
-        <v>1</v>
-      </c>
-      <c r="Z12" s="2">
-        <v>2</v>
-      </c>
-      <c r="AA12" s="2">
-        <v>0</v>
-      </c>
+        <v/>
+      </c>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+      <c r="M12" s="2"/>
+      <c r="N12" s="2"/>
+      <c r="O12" s="2"/>
+      <c r="P12" s="2"/>
+      <c r="Q12" s="2"/>
+      <c r="R12" s="2"/>
+      <c r="S12" s="2"/>
+      <c r="T12" s="2"/>
+      <c r="U12" s="2"/>
+      <c r="V12" s="2"/>
+      <c r="W12" s="2"/>
+      <c r="X12" s="2"/>
+      <c r="Y12" s="2"/>
+      <c r="Z12" s="2"/>
+      <c r="AA12" s="2"/>
       <c r="AB12" s="2"/>
       <c r="AC12" s="2"/>
       <c r="AD12" s="2"/>
@@ -3582,86 +3431,38 @@
       <c r="A13" s="15">
         <v>8</v>
       </c>
-      <c r="B13" s="45" t="str">
+      <c r="B13" s="14" t="str">
         <f>Fixture!C12&amp;" vs "&amp;Fixture!F12</f>
         <v>Qatar vs Suiza</v>
       </c>
       <c r="C13" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D12),Fixture!D12&amp;"-"&amp;Fixture!E12,"")</f>
-        <v>1-1</v>
-      </c>
-      <c r="D13" s="6">
-        <v>0</v>
-      </c>
-      <c r="E13" s="6">
-        <v>2</v>
-      </c>
-      <c r="F13" s="6">
-        <v>0</v>
-      </c>
-      <c r="G13" s="6">
-        <v>2</v>
-      </c>
-      <c r="H13" s="6">
-        <v>0</v>
-      </c>
-      <c r="I13" s="6">
-        <v>2</v>
-      </c>
-      <c r="J13" s="6">
-        <v>2</v>
-      </c>
-      <c r="K13" s="6">
-        <v>1</v>
-      </c>
-      <c r="L13" s="6">
-        <v>0</v>
-      </c>
-      <c r="M13" s="6">
-        <v>3</v>
-      </c>
-      <c r="N13" s="6">
-        <v>0</v>
-      </c>
-      <c r="O13" s="6">
-        <v>2</v>
-      </c>
-      <c r="P13" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="Q13" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="R13" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="S13" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="T13" s="6">
-        <v>0</v>
-      </c>
-      <c r="U13" s="6">
-        <v>2</v>
-      </c>
-      <c r="V13" s="6">
-        <v>1</v>
-      </c>
-      <c r="W13" s="6">
-        <v>2</v>
-      </c>
-      <c r="X13" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y13" s="6">
-        <v>3</v>
-      </c>
-      <c r="Z13" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="AA13" s="6" t="s">
-        <v>112</v>
-      </c>
+        <v/>
+      </c>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="6"/>
+      <c r="S13" s="6"/>
+      <c r="T13" s="6"/>
+      <c r="U13" s="6"/>
+      <c r="V13" s="6"/>
+      <c r="W13" s="6"/>
+      <c r="X13" s="6"/>
+      <c r="Y13" s="6"/>
+      <c r="Z13" s="6"/>
+      <c r="AA13" s="6"/>
       <c r="AB13" s="6"/>
       <c r="AC13" s="6"/>
       <c r="AD13" s="6"/>
@@ -3845,86 +3646,38 @@
       <c r="A18" s="12">
         <v>13</v>
       </c>
-      <c r="B18" s="44" t="str">
+      <c r="B18" s="11" t="str">
         <f>Fixture!C17&amp;" vs "&amp;Fixture!F17</f>
         <v>Brasil vs Marruecos</v>
       </c>
       <c r="C18" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D17),Fixture!D17&amp;"-"&amp;Fixture!E17,"")</f>
-        <v>1-1</v>
-      </c>
-      <c r="D18" s="2">
-        <v>1</v>
-      </c>
-      <c r="E18" s="2">
-        <v>1</v>
-      </c>
-      <c r="F18" s="2">
-        <v>1</v>
-      </c>
-      <c r="G18" s="2">
-        <v>0</v>
-      </c>
-      <c r="H18" s="2">
-        <v>2</v>
-      </c>
-      <c r="I18" s="2">
-        <v>1</v>
-      </c>
-      <c r="J18" s="2">
-        <v>2</v>
-      </c>
-      <c r="K18" s="2">
-        <v>2</v>
-      </c>
-      <c r="L18" s="2">
-        <v>2</v>
-      </c>
-      <c r="M18" s="2">
-        <v>1</v>
-      </c>
-      <c r="N18" s="2">
-        <v>2</v>
-      </c>
-      <c r="O18" s="2">
-        <v>1</v>
-      </c>
-      <c r="P18" s="2">
-        <v>3</v>
-      </c>
-      <c r="Q18" s="2">
-        <v>1</v>
-      </c>
-      <c r="R18" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="S18" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="T18" s="2">
-        <v>2</v>
-      </c>
-      <c r="U18" s="2">
-        <v>1</v>
-      </c>
-      <c r="V18" s="2">
-        <v>2</v>
-      </c>
-      <c r="W18" s="2">
-        <v>2</v>
-      </c>
-      <c r="X18" s="2">
-        <v>2</v>
-      </c>
-      <c r="Y18" s="2">
-        <v>1</v>
-      </c>
-      <c r="Z18" s="2">
-        <v>2</v>
-      </c>
-      <c r="AA18" s="2">
-        <v>0</v>
-      </c>
+        <v/>
+      </c>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
+      <c r="L18" s="2"/>
+      <c r="M18" s="2"/>
+      <c r="N18" s="2"/>
+      <c r="O18" s="2"/>
+      <c r="P18" s="2"/>
+      <c r="Q18" s="2"/>
+      <c r="R18" s="2"/>
+      <c r="S18" s="2"/>
+      <c r="T18" s="2"/>
+      <c r="U18" s="2"/>
+      <c r="V18" s="2"/>
+      <c r="W18" s="2"/>
+      <c r="X18" s="2"/>
+      <c r="Y18" s="2"/>
+      <c r="Z18" s="2"/>
+      <c r="AA18" s="2"/>
       <c r="AB18" s="2"/>
       <c r="AC18" s="2"/>
       <c r="AD18" s="2"/>
@@ -3936,86 +3689,38 @@
       <c r="A19" s="15">
         <v>14</v>
       </c>
-      <c r="B19" s="45" t="str">
+      <c r="B19" s="14" t="str">
         <f>Fixture!C18&amp;" vs "&amp;Fixture!F18</f>
         <v>Haití vs Escocia</v>
       </c>
       <c r="C19" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D18),Fixture!D18&amp;"-"&amp;Fixture!E18,"")</f>
-        <v>0-1</v>
-      </c>
-      <c r="D19" s="6">
-        <v>0</v>
-      </c>
-      <c r="E19" s="6">
-        <v>2</v>
-      </c>
-      <c r="F19" s="6">
-        <v>1</v>
-      </c>
-      <c r="G19" s="6">
-        <v>2</v>
-      </c>
-      <c r="H19" s="6">
-        <v>0</v>
-      </c>
-      <c r="I19" s="6">
-        <v>2</v>
-      </c>
-      <c r="J19" s="6">
-        <v>0</v>
-      </c>
-      <c r="K19" s="6">
-        <v>4</v>
-      </c>
-      <c r="L19" s="6">
-        <v>0</v>
-      </c>
-      <c r="M19" s="6">
-        <v>2</v>
-      </c>
-      <c r="N19" s="6">
-        <v>0</v>
-      </c>
-      <c r="O19" s="6">
-        <v>3</v>
-      </c>
-      <c r="P19" s="6">
-        <v>1</v>
-      </c>
-      <c r="Q19" s="6">
-        <v>1</v>
-      </c>
-      <c r="R19" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="S19" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="T19" s="6">
-        <v>0</v>
-      </c>
-      <c r="U19" s="6">
-        <v>2</v>
-      </c>
-      <c r="V19" s="6">
-        <v>0</v>
-      </c>
-      <c r="W19" s="6">
-        <v>2</v>
-      </c>
-      <c r="X19" s="6">
-        <v>1</v>
-      </c>
-      <c r="Y19" s="6">
-        <v>3</v>
-      </c>
-      <c r="Z19" s="6">
-        <v>1</v>
-      </c>
-      <c r="AA19" s="6">
-        <v>1</v>
-      </c>
+        <v/>
+      </c>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+      <c r="K19" s="6"/>
+      <c r="L19" s="6"/>
+      <c r="M19" s="6"/>
+      <c r="N19" s="6"/>
+      <c r="O19" s="6"/>
+      <c r="P19" s="6"/>
+      <c r="Q19" s="6"/>
+      <c r="R19" s="6"/>
+      <c r="S19" s="6"/>
+      <c r="T19" s="6"/>
+      <c r="U19" s="6"/>
+      <c r="V19" s="6"/>
+      <c r="W19" s="6"/>
+      <c r="X19" s="6"/>
+      <c r="Y19" s="6"/>
+      <c r="Z19" s="6"/>
+      <c r="AA19" s="6"/>
       <c r="AB19" s="6"/>
       <c r="AC19" s="6"/>
       <c r="AD19" s="6"/>
@@ -4199,86 +3904,38 @@
       <c r="A24" s="12">
         <v>19</v>
       </c>
-      <c r="B24" s="44" t="str">
+      <c r="B24" s="11" t="str">
         <f>Fixture!C23&amp;" vs "&amp;Fixture!F23</f>
         <v>Estados Unidos vs Paraguay</v>
       </c>
       <c r="C24" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D23),Fixture!D23&amp;"-"&amp;Fixture!E23,"")</f>
-        <v>4-1</v>
-      </c>
-      <c r="D24" s="2">
-        <v>2</v>
-      </c>
-      <c r="E24" s="2">
-        <v>0</v>
-      </c>
-      <c r="F24" s="2">
-        <v>0</v>
-      </c>
-      <c r="G24" s="2">
-        <v>1</v>
-      </c>
-      <c r="H24" s="2">
-        <v>1</v>
-      </c>
-      <c r="I24" s="2">
-        <v>0</v>
-      </c>
-      <c r="J24" s="2">
-        <v>3</v>
-      </c>
-      <c r="K24" s="2">
-        <v>1</v>
-      </c>
-      <c r="L24" s="2">
-        <v>1</v>
-      </c>
-      <c r="M24" s="2">
-        <v>2</v>
-      </c>
-      <c r="N24" s="2">
-        <v>1</v>
-      </c>
-      <c r="O24" s="2">
-        <v>2</v>
-      </c>
-      <c r="P24" s="2">
-        <v>1</v>
-      </c>
-      <c r="Q24" s="2">
-        <v>1</v>
-      </c>
-      <c r="R24" s="2">
-        <v>2</v>
-      </c>
-      <c r="S24" s="2">
-        <v>1</v>
-      </c>
-      <c r="T24" s="2">
-        <v>2</v>
-      </c>
-      <c r="U24" s="2">
-        <v>1</v>
-      </c>
-      <c r="V24" s="2">
-        <v>1</v>
-      </c>
-      <c r="W24" s="2">
-        <v>1</v>
-      </c>
-      <c r="X24" s="2">
-        <v>2</v>
-      </c>
-      <c r="Y24" s="2">
-        <v>1</v>
-      </c>
-      <c r="Z24" s="2">
-        <v>2</v>
-      </c>
-      <c r="AA24" s="2">
-        <v>1</v>
-      </c>
+        <v/>
+      </c>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="2"/>
+      <c r="M24" s="2"/>
+      <c r="N24" s="2"/>
+      <c r="O24" s="2"/>
+      <c r="P24" s="2"/>
+      <c r="Q24" s="2"/>
+      <c r="R24" s="2"/>
+      <c r="S24" s="2"/>
+      <c r="T24" s="2"/>
+      <c r="U24" s="2"/>
+      <c r="V24" s="2"/>
+      <c r="W24" s="2"/>
+      <c r="X24" s="2"/>
+      <c r="Y24" s="2"/>
+      <c r="Z24" s="2"/>
+      <c r="AA24" s="2"/>
       <c r="AB24" s="2"/>
       <c r="AC24" s="2"/>
       <c r="AD24" s="2"/>
@@ -4290,86 +3947,38 @@
       <c r="A25" s="15">
         <v>20</v>
       </c>
-      <c r="B25" s="45" t="str">
+      <c r="B25" s="14" t="str">
         <f>Fixture!C24&amp;" vs "&amp;Fixture!F24</f>
         <v>Australia vs Turquía</v>
       </c>
       <c r="C25" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D24),Fixture!D24&amp;"-"&amp;Fixture!E24,"")</f>
-        <v>2-0</v>
-      </c>
-      <c r="D25" s="6">
-        <v>1</v>
-      </c>
-      <c r="E25" s="6">
-        <v>2</v>
-      </c>
-      <c r="F25" s="6">
-        <v>1</v>
-      </c>
-      <c r="G25" s="6">
-        <v>1</v>
-      </c>
-      <c r="H25" s="6">
-        <v>1</v>
-      </c>
-      <c r="I25" s="6">
-        <v>1</v>
-      </c>
-      <c r="J25" s="6">
-        <v>0</v>
-      </c>
-      <c r="K25" s="6">
-        <v>2</v>
-      </c>
-      <c r="L25" s="6">
-        <v>1</v>
-      </c>
-      <c r="M25" s="6">
-        <v>1</v>
-      </c>
-      <c r="N25" s="6">
-        <v>1</v>
-      </c>
-      <c r="O25" s="6">
-        <v>3</v>
-      </c>
-      <c r="P25" s="6">
-        <v>1</v>
-      </c>
-      <c r="Q25" s="6">
-        <v>2</v>
-      </c>
-      <c r="R25" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="S25" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="T25" s="6">
-        <v>1</v>
-      </c>
-      <c r="U25" s="6">
-        <v>2</v>
-      </c>
-      <c r="V25" s="6">
-        <v>1</v>
-      </c>
-      <c r="W25" s="6">
-        <v>2</v>
-      </c>
-      <c r="X25" s="6">
-        <v>1</v>
-      </c>
-      <c r="Y25" s="6">
-        <v>1</v>
-      </c>
-      <c r="Z25" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="AA25" s="6" t="s">
-        <v>112</v>
-      </c>
+        <v/>
+      </c>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="6"/>
+      <c r="K25" s="6"/>
+      <c r="L25" s="6"/>
+      <c r="M25" s="6"/>
+      <c r="N25" s="6"/>
+      <c r="O25" s="6"/>
+      <c r="P25" s="6"/>
+      <c r="Q25" s="6"/>
+      <c r="R25" s="6"/>
+      <c r="S25" s="6"/>
+      <c r="T25" s="6"/>
+      <c r="U25" s="6"/>
+      <c r="V25" s="6"/>
+      <c r="W25" s="6"/>
+      <c r="X25" s="6"/>
+      <c r="Y25" s="6"/>
+      <c r="Z25" s="6"/>
+      <c r="AA25" s="6"/>
       <c r="AB25" s="6"/>
       <c r="AC25" s="6"/>
       <c r="AD25" s="6"/>
@@ -4553,86 +4162,38 @@
       <c r="A30" s="12">
         <v>25</v>
       </c>
-      <c r="B30" s="44" t="str">
+      <c r="B30" s="11" t="str">
         <f>Fixture!C29&amp;" vs "&amp;Fixture!F29</f>
         <v>Alemania vs Curazao</v>
       </c>
       <c r="C30" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D29),Fixture!D29&amp;"-"&amp;Fixture!E29,"")</f>
-        <v>7-1</v>
-      </c>
-      <c r="D30" s="2">
-        <v>5</v>
-      </c>
-      <c r="E30" s="2">
-        <v>0</v>
-      </c>
-      <c r="F30" s="2">
-        <v>3</v>
-      </c>
-      <c r="G30" s="2">
-        <v>0</v>
-      </c>
-      <c r="H30" s="2">
-        <v>7</v>
-      </c>
-      <c r="I30" s="2">
-        <v>0</v>
-      </c>
-      <c r="J30" s="2">
-        <v>6</v>
-      </c>
-      <c r="K30" s="2">
-        <v>0</v>
-      </c>
-      <c r="L30" s="2">
-        <v>4</v>
-      </c>
-      <c r="M30" s="2">
-        <v>0</v>
-      </c>
-      <c r="N30" s="2">
-        <v>6</v>
-      </c>
-      <c r="O30" s="2">
-        <v>0</v>
-      </c>
-      <c r="P30" s="2">
-        <v>2</v>
-      </c>
-      <c r="Q30" s="2">
-        <v>0</v>
-      </c>
-      <c r="R30" s="2">
-        <v>3</v>
-      </c>
-      <c r="S30" s="2">
-        <v>0</v>
-      </c>
-      <c r="T30" s="2">
-        <v>3</v>
-      </c>
-      <c r="U30" s="2">
-        <v>0</v>
-      </c>
-      <c r="V30" s="2">
-        <v>4</v>
-      </c>
-      <c r="W30" s="2">
-        <v>0</v>
-      </c>
-      <c r="X30" s="2">
-        <v>4</v>
-      </c>
-      <c r="Y30" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z30" s="2">
-        <v>2</v>
-      </c>
-      <c r="AA30" s="2">
-        <v>1</v>
-      </c>
+        <v/>
+      </c>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+      <c r="J30" s="2"/>
+      <c r="K30" s="2"/>
+      <c r="L30" s="2"/>
+      <c r="M30" s="2"/>
+      <c r="N30" s="2"/>
+      <c r="O30" s="2"/>
+      <c r="P30" s="2"/>
+      <c r="Q30" s="2"/>
+      <c r="R30" s="2"/>
+      <c r="S30" s="2"/>
+      <c r="T30" s="2"/>
+      <c r="U30" s="2"/>
+      <c r="V30" s="2"/>
+      <c r="W30" s="2"/>
+      <c r="X30" s="2"/>
+      <c r="Y30" s="2"/>
+      <c r="Z30" s="2"/>
+      <c r="AA30" s="2"/>
       <c r="AB30" s="2"/>
       <c r="AC30" s="2"/>
       <c r="AD30" s="2"/>
@@ -4644,86 +4205,38 @@
       <c r="A31" s="15">
         <v>26</v>
       </c>
-      <c r="B31" s="45" t="str">
+      <c r="B31" s="14" t="str">
         <f>Fixture!C30&amp;" vs "&amp;Fixture!F30</f>
         <v>Costa de Marfil vs Ecuador</v>
       </c>
       <c r="C31" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D30),Fixture!D30&amp;"-"&amp;Fixture!E30,"")</f>
-        <v>1-0</v>
-      </c>
-      <c r="D31" s="6">
-        <v>1</v>
-      </c>
-      <c r="E31" s="6">
-        <v>1</v>
-      </c>
-      <c r="F31" s="6">
-        <v>1</v>
-      </c>
-      <c r="G31" s="6">
-        <v>3</v>
-      </c>
-      <c r="H31" s="6">
-        <v>2</v>
-      </c>
-      <c r="I31" s="6">
-        <v>2</v>
-      </c>
-      <c r="J31" s="6">
-        <v>0</v>
-      </c>
-      <c r="K31" s="6">
-        <v>2</v>
-      </c>
-      <c r="L31" s="6">
-        <v>2</v>
-      </c>
-      <c r="M31" s="6">
-        <v>1</v>
-      </c>
-      <c r="N31" s="6">
-        <v>0</v>
-      </c>
-      <c r="O31" s="6">
-        <v>1</v>
-      </c>
-      <c r="P31" s="6">
-        <v>1</v>
-      </c>
-      <c r="Q31" s="6">
-        <v>1</v>
-      </c>
-      <c r="R31" s="6">
-        <v>1</v>
-      </c>
-      <c r="S31" s="6">
-        <v>1</v>
-      </c>
-      <c r="T31" s="6">
-        <v>0</v>
-      </c>
-      <c r="U31" s="6">
-        <v>1</v>
-      </c>
-      <c r="V31" s="6">
-        <v>1</v>
-      </c>
-      <c r="W31" s="6">
-        <v>1</v>
-      </c>
-      <c r="X31" s="6">
-        <v>2</v>
-      </c>
-      <c r="Y31" s="6">
-        <v>1</v>
-      </c>
-      <c r="Z31" s="6">
-        <v>3</v>
-      </c>
-      <c r="AA31" s="6">
-        <v>0</v>
-      </c>
+        <v/>
+      </c>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="6"/>
+      <c r="K31" s="6"/>
+      <c r="L31" s="6"/>
+      <c r="M31" s="6"/>
+      <c r="N31" s="6"/>
+      <c r="O31" s="6"/>
+      <c r="P31" s="6"/>
+      <c r="Q31" s="6"/>
+      <c r="R31" s="6"/>
+      <c r="S31" s="6"/>
+      <c r="T31" s="6"/>
+      <c r="U31" s="6"/>
+      <c r="V31" s="6"/>
+      <c r="W31" s="6"/>
+      <c r="X31" s="6"/>
+      <c r="Y31" s="6"/>
+      <c r="Z31" s="6"/>
+      <c r="AA31" s="6"/>
       <c r="AB31" s="6"/>
       <c r="AC31" s="6"/>
       <c r="AD31" s="6"/>
@@ -4907,86 +4420,38 @@
       <c r="A36" s="12">
         <v>31</v>
       </c>
-      <c r="B36" s="44" t="str">
+      <c r="B36" s="11" t="str">
         <f>Fixture!C35&amp;" vs "&amp;Fixture!F35</f>
         <v>Países Bajos vs Japón</v>
       </c>
       <c r="C36" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D35),Fixture!D35&amp;"-"&amp;Fixture!E35,"")</f>
-        <v>2-2</v>
-      </c>
-      <c r="D36" s="2">
-        <v>2</v>
-      </c>
-      <c r="E36" s="2">
-        <v>2</v>
-      </c>
-      <c r="F36" s="2">
-        <v>2</v>
-      </c>
-      <c r="G36" s="2">
-        <v>2</v>
-      </c>
-      <c r="H36" s="2">
-        <v>1</v>
-      </c>
-      <c r="I36" s="2">
-        <v>1</v>
-      </c>
-      <c r="J36" s="2">
-        <v>3</v>
-      </c>
-      <c r="K36" s="2">
-        <v>2</v>
-      </c>
-      <c r="L36" s="2">
-        <v>1</v>
-      </c>
-      <c r="M36" s="2">
-        <v>1</v>
-      </c>
-      <c r="N36" s="2">
-        <v>2</v>
-      </c>
-      <c r="O36" s="2">
-        <v>1</v>
-      </c>
-      <c r="P36" s="2">
-        <v>1</v>
-      </c>
-      <c r="Q36" s="2">
-        <v>2</v>
-      </c>
-      <c r="R36" s="2">
-        <v>2</v>
-      </c>
-      <c r="S36" s="2">
-        <v>1</v>
-      </c>
-      <c r="T36" s="2">
-        <v>2</v>
-      </c>
-      <c r="U36" s="2">
-        <v>1</v>
-      </c>
-      <c r="V36" s="2">
-        <v>2</v>
-      </c>
-      <c r="W36" s="2">
-        <v>2</v>
-      </c>
-      <c r="X36" s="2">
-        <v>1</v>
-      </c>
-      <c r="Y36" s="2">
-        <v>1</v>
-      </c>
-      <c r="Z36" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA36" s="2">
-        <v>2</v>
-      </c>
+        <v/>
+      </c>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="2"/>
+      <c r="K36" s="2"/>
+      <c r="L36" s="2"/>
+      <c r="M36" s="2"/>
+      <c r="N36" s="2"/>
+      <c r="O36" s="2"/>
+      <c r="P36" s="2"/>
+      <c r="Q36" s="2"/>
+      <c r="R36" s="2"/>
+      <c r="S36" s="2"/>
+      <c r="T36" s="2"/>
+      <c r="U36" s="2"/>
+      <c r="V36" s="2"/>
+      <c r="W36" s="2"/>
+      <c r="X36" s="2"/>
+      <c r="Y36" s="2"/>
+      <c r="Z36" s="2"/>
+      <c r="AA36" s="2"/>
       <c r="AB36" s="2"/>
       <c r="AC36" s="2"/>
       <c r="AD36" s="2"/>
@@ -4998,86 +4463,38 @@
       <c r="A37" s="15">
         <v>32</v>
       </c>
-      <c r="B37" s="45" t="str">
+      <c r="B37" s="14" t="str">
         <f>Fixture!C36&amp;" vs "&amp;Fixture!F36</f>
         <v>Suecia vs Túnez</v>
       </c>
       <c r="C37" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D36),Fixture!D36&amp;"-"&amp;Fixture!E36,"")</f>
-        <v>5-1</v>
-      </c>
-      <c r="D37" s="6">
-        <v>2</v>
-      </c>
-      <c r="E37" s="6">
-        <v>0</v>
-      </c>
-      <c r="F37" s="6">
-        <v>2</v>
-      </c>
-      <c r="G37" s="6">
-        <v>1</v>
-      </c>
-      <c r="H37" s="6">
-        <v>1</v>
-      </c>
-      <c r="I37" s="6">
-        <v>1</v>
-      </c>
-      <c r="J37" s="6">
-        <v>1</v>
-      </c>
-      <c r="K37" s="6">
-        <v>0</v>
-      </c>
-      <c r="L37" s="6">
-        <v>1</v>
-      </c>
-      <c r="M37" s="6">
-        <v>0</v>
-      </c>
-      <c r="N37" s="6">
-        <v>2</v>
-      </c>
-      <c r="O37" s="6">
-        <v>0</v>
-      </c>
-      <c r="P37" s="6">
-        <v>2</v>
-      </c>
-      <c r="Q37" s="6">
-        <v>1</v>
-      </c>
-      <c r="R37" s="6">
-        <v>1</v>
-      </c>
-      <c r="S37" s="6">
-        <v>0</v>
-      </c>
-      <c r="T37" s="6">
-        <v>1</v>
-      </c>
-      <c r="U37" s="6">
-        <v>0</v>
-      </c>
-      <c r="V37" s="6">
-        <v>2</v>
-      </c>
-      <c r="W37" s="6">
-        <v>0</v>
-      </c>
-      <c r="X37" s="6">
-        <v>2</v>
-      </c>
-      <c r="Y37" s="6">
-        <v>0</v>
-      </c>
-      <c r="Z37" s="6">
-        <v>2</v>
-      </c>
-      <c r="AA37" s="6">
-        <v>0</v>
-      </c>
+        <v/>
+      </c>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+      <c r="I37" s="6"/>
+      <c r="J37" s="6"/>
+      <c r="K37" s="6"/>
+      <c r="L37" s="6"/>
+      <c r="M37" s="6"/>
+      <c r="N37" s="6"/>
+      <c r="O37" s="6"/>
+      <c r="P37" s="6"/>
+      <c r="Q37" s="6"/>
+      <c r="R37" s="6"/>
+      <c r="S37" s="6"/>
+      <c r="T37" s="6"/>
+      <c r="U37" s="6"/>
+      <c r="V37" s="6"/>
+      <c r="W37" s="6"/>
+      <c r="X37" s="6"/>
+      <c r="Y37" s="6"/>
+      <c r="Z37" s="6"/>
+      <c r="AA37" s="6"/>
       <c r="AB37" s="6"/>
       <c r="AC37" s="6"/>
       <c r="AD37" s="6"/>
@@ -5261,86 +4678,38 @@
       <c r="A42" s="12">
         <v>37</v>
       </c>
-      <c r="B42" s="44" t="str">
+      <c r="B42" s="11" t="str">
         <f>Fixture!C41&amp;" vs "&amp;Fixture!F41</f>
         <v>Bélgica vs Egipto</v>
       </c>
       <c r="C42" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D41),Fixture!D41&amp;"-"&amp;Fixture!E41,"")</f>
-        <v>1-1</v>
-      </c>
-      <c r="D42" s="2">
-        <v>2</v>
-      </c>
-      <c r="E42" s="2">
-        <v>1</v>
-      </c>
-      <c r="F42" s="2">
-        <v>2</v>
-      </c>
-      <c r="G42" s="2">
-        <v>1</v>
-      </c>
-      <c r="H42" s="2">
-        <v>2</v>
-      </c>
-      <c r="I42" s="2">
-        <v>2</v>
-      </c>
-      <c r="J42" s="2">
-        <v>1</v>
-      </c>
-      <c r="K42" s="2">
-        <v>1</v>
-      </c>
-      <c r="L42" s="2">
-        <v>2</v>
-      </c>
-      <c r="M42" s="2">
-        <v>0</v>
-      </c>
-      <c r="N42" s="2">
-        <v>1</v>
-      </c>
-      <c r="O42" s="2">
-        <v>1</v>
-      </c>
-      <c r="P42" s="2">
-        <v>2</v>
-      </c>
-      <c r="Q42" s="2">
-        <v>2</v>
-      </c>
-      <c r="R42" s="2">
-        <v>2</v>
-      </c>
-      <c r="S42" s="2">
-        <v>2</v>
-      </c>
-      <c r="T42" s="2">
-        <v>2</v>
-      </c>
-      <c r="U42" s="2">
-        <v>1</v>
-      </c>
-      <c r="V42" s="2">
-        <v>2</v>
-      </c>
-      <c r="W42" s="2">
-        <v>1</v>
-      </c>
-      <c r="X42" s="2">
-        <v>2</v>
-      </c>
-      <c r="Y42" s="2">
-        <v>1</v>
-      </c>
-      <c r="Z42" s="2">
-        <v>2</v>
-      </c>
-      <c r="AA42" s="2">
-        <v>0</v>
-      </c>
+        <v/>
+      </c>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
+      <c r="I42" s="2"/>
+      <c r="J42" s="2"/>
+      <c r="K42" s="2"/>
+      <c r="L42" s="2"/>
+      <c r="M42" s="2"/>
+      <c r="N42" s="2"/>
+      <c r="O42" s="2"/>
+      <c r="P42" s="2"/>
+      <c r="Q42" s="2"/>
+      <c r="R42" s="2"/>
+      <c r="S42" s="2"/>
+      <c r="T42" s="2"/>
+      <c r="U42" s="2"/>
+      <c r="V42" s="2"/>
+      <c r="W42" s="2"/>
+      <c r="X42" s="2"/>
+      <c r="Y42" s="2"/>
+      <c r="Z42" s="2"/>
+      <c r="AA42" s="2"/>
       <c r="AB42" s="2"/>
       <c r="AC42" s="2"/>
       <c r="AD42" s="2"/>
@@ -5352,86 +4721,38 @@
       <c r="A43" s="15">
         <v>38</v>
       </c>
-      <c r="B43" s="45" t="str">
+      <c r="B43" s="14" t="str">
         <f>Fixture!C42&amp;" vs "&amp;Fixture!F42</f>
         <v>Irán vs Nueva Zelanda</v>
       </c>
       <c r="C43" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D42),Fixture!D42&amp;"-"&amp;Fixture!E42,"")</f>
-        <v>2-2</v>
-      </c>
-      <c r="D43" s="6">
-        <v>1</v>
-      </c>
-      <c r="E43" s="6">
-        <v>1</v>
-      </c>
-      <c r="F43" s="6">
-        <v>3</v>
-      </c>
-      <c r="G43" s="6">
-        <v>0</v>
-      </c>
-      <c r="H43" s="6">
-        <v>2</v>
-      </c>
-      <c r="I43" s="6">
-        <v>0</v>
-      </c>
-      <c r="J43" s="6">
-        <v>2</v>
-      </c>
-      <c r="K43" s="6">
-        <v>1</v>
-      </c>
-      <c r="L43" s="6">
-        <v>0</v>
-      </c>
-      <c r="M43" s="6">
-        <v>2</v>
-      </c>
-      <c r="N43" s="6">
-        <v>3</v>
-      </c>
-      <c r="O43" s="6">
-        <v>1</v>
-      </c>
-      <c r="P43" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q43" s="6">
-        <v>2</v>
-      </c>
-      <c r="R43" s="6">
-        <v>0</v>
-      </c>
-      <c r="S43" s="6">
-        <v>2</v>
-      </c>
-      <c r="T43" s="6">
-        <v>1</v>
-      </c>
-      <c r="U43" s="6">
-        <v>0</v>
-      </c>
-      <c r="V43" s="6">
-        <v>2</v>
-      </c>
-      <c r="W43" s="6">
-        <v>0</v>
-      </c>
-      <c r="X43" s="6">
-        <v>2</v>
-      </c>
-      <c r="Y43" s="6">
-        <v>0</v>
-      </c>
-      <c r="Z43" s="6">
-        <v>1</v>
-      </c>
-      <c r="AA43" s="6">
-        <v>0</v>
-      </c>
+        <v/>
+      </c>
+      <c r="D43" s="6"/>
+      <c r="E43" s="6"/>
+      <c r="F43" s="6"/>
+      <c r="G43" s="6"/>
+      <c r="H43" s="6"/>
+      <c r="I43" s="6"/>
+      <c r="J43" s="6"/>
+      <c r="K43" s="6"/>
+      <c r="L43" s="6"/>
+      <c r="M43" s="6"/>
+      <c r="N43" s="6"/>
+      <c r="O43" s="6"/>
+      <c r="P43" s="6"/>
+      <c r="Q43" s="6"/>
+      <c r="R43" s="6"/>
+      <c r="S43" s="6"/>
+      <c r="T43" s="6"/>
+      <c r="U43" s="6"/>
+      <c r="V43" s="6"/>
+      <c r="W43" s="6"/>
+      <c r="X43" s="6"/>
+      <c r="Y43" s="6"/>
+      <c r="Z43" s="6"/>
+      <c r="AA43" s="6"/>
       <c r="AB43" s="6"/>
       <c r="AC43" s="6"/>
       <c r="AD43" s="6"/>
@@ -5615,86 +4936,38 @@
       <c r="A48" s="12">
         <v>43</v>
       </c>
-      <c r="B48" s="44" t="str">
+      <c r="B48" s="11" t="str">
         <f>Fixture!C47&amp;" vs "&amp;Fixture!F47</f>
         <v>España vs Cabo Verde</v>
       </c>
       <c r="C48" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D47),Fixture!D47&amp;"-"&amp;Fixture!E47,"")</f>
-        <v>0-0</v>
-      </c>
-      <c r="D48" s="2">
-        <v>4</v>
-      </c>
-      <c r="E48" s="2">
-        <v>1</v>
-      </c>
-      <c r="F48" s="2">
-        <v>4</v>
-      </c>
-      <c r="G48" s="2">
-        <v>1</v>
-      </c>
-      <c r="H48" s="2">
-        <v>3</v>
-      </c>
-      <c r="I48" s="2">
-        <v>1</v>
-      </c>
-      <c r="J48" s="2">
-        <v>3</v>
-      </c>
-      <c r="K48" s="2">
-        <v>1</v>
-      </c>
-      <c r="L48" s="2">
-        <v>4</v>
-      </c>
-      <c r="M48" s="2">
-        <v>1</v>
-      </c>
-      <c r="N48" s="2">
-        <v>4</v>
-      </c>
-      <c r="O48" s="2">
-        <v>1</v>
-      </c>
-      <c r="P48" s="2">
-        <v>4</v>
-      </c>
-      <c r="Q48" s="2">
-        <v>0</v>
-      </c>
-      <c r="R48" s="2">
-        <v>5</v>
-      </c>
-      <c r="S48" s="2">
-        <v>1</v>
-      </c>
-      <c r="T48" s="2">
-        <v>3</v>
-      </c>
-      <c r="U48" s="2">
-        <v>0</v>
-      </c>
-      <c r="V48" s="2">
-        <v>3</v>
-      </c>
-      <c r="W48" s="2">
-        <v>0</v>
-      </c>
-      <c r="X48" s="2">
-        <v>3</v>
-      </c>
-      <c r="Y48" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z48" s="2">
-        <v>4</v>
-      </c>
-      <c r="AA48" s="2">
-        <v>0</v>
-      </c>
+        <v/>
+      </c>
+      <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="2"/>
+      <c r="G48" s="2"/>
+      <c r="H48" s="2"/>
+      <c r="I48" s="2"/>
+      <c r="J48" s="2"/>
+      <c r="K48" s="2"/>
+      <c r="L48" s="2"/>
+      <c r="M48" s="2"/>
+      <c r="N48" s="2"/>
+      <c r="O48" s="2"/>
+      <c r="P48" s="2"/>
+      <c r="Q48" s="2"/>
+      <c r="R48" s="2"/>
+      <c r="S48" s="2"/>
+      <c r="T48" s="2"/>
+      <c r="U48" s="2"/>
+      <c r="V48" s="2"/>
+      <c r="W48" s="2"/>
+      <c r="X48" s="2"/>
+      <c r="Y48" s="2"/>
+      <c r="Z48" s="2"/>
+      <c r="AA48" s="2"/>
       <c r="AB48" s="2"/>
       <c r="AC48" s="2"/>
       <c r="AD48" s="2"/>
@@ -5706,86 +4979,38 @@
       <c r="A49" s="15">
         <v>44</v>
       </c>
-      <c r="B49" s="45" t="str">
+      <c r="B49" s="14" t="str">
         <f>Fixture!C48&amp;" vs "&amp;Fixture!F48</f>
         <v>Arabia Saudita vs Uruguay</v>
       </c>
       <c r="C49" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D48),Fixture!D48&amp;"-"&amp;Fixture!E48,"")</f>
-        <v>1-1</v>
-      </c>
-      <c r="D49" s="6">
-        <v>1</v>
-      </c>
-      <c r="E49" s="6">
-        <v>3</v>
-      </c>
-      <c r="F49" s="6">
-        <v>1</v>
-      </c>
-      <c r="G49" s="6">
-        <v>3</v>
-      </c>
-      <c r="H49" s="6">
-        <v>2</v>
-      </c>
-      <c r="I49" s="6">
-        <v>3</v>
-      </c>
-      <c r="J49" s="6">
-        <v>0</v>
-      </c>
-      <c r="K49" s="6">
-        <v>2</v>
-      </c>
-      <c r="L49" s="6">
-        <v>1</v>
-      </c>
-      <c r="M49" s="6">
-        <v>3</v>
-      </c>
-      <c r="N49" s="6">
-        <v>1</v>
-      </c>
-      <c r="O49" s="6">
-        <v>2</v>
-      </c>
-      <c r="P49" s="6">
-        <v>1</v>
-      </c>
-      <c r="Q49" s="6">
-        <v>2</v>
-      </c>
-      <c r="R49" s="6">
-        <v>1</v>
-      </c>
-      <c r="S49" s="6">
-        <v>2</v>
-      </c>
-      <c r="T49" s="6">
-        <v>1</v>
-      </c>
-      <c r="U49" s="6">
-        <v>2</v>
-      </c>
-      <c r="V49" s="6">
-        <v>0</v>
-      </c>
-      <c r="W49" s="6">
-        <v>2</v>
-      </c>
-      <c r="X49" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y49" s="6">
-        <v>2</v>
-      </c>
-      <c r="Z49" s="6">
-        <v>1</v>
-      </c>
-      <c r="AA49" s="6">
-        <v>2</v>
-      </c>
+        <v/>
+      </c>
+      <c r="D49" s="6"/>
+      <c r="E49" s="6"/>
+      <c r="F49" s="6"/>
+      <c r="G49" s="6"/>
+      <c r="H49" s="6"/>
+      <c r="I49" s="6"/>
+      <c r="J49" s="6"/>
+      <c r="K49" s="6"/>
+      <c r="L49" s="6"/>
+      <c r="M49" s="6"/>
+      <c r="N49" s="6"/>
+      <c r="O49" s="6"/>
+      <c r="P49" s="6"/>
+      <c r="Q49" s="6"/>
+      <c r="R49" s="6"/>
+      <c r="S49" s="6"/>
+      <c r="T49" s="6"/>
+      <c r="U49" s="6"/>
+      <c r="V49" s="6"/>
+      <c r="W49" s="6"/>
+      <c r="X49" s="6"/>
+      <c r="Y49" s="6"/>
+      <c r="Z49" s="6"/>
+      <c r="AA49" s="6"/>
       <c r="AB49" s="6"/>
       <c r="AC49" s="6"/>
       <c r="AD49" s="6"/>
@@ -5969,86 +5194,38 @@
       <c r="A54" s="12">
         <v>49</v>
       </c>
-      <c r="B54" s="44" t="str">
+      <c r="B54" s="11" t="str">
         <f>Fixture!C53&amp;" vs "&amp;Fixture!F53</f>
         <v>Francia vs Senegal</v>
       </c>
       <c r="C54" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D53),Fixture!D53&amp;"-"&amp;Fixture!E53,"")</f>
-        <v>3-1</v>
-      </c>
-      <c r="D54" s="2">
-        <v>2</v>
-      </c>
-      <c r="E54" s="2">
-        <v>0</v>
-      </c>
-      <c r="F54" s="2">
-        <v>3</v>
-      </c>
-      <c r="G54" s="2">
-        <v>1</v>
-      </c>
-      <c r="H54" s="2">
-        <v>3</v>
-      </c>
-      <c r="I54" s="2">
-        <v>0</v>
-      </c>
-      <c r="J54" s="2">
-        <v>1</v>
-      </c>
-      <c r="K54" s="2">
-        <v>1</v>
-      </c>
-      <c r="L54" s="2">
-        <v>3</v>
-      </c>
-      <c r="M54" s="2">
-        <v>1</v>
-      </c>
-      <c r="N54" s="2">
-        <v>3</v>
-      </c>
-      <c r="O54" s="2">
-        <v>1</v>
-      </c>
-      <c r="P54" s="2">
-        <v>3</v>
-      </c>
-      <c r="Q54" s="2">
-        <v>1</v>
-      </c>
-      <c r="R54" s="2">
-        <v>2</v>
-      </c>
-      <c r="S54" s="2">
-        <v>1</v>
-      </c>
-      <c r="T54" s="2">
-        <v>2</v>
-      </c>
-      <c r="U54" s="2">
-        <v>1</v>
-      </c>
-      <c r="V54" s="2">
-        <v>2</v>
-      </c>
-      <c r="W54" s="2">
-        <v>1</v>
-      </c>
-      <c r="X54" s="2">
-        <v>2</v>
-      </c>
-      <c r="Y54" s="2">
-        <v>1</v>
-      </c>
-      <c r="Z54" s="2">
-        <v>3</v>
-      </c>
-      <c r="AA54" s="2">
-        <v>1</v>
-      </c>
+        <v/>
+      </c>
+      <c r="D54" s="2"/>
+      <c r="E54" s="2"/>
+      <c r="F54" s="2"/>
+      <c r="G54" s="2"/>
+      <c r="H54" s="2"/>
+      <c r="I54" s="2"/>
+      <c r="J54" s="2"/>
+      <c r="K54" s="2"/>
+      <c r="L54" s="2"/>
+      <c r="M54" s="2"/>
+      <c r="N54" s="2"/>
+      <c r="O54" s="2"/>
+      <c r="P54" s="2"/>
+      <c r="Q54" s="2"/>
+      <c r="R54" s="2"/>
+      <c r="S54" s="2"/>
+      <c r="T54" s="2"/>
+      <c r="U54" s="2"/>
+      <c r="V54" s="2"/>
+      <c r="W54" s="2"/>
+      <c r="X54" s="2"/>
+      <c r="Y54" s="2"/>
+      <c r="Z54" s="2"/>
+      <c r="AA54" s="2"/>
       <c r="AB54" s="2"/>
       <c r="AC54" s="2"/>
       <c r="AD54" s="2"/>
@@ -6060,86 +5237,38 @@
       <c r="A55" s="15">
         <v>50</v>
       </c>
-      <c r="B55" s="45" t="str">
+      <c r="B55" s="14" t="str">
         <f>Fixture!C54&amp;" vs "&amp;Fixture!F54</f>
         <v>Irak vs Noruega</v>
       </c>
       <c r="C55" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D54),Fixture!D54&amp;"-"&amp;Fixture!E54,"")</f>
-        <v>1-4</v>
-      </c>
-      <c r="D55" s="6">
-        <v>1</v>
-      </c>
-      <c r="E55" s="6">
-        <v>6</v>
-      </c>
-      <c r="F55" s="6">
-        <v>1</v>
-      </c>
-      <c r="G55" s="6">
-        <v>2</v>
-      </c>
-      <c r="H55" s="6">
-        <v>0</v>
-      </c>
-      <c r="I55" s="6">
-        <v>5</v>
-      </c>
-      <c r="J55" s="6">
-        <v>2</v>
-      </c>
-      <c r="K55" s="6">
-        <v>1</v>
-      </c>
-      <c r="L55" s="6">
-        <v>0</v>
-      </c>
-      <c r="M55" s="6">
-        <v>2</v>
-      </c>
-      <c r="N55" s="6">
-        <v>0</v>
-      </c>
-      <c r="O55" s="6">
-        <v>4</v>
-      </c>
-      <c r="P55" s="6">
-        <v>1</v>
-      </c>
-      <c r="Q55" s="6">
-        <v>3</v>
-      </c>
-      <c r="R55" s="6">
-        <v>1</v>
-      </c>
-      <c r="S55" s="6">
-        <v>2</v>
-      </c>
-      <c r="T55" s="6">
-        <v>0</v>
-      </c>
-      <c r="U55" s="6">
-        <v>1</v>
-      </c>
-      <c r="V55" s="6">
-        <v>0</v>
-      </c>
-      <c r="W55" s="6">
-        <v>2</v>
-      </c>
-      <c r="X55" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y55" s="6">
-        <v>2</v>
-      </c>
-      <c r="Z55" s="6">
-        <v>0</v>
-      </c>
-      <c r="AA55" s="6">
-        <v>2</v>
-      </c>
+        <v/>
+      </c>
+      <c r="D55" s="6"/>
+      <c r="E55" s="6"/>
+      <c r="F55" s="6"/>
+      <c r="G55" s="6"/>
+      <c r="H55" s="6"/>
+      <c r="I55" s="6"/>
+      <c r="J55" s="6"/>
+      <c r="K55" s="6"/>
+      <c r="L55" s="6"/>
+      <c r="M55" s="6"/>
+      <c r="N55" s="6"/>
+      <c r="O55" s="6"/>
+      <c r="P55" s="6"/>
+      <c r="Q55" s="6"/>
+      <c r="R55" s="6"/>
+      <c r="S55" s="6"/>
+      <c r="T55" s="6"/>
+      <c r="U55" s="6"/>
+      <c r="V55" s="6"/>
+      <c r="W55" s="6"/>
+      <c r="X55" s="6"/>
+      <c r="Y55" s="6"/>
+      <c r="Z55" s="6"/>
+      <c r="AA55" s="6"/>
       <c r="AB55" s="6"/>
       <c r="AC55" s="6"/>
       <c r="AD55" s="6"/>
@@ -6323,86 +5452,38 @@
       <c r="A60" s="12">
         <v>55</v>
       </c>
-      <c r="B60" s="44" t="str">
+      <c r="B60" s="11" t="str">
         <f>Fixture!C59&amp;" vs "&amp;Fixture!F59</f>
         <v>Argentina vs Argelia</v>
       </c>
       <c r="C60" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D59),Fixture!D59&amp;"-"&amp;Fixture!E59,"")</f>
-        <v>3-0</v>
-      </c>
-      <c r="D60" s="2">
-        <v>2</v>
-      </c>
-      <c r="E60" s="2">
-        <v>0</v>
-      </c>
-      <c r="F60" s="2">
-        <v>3</v>
-      </c>
-      <c r="G60" s="2">
-        <v>2</v>
-      </c>
-      <c r="H60" s="2">
-        <v>3</v>
-      </c>
-      <c r="I60" s="2">
-        <v>1</v>
-      </c>
-      <c r="J60" s="2">
-        <v>2</v>
-      </c>
-      <c r="K60" s="2">
-        <v>2</v>
-      </c>
-      <c r="L60" s="2">
-        <v>2</v>
-      </c>
-      <c r="M60" s="2">
-        <v>1</v>
-      </c>
-      <c r="N60" s="2">
-        <v>2</v>
-      </c>
-      <c r="O60" s="2">
-        <v>1</v>
-      </c>
-      <c r="P60" s="2">
-        <v>2</v>
-      </c>
-      <c r="Q60" s="2">
-        <v>1</v>
-      </c>
-      <c r="R60" s="2">
-        <v>2</v>
-      </c>
-      <c r="S60" s="2">
-        <v>0</v>
-      </c>
-      <c r="T60" s="2">
-        <v>2</v>
-      </c>
-      <c r="U60" s="2">
-        <v>0</v>
-      </c>
-      <c r="V60" s="2">
-        <v>3</v>
-      </c>
-      <c r="W60" s="2">
-        <v>1</v>
-      </c>
-      <c r="X60" s="2">
-        <v>2</v>
-      </c>
-      <c r="Y60" s="2">
-        <v>1</v>
-      </c>
-      <c r="Z60" s="2">
-        <v>2</v>
-      </c>
-      <c r="AA60" s="2">
-        <v>0</v>
-      </c>
+        <v/>
+      </c>
+      <c r="D60" s="2"/>
+      <c r="E60" s="2"/>
+      <c r="F60" s="2"/>
+      <c r="G60" s="2"/>
+      <c r="H60" s="2"/>
+      <c r="I60" s="2"/>
+      <c r="J60" s="2"/>
+      <c r="K60" s="2"/>
+      <c r="L60" s="2"/>
+      <c r="M60" s="2"/>
+      <c r="N60" s="2"/>
+      <c r="O60" s="2"/>
+      <c r="P60" s="2"/>
+      <c r="Q60" s="2"/>
+      <c r="R60" s="2"/>
+      <c r="S60" s="2"/>
+      <c r="T60" s="2"/>
+      <c r="U60" s="2"/>
+      <c r="V60" s="2"/>
+      <c r="W60" s="2"/>
+      <c r="X60" s="2"/>
+      <c r="Y60" s="2"/>
+      <c r="Z60" s="2"/>
+      <c r="AA60" s="2"/>
       <c r="AB60" s="2"/>
       <c r="AC60" s="2"/>
       <c r="AD60" s="2"/>
@@ -6422,78 +5503,30 @@
         <f>IF(ISNUMBER(Fixture!D60),Fixture!D60&amp;"-"&amp;Fixture!E60,"")</f>
         <v/>
       </c>
-      <c r="D61" s="6">
-        <v>1</v>
-      </c>
-      <c r="E61" s="6">
-        <v>0</v>
-      </c>
-      <c r="F61" s="6">
-        <v>2</v>
-      </c>
-      <c r="G61" s="6">
-        <v>1</v>
-      </c>
-      <c r="H61" s="6">
-        <v>1</v>
-      </c>
-      <c r="I61" s="6">
-        <v>0</v>
-      </c>
-      <c r="J61" s="6">
-        <v>3</v>
-      </c>
-      <c r="K61" s="6">
-        <v>0</v>
-      </c>
-      <c r="L61" s="6">
-        <v>1</v>
-      </c>
-      <c r="M61" s="6">
-        <v>1</v>
-      </c>
-      <c r="N61" s="6">
-        <v>2</v>
-      </c>
-      <c r="O61" s="6">
-        <v>0</v>
-      </c>
-      <c r="P61" s="6">
-        <v>2</v>
-      </c>
-      <c r="Q61" s="6">
-        <v>1</v>
-      </c>
-      <c r="R61" s="6">
-        <v>2</v>
-      </c>
-      <c r="S61" s="6">
-        <v>1</v>
-      </c>
-      <c r="T61" s="6">
-        <v>1</v>
-      </c>
-      <c r="U61" s="6">
-        <v>0</v>
-      </c>
-      <c r="V61" s="6">
-        <v>2</v>
-      </c>
-      <c r="W61" s="6">
-        <v>0</v>
-      </c>
-      <c r="X61" s="6">
-        <v>2</v>
-      </c>
-      <c r="Y61" s="6">
-        <v>0</v>
-      </c>
-      <c r="Z61" s="6">
-        <v>2</v>
-      </c>
-      <c r="AA61" s="6">
-        <v>1</v>
-      </c>
+      <c r="D61" s="6"/>
+      <c r="E61" s="6"/>
+      <c r="F61" s="6"/>
+      <c r="G61" s="6"/>
+      <c r="H61" s="6"/>
+      <c r="I61" s="6"/>
+      <c r="J61" s="6"/>
+      <c r="K61" s="6"/>
+      <c r="L61" s="6"/>
+      <c r="M61" s="6"/>
+      <c r="N61" s="6"/>
+      <c r="O61" s="6"/>
+      <c r="P61" s="6"/>
+      <c r="Q61" s="6"/>
+      <c r="R61" s="6"/>
+      <c r="S61" s="6"/>
+      <c r="T61" s="6"/>
+      <c r="U61" s="6"/>
+      <c r="V61" s="6"/>
+      <c r="W61" s="6"/>
+      <c r="X61" s="6"/>
+      <c r="Y61" s="6"/>
+      <c r="Z61" s="6"/>
+      <c r="AA61" s="6"/>
       <c r="AB61" s="6"/>
       <c r="AC61" s="6"/>
       <c r="AD61" s="6"/>
@@ -6685,62 +5718,30 @@
         <f>IF(ISNUMBER(Fixture!D65),Fixture!D65&amp;"-"&amp;Fixture!E65,"")</f>
         <v/>
       </c>
-      <c r="D66" s="2">
-        <v>4</v>
-      </c>
-      <c r="E66" s="2">
-        <v>1</v>
-      </c>
-      <c r="F66" s="2">
-        <v>3</v>
-      </c>
-      <c r="G66" s="2">
-        <v>0</v>
-      </c>
-      <c r="H66" s="2">
-        <v>1</v>
-      </c>
-      <c r="I66" s="2">
-        <v>0</v>
-      </c>
-      <c r="J66" s="2">
-        <v>3</v>
-      </c>
-      <c r="K66" s="2">
-        <v>0</v>
-      </c>
-      <c r="L66" s="2">
-        <v>2</v>
-      </c>
-      <c r="M66" s="2">
-        <v>1</v>
-      </c>
-      <c r="N66" s="2">
-        <v>2</v>
-      </c>
-      <c r="O66" s="2">
-        <v>1</v>
-      </c>
+      <c r="D66" s="2"/>
+      <c r="E66" s="2"/>
+      <c r="F66" s="2"/>
+      <c r="G66" s="2"/>
+      <c r="H66" s="2"/>
+      <c r="I66" s="2"/>
+      <c r="J66" s="2"/>
+      <c r="K66" s="2"/>
+      <c r="L66" s="2"/>
+      <c r="M66" s="2"/>
+      <c r="N66" s="2"/>
+      <c r="O66" s="2"/>
       <c r="P66" s="2"/>
       <c r="Q66" s="2"/>
       <c r="R66" s="2"/>
       <c r="S66" s="2"/>
       <c r="T66" s="2"/>
       <c r="U66" s="2"/>
-      <c r="V66" s="2">
-        <v>2</v>
-      </c>
-      <c r="W66" s="2">
-        <v>0</v>
-      </c>
+      <c r="V66" s="2"/>
+      <c r="W66" s="2"/>
       <c r="X66" s="2"/>
       <c r="Y66" s="2"/>
-      <c r="Z66" s="2">
-        <v>2</v>
-      </c>
-      <c r="AA66" s="2">
-        <v>0</v>
-      </c>
+      <c r="Z66" s="2"/>
+      <c r="AA66" s="2"/>
       <c r="AB66" s="2"/>
       <c r="AC66" s="2"/>
       <c r="AD66" s="2"/>
@@ -6760,58 +5761,30 @@
         <f>IF(ISNUMBER(Fixture!D66),Fixture!D66&amp;"-"&amp;Fixture!E66,"")</f>
         <v/>
       </c>
-      <c r="D67" s="6">
-        <v>0</v>
-      </c>
-      <c r="E67" s="6">
-        <v>3</v>
-      </c>
-      <c r="F67" s="6">
-        <v>1</v>
-      </c>
-      <c r="G67" s="6">
-        <v>2</v>
-      </c>
-      <c r="H67" s="6">
-        <v>1</v>
-      </c>
-      <c r="I67" s="6">
-        <v>2</v>
-      </c>
-      <c r="J67" s="6">
-        <v>0</v>
-      </c>
-      <c r="K67" s="6">
-        <v>2</v>
-      </c>
+      <c r="D67" s="6"/>
+      <c r="E67" s="6"/>
+      <c r="F67" s="6"/>
+      <c r="G67" s="6"/>
+      <c r="H67" s="6"/>
+      <c r="I67" s="6"/>
+      <c r="J67" s="6"/>
+      <c r="K67" s="6"/>
       <c r="L67" s="6"/>
       <c r="M67" s="6"/>
-      <c r="N67" s="6">
-        <v>1</v>
-      </c>
-      <c r="O67" s="6">
-        <v>2</v>
-      </c>
+      <c r="N67" s="6"/>
+      <c r="O67" s="6"/>
       <c r="P67" s="6"/>
       <c r="Q67" s="6"/>
       <c r="R67" s="6"/>
       <c r="S67" s="6"/>
       <c r="T67" s="6"/>
       <c r="U67" s="6"/>
-      <c r="V67" s="6">
-        <v>1</v>
-      </c>
-      <c r="W67" s="6">
-        <v>2</v>
-      </c>
+      <c r="V67" s="6"/>
+      <c r="W67" s="6"/>
       <c r="X67" s="6"/>
       <c r="Y67" s="6"/>
-      <c r="Z67" s="6">
-        <v>0</v>
-      </c>
-      <c r="AA67" s="6">
-        <v>2</v>
-      </c>
+      <c r="Z67" s="6"/>
+      <c r="AA67" s="6"/>
       <c r="AB67" s="6"/>
       <c r="AC67" s="6"/>
       <c r="AD67" s="6"/>
@@ -7003,62 +5976,30 @@
         <f>IF(ISNUMBER(Fixture!D71),Fixture!D71&amp;"-"&amp;Fixture!E71,"")</f>
         <v/>
       </c>
-      <c r="D72" s="2">
-        <v>2</v>
-      </c>
-      <c r="E72" s="2">
-        <v>3</v>
-      </c>
-      <c r="F72" s="2">
-        <v>2</v>
-      </c>
-      <c r="G72" s="2">
-        <v>2</v>
-      </c>
-      <c r="H72" s="2">
-        <v>3</v>
-      </c>
-      <c r="I72" s="2">
-        <v>2</v>
-      </c>
-      <c r="J72" s="2">
-        <v>1</v>
-      </c>
-      <c r="K72" s="2">
-        <v>0</v>
-      </c>
-      <c r="L72" s="2">
-        <v>1</v>
-      </c>
-      <c r="M72" s="2">
-        <v>2</v>
-      </c>
-      <c r="N72" s="2">
-        <v>2</v>
-      </c>
-      <c r="O72" s="2">
-        <v>2</v>
-      </c>
+      <c r="D72" s="2"/>
+      <c r="E72" s="2"/>
+      <c r="F72" s="2"/>
+      <c r="G72" s="2"/>
+      <c r="H72" s="2"/>
+      <c r="I72" s="2"/>
+      <c r="J72" s="2"/>
+      <c r="K72" s="2"/>
+      <c r="L72" s="2"/>
+      <c r="M72" s="2"/>
+      <c r="N72" s="2"/>
+      <c r="O72" s="2"/>
       <c r="P72" s="2"/>
       <c r="Q72" s="2"/>
       <c r="R72" s="2"/>
       <c r="S72" s="2"/>
       <c r="T72" s="2"/>
       <c r="U72" s="2"/>
-      <c r="V72" s="2">
-        <v>1</v>
-      </c>
-      <c r="W72" s="2">
-        <v>1</v>
-      </c>
+      <c r="V72" s="2"/>
+      <c r="W72" s="2"/>
       <c r="X72" s="2"/>
       <c r="Y72" s="2"/>
-      <c r="Z72" s="2">
-        <v>2</v>
-      </c>
-      <c r="AA72" s="2">
-        <v>1</v>
-      </c>
+      <c r="Z72" s="2"/>
+      <c r="AA72" s="2"/>
       <c r="AB72" s="2"/>
       <c r="AC72" s="2"/>
       <c r="AD72" s="2"/>
@@ -7078,58 +6019,30 @@
         <f>IF(ISNUMBER(Fixture!D72),Fixture!D72&amp;"-"&amp;Fixture!E72,"")</f>
         <v/>
       </c>
-      <c r="D73" s="6">
-        <v>3</v>
-      </c>
-      <c r="E73" s="6">
-        <v>1</v>
-      </c>
-      <c r="F73" s="6">
-        <v>1</v>
-      </c>
-      <c r="G73" s="6">
-        <v>1</v>
-      </c>
-      <c r="H73" s="6">
-        <v>2</v>
-      </c>
-      <c r="I73" s="6">
-        <v>1</v>
-      </c>
-      <c r="J73" s="6">
-        <v>3</v>
-      </c>
-      <c r="K73" s="6">
-        <v>1</v>
-      </c>
+      <c r="D73" s="6"/>
+      <c r="E73" s="6"/>
+      <c r="F73" s="6"/>
+      <c r="G73" s="6"/>
+      <c r="H73" s="6"/>
+      <c r="I73" s="6"/>
+      <c r="J73" s="6"/>
+      <c r="K73" s="6"/>
       <c r="L73" s="6"/>
       <c r="M73" s="6"/>
-      <c r="N73" s="6">
-        <v>3</v>
-      </c>
-      <c r="O73" s="6">
-        <v>1</v>
-      </c>
+      <c r="N73" s="6"/>
+      <c r="O73" s="6"/>
       <c r="P73" s="6"/>
       <c r="Q73" s="6"/>
       <c r="R73" s="6"/>
       <c r="S73" s="6"/>
       <c r="T73" s="6"/>
       <c r="U73" s="6"/>
-      <c r="V73" s="6">
-        <v>2</v>
-      </c>
-      <c r="W73" s="6">
-        <v>1</v>
-      </c>
+      <c r="V73" s="6"/>
+      <c r="W73" s="6"/>
       <c r="X73" s="6"/>
       <c r="Y73" s="6"/>
-      <c r="Z73" s="6">
-        <v>1</v>
-      </c>
-      <c r="AA73" s="6">
-        <v>1</v>
-      </c>
+      <c r="Z73" s="6"/>
+      <c r="AA73" s="6"/>
       <c r="AB73" s="6"/>
       <c r="AC73" s="6"/>
       <c r="AD73" s="6"/>
@@ -7311,6 +6224,7 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AD4:AE4"/>
     <mergeCell ref="AF4:AG4"/>
     <mergeCell ref="A1:AG1"/>
@@ -7327,7 +6241,6 @@
     <mergeCell ref="V4:W4"/>
     <mergeCell ref="X4:Y4"/>
     <mergeCell ref="Z4:AA4"/>
-    <mergeCell ref="AB4:AC4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Actualizar - 06-27-sáb 11:58
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\web poll\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24785528-BABD-4781-934F-17A054BA5165}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A75697AA-2B40-48FE-B862-06CACC04310F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -58,9 +58,6 @@
     <t>Posición</t>
   </si>
   <si>
-    <t>Participante 14</t>
-  </si>
-  <si>
     <t>Participante 15</t>
   </si>
   <si>
@@ -377,6 +374,9 @@
   </si>
   <si>
     <t>Cesar Lindarte</t>
+  </si>
+  <si>
+    <t>Andrea Carolina</t>
   </si>
 </sst>
 </file>
@@ -773,16 +773,16 @@
     <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1058,20 +1058,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
     </row>
     <row r="2" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
     </row>
     <row r="3" spans="1:4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1093,7 +1093,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C5" s="4">
         <v>0</v>
@@ -1108,7 +1108,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C6" s="8">
         <v>0</v>
@@ -1123,7 +1123,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C7" s="4">
         <v>0</v>
@@ -1138,7 +1138,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C8" s="8">
         <v>0</v>
@@ -1153,7 +1153,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C9" s="4">
         <v>0</v>
@@ -1168,7 +1168,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C10" s="8">
         <v>0</v>
@@ -1183,7 +1183,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C11" s="4">
         <v>0</v>
@@ -1198,7 +1198,7 @@
         <v>8</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C12" s="8">
         <v>0</v>
@@ -1213,7 +1213,7 @@
         <v>9</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C13" s="4">
         <v>0</v>
@@ -1228,7 +1228,7 @@
         <v>10</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C14" s="8">
         <v>0</v>
@@ -1243,7 +1243,7 @@
         <v>11</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C15" s="4">
         <v>0</v>
@@ -1258,7 +1258,7 @@
         <v>12</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C16" s="8">
         <v>0</v>
@@ -1273,7 +1273,7 @@
         <v>13</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C17" s="4">
         <v>0</v>
@@ -1288,7 +1288,7 @@
         <v>14</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>6</v>
+        <v>111</v>
       </c>
       <c r="C18" s="8">
         <v>0</v>
@@ -1303,7 +1303,7 @@
         <v>15</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C19" s="4">
         <v>0</v>
@@ -1338,26 +1338,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="46" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+    </row>
+    <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-    </row>
-    <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="46" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
     </row>
     <row r="3" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1365,22 +1365,22 @@
         <v>2</v>
       </c>
       <c r="B4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="D4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="E4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="F4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="G4" s="10" t="s">
         <v>14</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1388,18 +1388,18 @@
         <v>1</v>
       </c>
       <c r="B5" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="11" t="s">
         <v>16</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>17</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
       <c r="F5" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="11" t="s">
         <v>18</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1407,18 +1407,18 @@
         <v>2</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
       <c r="F6" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1426,18 +1426,18 @@
         <v>3</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D7" s="13"/>
       <c r="E7" s="13"/>
       <c r="F7" s="11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1445,18 +1445,18 @@
         <v>4</v>
       </c>
       <c r="B8" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="14" t="s">
         <v>16</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>17</v>
       </c>
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
       <c r="F8" s="14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1464,18 +1464,18 @@
         <v>5</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D9" s="13"/>
       <c r="E9" s="13"/>
       <c r="F9" s="11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1483,18 +1483,18 @@
         <v>6</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D10" s="13"/>
       <c r="E10" s="13"/>
       <c r="F10" s="14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1502,18 +1502,18 @@
         <v>7</v>
       </c>
       <c r="B11" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="11" t="s">
         <v>24</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>25</v>
       </c>
       <c r="D11" s="13"/>
       <c r="E11" s="13"/>
       <c r="F11" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11" s="11" t="s">
         <v>26</v>
-      </c>
-      <c r="G11" s="11" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1521,18 +1521,18 @@
         <v>8</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D12" s="13"/>
       <c r="E12" s="13"/>
       <c r="F12" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="G12" s="14" t="s">
         <v>29</v>
-      </c>
-      <c r="G12" s="14" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1540,18 +1540,18 @@
         <v>9</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D13" s="13"/>
       <c r="E13" s="13"/>
       <c r="F13" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1559,18 +1559,18 @@
         <v>10</v>
       </c>
       <c r="B14" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="14" t="s">
         <v>24</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>25</v>
       </c>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
       <c r="F14" s="14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1578,18 +1578,18 @@
         <v>11</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D15" s="13"/>
       <c r="E15" s="13"/>
       <c r="F15" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1597,18 +1597,18 @@
         <v>12</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D16" s="13"/>
       <c r="E16" s="13"/>
       <c r="F16" s="14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G16" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1616,18 +1616,18 @@
         <v>13</v>
       </c>
       <c r="B17" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="11" t="s">
         <v>31</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>32</v>
       </c>
       <c r="D17" s="13"/>
       <c r="E17" s="13"/>
       <c r="F17" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1635,18 +1635,18 @@
         <v>14</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D18" s="13"/>
       <c r="E18" s="13"/>
       <c r="F18" s="14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G18" s="14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1654,18 +1654,18 @@
         <v>15</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D19" s="13"/>
       <c r="E19" s="13"/>
       <c r="F19" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1673,18 +1673,18 @@
         <v>16</v>
       </c>
       <c r="B20" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" s="14" t="s">
         <v>31</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>32</v>
       </c>
       <c r="D20" s="13"/>
       <c r="E20" s="13"/>
       <c r="F20" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G20" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1692,18 +1692,18 @@
         <v>17</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D21" s="13"/>
       <c r="E21" s="13"/>
       <c r="F21" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1711,18 +1711,18 @@
         <v>18</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D22" s="13"/>
       <c r="E22" s="13"/>
       <c r="F22" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G22" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1730,18 +1730,18 @@
         <v>19</v>
       </c>
       <c r="B23" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="C23" s="11" t="s">
         <v>37</v>
-      </c>
-      <c r="C23" s="11" t="s">
-        <v>38</v>
       </c>
       <c r="D23" s="13"/>
       <c r="E23" s="13"/>
       <c r="F23" s="11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1749,18 +1749,18 @@
         <v>20</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D24" s="13"/>
       <c r="E24" s="13"/>
       <c r="F24" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G24" s="14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1768,18 +1768,18 @@
         <v>21</v>
       </c>
       <c r="B25" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="C25" s="11" t="s">
         <v>37</v>
-      </c>
-      <c r="C25" s="11" t="s">
-        <v>38</v>
       </c>
       <c r="D25" s="13"/>
       <c r="E25" s="13"/>
       <c r="F25" s="11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1787,18 +1787,18 @@
         <v>22</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D26" s="13"/>
       <c r="E26" s="13"/>
       <c r="F26" s="14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G26" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1806,18 +1806,18 @@
         <v>23</v>
       </c>
       <c r="B27" s="20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D27" s="13"/>
       <c r="E27" s="13"/>
       <c r="F27" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1825,18 +1825,18 @@
         <v>24</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D28" s="13"/>
       <c r="E28" s="13"/>
       <c r="F28" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G28" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1844,18 +1844,18 @@
         <v>25</v>
       </c>
       <c r="B29" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C29" s="11" t="s">
         <v>43</v>
-      </c>
-      <c r="C29" s="11" t="s">
-        <v>44</v>
       </c>
       <c r="D29" s="13"/>
       <c r="E29" s="13"/>
       <c r="F29" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="G29" s="11" t="s">
         <v>45</v>
-      </c>
-      <c r="G29" s="11" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1863,18 +1863,18 @@
         <v>26</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D30" s="13"/>
       <c r="E30" s="13"/>
       <c r="F30" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G30" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1882,18 +1882,18 @@
         <v>27</v>
       </c>
       <c r="B31" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C31" s="11" t="s">
         <v>43</v>
-      </c>
-      <c r="C31" s="11" t="s">
-        <v>44</v>
       </c>
       <c r="D31" s="13"/>
       <c r="E31" s="13"/>
       <c r="F31" s="11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1901,18 +1901,18 @@
         <v>28</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D32" s="13"/>
       <c r="E32" s="13"/>
       <c r="F32" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G32" s="14" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1920,18 +1920,18 @@
         <v>29</v>
       </c>
       <c r="B33" s="22" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D33" s="13"/>
       <c r="E33" s="13"/>
       <c r="F33" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1939,18 +1939,18 @@
         <v>30</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D34" s="13"/>
       <c r="E34" s="13"/>
       <c r="F34" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G34" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1958,18 +1958,18 @@
         <v>31</v>
       </c>
       <c r="B35" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="C35" s="11" t="s">
         <v>50</v>
-      </c>
-      <c r="C35" s="11" t="s">
-        <v>51</v>
       </c>
       <c r="D35" s="13"/>
       <c r="E35" s="13"/>
       <c r="F35" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1977,18 +1977,18 @@
         <v>32</v>
       </c>
       <c r="B36" s="25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D36" s="13"/>
       <c r="E36" s="13"/>
       <c r="F36" s="14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G36" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1996,18 +1996,18 @@
         <v>33</v>
       </c>
       <c r="B37" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="C37" s="11" t="s">
         <v>50</v>
-      </c>
-      <c r="C37" s="11" t="s">
-        <v>51</v>
       </c>
       <c r="D37" s="13"/>
       <c r="E37" s="13"/>
       <c r="F37" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2015,18 +2015,18 @@
         <v>34</v>
       </c>
       <c r="B38" s="25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D38" s="13"/>
       <c r="E38" s="13"/>
       <c r="F38" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G38" s="14" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2034,18 +2034,18 @@
         <v>35</v>
       </c>
       <c r="B39" s="24" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D39" s="13"/>
       <c r="E39" s="13"/>
       <c r="F39" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2053,18 +2053,18 @@
         <v>36</v>
       </c>
       <c r="B40" s="25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D40" s="13"/>
       <c r="E40" s="13"/>
       <c r="F40" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2072,18 +2072,18 @@
         <v>37</v>
       </c>
       <c r="B41" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="C41" s="11" t="s">
         <v>55</v>
-      </c>
-      <c r="C41" s="11" t="s">
-        <v>56</v>
       </c>
       <c r="D41" s="13"/>
       <c r="E41" s="13"/>
       <c r="F41" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="G41" s="11" t="s">
         <v>57</v>
-      </c>
-      <c r="G41" s="11" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2091,18 +2091,18 @@
         <v>38</v>
       </c>
       <c r="B42" s="27" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D42" s="13"/>
       <c r="E42" s="13"/>
       <c r="F42" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2110,18 +2110,18 @@
         <v>39</v>
       </c>
       <c r="B43" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="C43" s="11" t="s">
         <v>55</v>
-      </c>
-      <c r="C43" s="11" t="s">
-        <v>56</v>
       </c>
       <c r="D43" s="13"/>
       <c r="E43" s="13"/>
       <c r="F43" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G43" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2129,18 +2129,18 @@
         <v>40</v>
       </c>
       <c r="B44" s="27" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D44" s="13"/>
       <c r="E44" s="13"/>
       <c r="F44" s="14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G44" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2148,18 +2148,18 @@
         <v>41</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D45" s="13"/>
       <c r="E45" s="13"/>
       <c r="F45" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G45" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2167,18 +2167,18 @@
         <v>42</v>
       </c>
       <c r="B46" s="27" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D46" s="13"/>
       <c r="E46" s="13"/>
       <c r="F46" s="14" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G46" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2186,18 +2186,18 @@
         <v>43</v>
       </c>
       <c r="B47" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="C47" s="11" t="s">
         <v>63</v>
-      </c>
-      <c r="C47" s="11" t="s">
-        <v>64</v>
       </c>
       <c r="D47" s="13"/>
       <c r="E47" s="13"/>
       <c r="F47" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G47" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2205,18 +2205,18 @@
         <v>44</v>
       </c>
       <c r="B48" s="29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D48" s="13"/>
       <c r="E48" s="13"/>
       <c r="F48" s="14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G48" s="14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2224,18 +2224,18 @@
         <v>45</v>
       </c>
       <c r="B49" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="C49" s="11" t="s">
         <v>63</v>
-      </c>
-      <c r="C49" s="11" t="s">
-        <v>64</v>
       </c>
       <c r="D49" s="13"/>
       <c r="E49" s="13"/>
       <c r="F49" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G49" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2243,18 +2243,18 @@
         <v>46</v>
       </c>
       <c r="B50" s="29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D50" s="13"/>
       <c r="E50" s="13"/>
       <c r="F50" s="14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G50" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2262,18 +2262,18 @@
         <v>47</v>
       </c>
       <c r="B51" s="28" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D51" s="13"/>
       <c r="E51" s="13"/>
       <c r="F51" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G51" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2281,18 +2281,18 @@
         <v>48</v>
       </c>
       <c r="B52" s="29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D52" s="13"/>
       <c r="E52" s="13"/>
       <c r="F52" s="14" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G52" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2300,18 +2300,18 @@
         <v>49</v>
       </c>
       <c r="B53" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="C53" s="11" t="s">
         <v>68</v>
-      </c>
-      <c r="C53" s="11" t="s">
-        <v>69</v>
       </c>
       <c r="D53" s="13"/>
       <c r="E53" s="13"/>
       <c r="F53" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="G53" s="11" t="s">
         <v>70</v>
-      </c>
-      <c r="G53" s="11" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2319,18 +2319,18 @@
         <v>50</v>
       </c>
       <c r="B54" s="31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D54" s="13"/>
       <c r="E54" s="13"/>
       <c r="F54" s="14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G54" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2338,18 +2338,18 @@
         <v>51</v>
       </c>
       <c r="B55" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="C55" s="11" t="s">
         <v>68</v>
-      </c>
-      <c r="C55" s="11" t="s">
-        <v>69</v>
       </c>
       <c r="D55" s="13"/>
       <c r="E55" s="13"/>
       <c r="F55" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G55" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2357,18 +2357,18 @@
         <v>52</v>
       </c>
       <c r="B56" s="31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D56" s="13"/>
       <c r="E56" s="13"/>
       <c r="F56" s="14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G56" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2376,18 +2376,18 @@
         <v>53</v>
       </c>
       <c r="B57" s="30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C57" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D57" s="13"/>
       <c r="E57" s="13"/>
       <c r="F57" s="11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G57" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2395,18 +2395,18 @@
         <v>54</v>
       </c>
       <c r="B58" s="31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D58" s="13"/>
       <c r="E58" s="13"/>
       <c r="F58" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G58" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2414,18 +2414,18 @@
         <v>55</v>
       </c>
       <c r="B59" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="C59" s="11" t="s">
         <v>75</v>
-      </c>
-      <c r="C59" s="11" t="s">
-        <v>76</v>
       </c>
       <c r="D59" s="13"/>
       <c r="E59" s="13"/>
       <c r="F59" s="11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G59" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2433,18 +2433,18 @@
         <v>56</v>
       </c>
       <c r="B60" s="33" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C60" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D60" s="13"/>
       <c r="E60" s="13"/>
       <c r="F60" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G60" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2452,18 +2452,18 @@
         <v>57</v>
       </c>
       <c r="B61" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="C61" s="11" t="s">
         <v>75</v>
-      </c>
-      <c r="C61" s="11" t="s">
-        <v>76</v>
       </c>
       <c r="D61" s="13"/>
       <c r="E61" s="13"/>
       <c r="F61" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G61" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2471,18 +2471,18 @@
         <v>58</v>
       </c>
       <c r="B62" s="33" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C62" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D62" s="13"/>
       <c r="E62" s="13"/>
       <c r="F62" s="14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G62" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2490,18 +2490,18 @@
         <v>59</v>
       </c>
       <c r="B63" s="32" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C63" s="11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D63" s="13"/>
       <c r="E63" s="13"/>
       <c r="F63" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G63" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2509,18 +2509,18 @@
         <v>60</v>
       </c>
       <c r="B64" s="33" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C64" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D64" s="13"/>
       <c r="E64" s="13"/>
       <c r="F64" s="14" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G64" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2528,18 +2528,18 @@
         <v>61</v>
       </c>
       <c r="B65" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="C65" s="11" t="s">
         <v>81</v>
-      </c>
-      <c r="C65" s="11" t="s">
-        <v>82</v>
       </c>
       <c r="D65" s="13"/>
       <c r="E65" s="13"/>
       <c r="F65" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="G65" s="11" t="s">
         <v>83</v>
-      </c>
-      <c r="G65" s="11" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2547,18 +2547,18 @@
         <v>62</v>
       </c>
       <c r="B66" s="35" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D66" s="13"/>
       <c r="E66" s="13"/>
       <c r="F66" s="14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G66" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2566,18 +2566,18 @@
         <v>63</v>
       </c>
       <c r="B67" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="C67" s="11" t="s">
         <v>81</v>
-      </c>
-      <c r="C67" s="11" t="s">
-        <v>82</v>
       </c>
       <c r="D67" s="13"/>
       <c r="E67" s="13"/>
       <c r="F67" s="11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G67" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2585,18 +2585,18 @@
         <v>64</v>
       </c>
       <c r="B68" s="35" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C68" s="14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D68" s="13"/>
       <c r="E68" s="13"/>
       <c r="F68" s="14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G68" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2604,18 +2604,18 @@
         <v>65</v>
       </c>
       <c r="B69" s="34" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C69" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D69" s="13"/>
       <c r="E69" s="13"/>
       <c r="F69" s="11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G69" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2623,18 +2623,18 @@
         <v>66</v>
       </c>
       <c r="B70" s="35" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C70" s="14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D70" s="13"/>
       <c r="E70" s="13"/>
       <c r="F70" s="14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G70" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2642,18 +2642,18 @@
         <v>67</v>
       </c>
       <c r="B71" s="36" t="s">
+        <v>87</v>
+      </c>
+      <c r="C71" s="11" t="s">
         <v>88</v>
-      </c>
-      <c r="C71" s="11" t="s">
-        <v>89</v>
       </c>
       <c r="D71" s="13"/>
       <c r="E71" s="13"/>
       <c r="F71" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G71" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2661,18 +2661,18 @@
         <v>68</v>
       </c>
       <c r="B72" s="37" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C72" s="14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D72" s="13"/>
       <c r="E72" s="13"/>
       <c r="F72" s="14" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G72" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="73" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2680,18 +2680,18 @@
         <v>69</v>
       </c>
       <c r="B73" s="36" t="s">
+        <v>87</v>
+      </c>
+      <c r="C73" s="11" t="s">
         <v>88</v>
-      </c>
-      <c r="C73" s="11" t="s">
-        <v>89</v>
       </c>
       <c r="D73" s="13"/>
       <c r="E73" s="13"/>
       <c r="F73" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G73" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="74" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2699,18 +2699,18 @@
         <v>70</v>
       </c>
       <c r="B74" s="37" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C74" s="14" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D74" s="13"/>
       <c r="E74" s="13"/>
       <c r="F74" s="14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G74" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2718,18 +2718,18 @@
         <v>71</v>
       </c>
       <c r="B75" s="36" t="s">
+        <v>87</v>
+      </c>
+      <c r="C75" s="11" t="s">
         <v>88</v>
-      </c>
-      <c r="C75" s="11" t="s">
-        <v>89</v>
       </c>
       <c r="D75" s="13"/>
       <c r="E75" s="13"/>
       <c r="F75" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G75" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2737,18 +2737,18 @@
         <v>72</v>
       </c>
       <c r="B76" s="37" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C76" s="14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D76" s="13"/>
       <c r="E76" s="13"/>
       <c r="F76" s="14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G76" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -2773,78 +2773,78 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="46" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
+      <c r="M1" s="46"/>
+      <c r="N1" s="46"/>
+      <c r="O1" s="46"/>
+      <c r="P1" s="46"/>
+      <c r="Q1" s="46"/>
+      <c r="R1" s="46"/>
+      <c r="S1" s="46"/>
+      <c r="T1" s="46"/>
+      <c r="U1" s="46"/>
+      <c r="V1" s="46"/>
+      <c r="W1" s="46"/>
+      <c r="X1" s="46"/>
+      <c r="Y1" s="46"/>
+      <c r="Z1" s="46"/>
+      <c r="AA1" s="46"/>
+      <c r="AB1" s="46"/>
+      <c r="AC1" s="46"/>
+      <c r="AD1" s="46"/>
+      <c r="AE1" s="46"/>
+      <c r="AF1" s="46"/>
+      <c r="AG1" s="46"/>
+    </row>
+    <row r="2" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="45" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
-      <c r="K1" s="45"/>
-      <c r="L1" s="45"/>
-      <c r="M1" s="45"/>
-      <c r="N1" s="45"/>
-      <c r="O1" s="45"/>
-      <c r="P1" s="45"/>
-      <c r="Q1" s="45"/>
-      <c r="R1" s="45"/>
-      <c r="S1" s="45"/>
-      <c r="T1" s="45"/>
-      <c r="U1" s="45"/>
-      <c r="V1" s="45"/>
-      <c r="W1" s="45"/>
-      <c r="X1" s="45"/>
-      <c r="Y1" s="45"/>
-      <c r="Z1" s="45"/>
-      <c r="AA1" s="45"/>
-      <c r="AB1" s="45"/>
-      <c r="AC1" s="45"/>
-      <c r="AD1" s="45"/>
-      <c r="AE1" s="45"/>
-      <c r="AF1" s="45"/>
-      <c r="AG1" s="45"/>
-    </row>
-    <row r="2" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="46" t="s">
-        <v>94</v>
-      </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
-      <c r="N2" s="46"/>
-      <c r="O2" s="46"/>
-      <c r="P2" s="46"/>
-      <c r="Q2" s="46"/>
-      <c r="R2" s="46"/>
-      <c r="S2" s="46"/>
-      <c r="T2" s="46"/>
-      <c r="U2" s="46"/>
-      <c r="V2" s="46"/>
-      <c r="W2" s="46"/>
-      <c r="X2" s="46"/>
-      <c r="Y2" s="46"/>
-      <c r="Z2" s="46"/>
-      <c r="AA2" s="46"/>
-      <c r="AB2" s="46"/>
-      <c r="AC2" s="46"/>
-      <c r="AD2" s="46"/>
-      <c r="AE2" s="46"/>
-      <c r="AF2" s="46"/>
-      <c r="AG2" s="46"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="45"/>
+      <c r="P2" s="45"/>
+      <c r="Q2" s="45"/>
+      <c r="R2" s="45"/>
+      <c r="S2" s="45"/>
+      <c r="T2" s="45"/>
+      <c r="U2" s="45"/>
+      <c r="V2" s="45"/>
+      <c r="W2" s="45"/>
+      <c r="X2" s="45"/>
+      <c r="Y2" s="45"/>
+      <c r="Z2" s="45"/>
+      <c r="AA2" s="45"/>
+      <c r="AB2" s="45"/>
+      <c r="AC2" s="45"/>
+      <c r="AD2" s="45"/>
+      <c r="AE2" s="45"/>
+      <c r="AF2" s="45"/>
+      <c r="AG2" s="45"/>
     </row>
     <row r="3" spans="1:33" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2852,182 +2852,182 @@
         <v>2</v>
       </c>
       <c r="B4" s="38" t="s">
+        <v>94</v>
+      </c>
+      <c r="C4" s="39" t="s">
         <v>95</v>
       </c>
-      <c r="C4" s="39" t="s">
-        <v>96</v>
-      </c>
-      <c r="D4" s="44" t="str">
+      <c r="D4" s="47" t="str">
         <f>Participantes!B5</f>
         <v>Andres Jesús</v>
       </c>
-      <c r="E4" s="44"/>
-      <c r="F4" s="44" t="str">
+      <c r="E4" s="47"/>
+      <c r="F4" s="47" t="str">
         <f>Participantes!B6</f>
         <v>Leonardo Fabio</v>
       </c>
-      <c r="G4" s="44"/>
-      <c r="H4" s="44" t="str">
+      <c r="G4" s="47"/>
+      <c r="H4" s="47" t="str">
         <f>Participantes!B7</f>
         <v>Martha Cenidia</v>
       </c>
-      <c r="I4" s="44"/>
-      <c r="J4" s="44" t="str">
+      <c r="I4" s="47"/>
+      <c r="J4" s="47" t="str">
         <f>Participantes!B8</f>
         <v>Freddy Ramón</v>
       </c>
-      <c r="K4" s="44"/>
-      <c r="L4" s="44" t="str">
+      <c r="K4" s="47"/>
+      <c r="L4" s="47" t="str">
         <f>Participantes!B9</f>
         <v xml:space="preserve">Juan Camilo </v>
       </c>
-      <c r="M4" s="44"/>
-      <c r="N4" s="44" t="str">
+      <c r="M4" s="47"/>
+      <c r="N4" s="47" t="str">
         <f>Participantes!B10</f>
         <v xml:space="preserve">Juan David </v>
       </c>
-      <c r="O4" s="44"/>
-      <c r="P4" s="44" t="str">
+      <c r="O4" s="47"/>
+      <c r="P4" s="47" t="str">
         <f>Participantes!B11</f>
         <v>María Trinidad</v>
       </c>
-      <c r="Q4" s="44"/>
-      <c r="R4" s="44" t="str">
+      <c r="Q4" s="47"/>
+      <c r="R4" s="47" t="str">
         <f>Participantes!B12</f>
         <v xml:space="preserve">María Gabriela </v>
       </c>
-      <c r="S4" s="44"/>
-      <c r="T4" s="44" t="str">
+      <c r="S4" s="47"/>
+      <c r="T4" s="47" t="str">
         <f>Participantes!B13</f>
         <v>Laura Valentina</v>
       </c>
-      <c r="U4" s="44"/>
-      <c r="V4" s="44" t="str">
+      <c r="U4" s="47"/>
+      <c r="V4" s="47" t="str">
         <f>Participantes!B14</f>
         <v>Gloria Isabel</v>
       </c>
-      <c r="W4" s="44"/>
-      <c r="X4" s="44" t="str">
+      <c r="W4" s="47"/>
+      <c r="X4" s="47" t="str">
         <f>Participantes!B15</f>
         <v xml:space="preserve">María del Pilar </v>
       </c>
-      <c r="Y4" s="44"/>
-      <c r="Z4" s="44" t="str">
+      <c r="Y4" s="47"/>
+      <c r="Z4" s="47" t="str">
         <f>Participantes!B16</f>
         <v>Jaime Andres</v>
       </c>
-      <c r="AA4" s="44"/>
-      <c r="AB4" s="44" t="str">
+      <c r="AA4" s="47"/>
+      <c r="AB4" s="47" t="str">
         <f>Participantes!B17</f>
         <v>Cesar Lindarte</v>
       </c>
-      <c r="AC4" s="44"/>
-      <c r="AD4" s="44" t="str">
+      <c r="AC4" s="47"/>
+      <c r="AD4" s="47" t="str">
         <f>Participantes!B18</f>
-        <v>Participante 14</v>
-      </c>
-      <c r="AE4" s="44"/>
-      <c r="AF4" s="44" t="str">
+        <v>Andrea Carolina</v>
+      </c>
+      <c r="AE4" s="47"/>
+      <c r="AF4" s="47" t="str">
         <f>Participantes!B19</f>
         <v>Participante 15</v>
       </c>
-      <c r="AG4" s="44"/>
+      <c r="AG4" s="47"/>
     </row>
     <row r="5" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="40"/>
       <c r="B5" s="40"/>
       <c r="C5" s="41" t="s">
+        <v>96</v>
+      </c>
+      <c r="D5" s="42" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="42" t="s">
         <v>97</v>
       </c>
-      <c r="D5" s="42" t="s">
-        <v>88</v>
-      </c>
-      <c r="E5" s="42" t="s">
-        <v>98</v>
-      </c>
       <c r="F5" s="42" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G5" s="42" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H5" s="42" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I5" s="42" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J5" s="42" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K5" s="42" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="L5" s="42" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="M5" s="42" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="N5" s="42" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O5" s="42" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="P5" s="42" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Q5" s="42" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="R5" s="42" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="S5" s="42" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="T5" s="42" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="U5" s="42" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="V5" s="42" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="W5" s="42" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="X5" s="42" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Y5" s="42" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="Z5" s="42" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AA5" s="42" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AB5" s="42" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AC5" s="42" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AD5" s="42" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AE5" s="42" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AF5" s="42" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AG5" s="42" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:33" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -6224,6 +6224,7 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="Z4:AA4"/>
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AD4:AE4"/>
     <mergeCell ref="AF4:AG4"/>
@@ -6240,7 +6241,6 @@
     <mergeCell ref="T4:U4"/>
     <mergeCell ref="V4:W4"/>
     <mergeCell ref="X4:Y4"/>
-    <mergeCell ref="Z4:AA4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Actualizar - 06-27-sáb 20:58
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A75697AA-2B40-48FE-B862-06CACC04310F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDCCC5A2-4B34-41D7-95DA-FB645C488F1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -2721,12 +2721,12 @@
         <v>87</v>
       </c>
       <c r="C75" s="11" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D75" s="13"/>
       <c r="E75" s="13"/>
       <c r="F75" s="11" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="G75" s="11" t="s">
         <v>79</v>
@@ -6142,7 +6142,7 @@
       </c>
       <c r="B76" s="11" t="str">
         <f>Fixture!C75&amp;" vs "&amp;Fixture!F75</f>
-        <v>Inglaterra vs Panamá</v>
+        <v>Panamá vs Inglaterra</v>
       </c>
       <c r="C76" s="43" t="str">
         <f>IF(ISNUMBER(Fixture!D75),Fixture!D75&amp;"-"&amp;Fixture!E75,"")</f>
@@ -6224,6 +6224,7 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="X4:Y4"/>
     <mergeCell ref="Z4:AA4"/>
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AD4:AE4"/>
@@ -6240,7 +6241,6 @@
     <mergeCell ref="R4:S4"/>
     <mergeCell ref="T4:U4"/>
     <mergeCell ref="V4:W4"/>
-    <mergeCell ref="X4:Y4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Actualizar - 06-28-dom  9:44
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDCCC5A2-4B34-41D7-95DA-FB645C488F1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBDB6330-5876-4EA7-94E4-67DA0DECFDFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -58,9 +58,6 @@
     <t>Posición</t>
   </si>
   <si>
-    <t>Participante 15</t>
-  </si>
-  <si>
     <t>⚽  FIXTURE FASE DE GRUPOS — FIFA WORLD CUP 2026</t>
   </si>
   <si>
@@ -377,6 +374,9 @@
   </si>
   <si>
     <t>Andrea Carolina</t>
+  </si>
+  <si>
+    <t>Maria Camila</t>
   </si>
 </sst>
 </file>
@@ -1093,7 +1093,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C5" s="4">
         <v>0</v>
@@ -1108,7 +1108,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C6" s="8">
         <v>0</v>
@@ -1123,7 +1123,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C7" s="4">
         <v>0</v>
@@ -1138,7 +1138,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C8" s="8">
         <v>0</v>
@@ -1153,7 +1153,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C9" s="4">
         <v>0</v>
@@ -1168,7 +1168,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C10" s="8">
         <v>0</v>
@@ -1183,7 +1183,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C11" s="4">
         <v>0</v>
@@ -1198,7 +1198,7 @@
         <v>8</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C12" s="8">
         <v>0</v>
@@ -1213,7 +1213,7 @@
         <v>9</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C13" s="4">
         <v>0</v>
@@ -1228,7 +1228,7 @@
         <v>10</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C14" s="8">
         <v>0</v>
@@ -1243,7 +1243,7 @@
         <v>11</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C15" s="4">
         <v>0</v>
@@ -1258,7 +1258,7 @@
         <v>12</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C16" s="8">
         <v>0</v>
@@ -1273,7 +1273,7 @@
         <v>13</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C17" s="4">
         <v>0</v>
@@ -1288,7 +1288,7 @@
         <v>14</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C18" s="8">
         <v>0</v>
@@ -1303,7 +1303,7 @@
         <v>15</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>6</v>
+        <v>111</v>
       </c>
       <c r="C19" s="4">
         <v>0</v>
@@ -1339,7 +1339,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="46" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B1" s="46"/>
       <c r="C1" s="46"/>
@@ -1350,7 +1350,7 @@
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="45" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B2" s="45"/>
       <c r="C2" s="45"/>
@@ -1365,22 +1365,22 @@
         <v>2</v>
       </c>
       <c r="B4" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="D4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="E4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="F4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="G4" s="10" t="s">
         <v>13</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1388,18 +1388,18 @@
         <v>1</v>
       </c>
       <c r="B5" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="11" t="s">
         <v>15</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>16</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
       <c r="F5" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="11" t="s">
         <v>17</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1407,18 +1407,18 @@
         <v>2</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
       <c r="F6" s="14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1426,18 +1426,18 @@
         <v>3</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D7" s="13"/>
       <c r="E7" s="13"/>
       <c r="F7" s="11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1445,18 +1445,18 @@
         <v>4</v>
       </c>
       <c r="B8" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="14" t="s">
         <v>15</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>16</v>
       </c>
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
       <c r="F8" s="14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1464,18 +1464,18 @@
         <v>5</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D9" s="13"/>
       <c r="E9" s="13"/>
       <c r="F9" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1483,18 +1483,18 @@
         <v>6</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D10" s="13"/>
       <c r="E10" s="13"/>
       <c r="F10" s="14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1502,18 +1502,18 @@
         <v>7</v>
       </c>
       <c r="B11" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="11" t="s">
         <v>23</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>24</v>
       </c>
       <c r="D11" s="13"/>
       <c r="E11" s="13"/>
       <c r="F11" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="11" t="s">
         <v>25</v>
-      </c>
-      <c r="G11" s="11" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1521,18 +1521,18 @@
         <v>8</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D12" s="13"/>
       <c r="E12" s="13"/>
       <c r="F12" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" s="14" t="s">
         <v>28</v>
-      </c>
-      <c r="G12" s="14" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1540,18 +1540,18 @@
         <v>9</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D13" s="13"/>
       <c r="E13" s="13"/>
       <c r="F13" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1559,18 +1559,18 @@
         <v>10</v>
       </c>
       <c r="B14" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="14" t="s">
         <v>23</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>24</v>
       </c>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
       <c r="F14" s="14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1578,18 +1578,18 @@
         <v>11</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D15" s="13"/>
       <c r="E15" s="13"/>
       <c r="F15" s="11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1597,18 +1597,18 @@
         <v>12</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D16" s="13"/>
       <c r="E16" s="13"/>
       <c r="F16" s="14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G16" s="14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1616,18 +1616,18 @@
         <v>13</v>
       </c>
       <c r="B17" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="11" t="s">
         <v>30</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>31</v>
       </c>
       <c r="D17" s="13"/>
       <c r="E17" s="13"/>
       <c r="F17" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1635,18 +1635,18 @@
         <v>14</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D18" s="13"/>
       <c r="E18" s="13"/>
       <c r="F18" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G18" s="14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1654,18 +1654,18 @@
         <v>15</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D19" s="13"/>
       <c r="E19" s="13"/>
       <c r="F19" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1673,18 +1673,18 @@
         <v>16</v>
       </c>
       <c r="B20" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" s="14" t="s">
         <v>30</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>31</v>
       </c>
       <c r="D20" s="13"/>
       <c r="E20" s="13"/>
       <c r="F20" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G20" s="14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1692,18 +1692,18 @@
         <v>17</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D21" s="13"/>
       <c r="E21" s="13"/>
       <c r="F21" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1711,18 +1711,18 @@
         <v>18</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D22" s="13"/>
       <c r="E22" s="13"/>
       <c r="F22" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G22" s="14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1730,18 +1730,18 @@
         <v>19</v>
       </c>
       <c r="B23" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="C23" s="11" t="s">
         <v>36</v>
-      </c>
-      <c r="C23" s="11" t="s">
-        <v>37</v>
       </c>
       <c r="D23" s="13"/>
       <c r="E23" s="13"/>
       <c r="F23" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1749,18 +1749,18 @@
         <v>20</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D24" s="13"/>
       <c r="E24" s="13"/>
       <c r="F24" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G24" s="14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1768,18 +1768,18 @@
         <v>21</v>
       </c>
       <c r="B25" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="C25" s="11" t="s">
         <v>36</v>
-      </c>
-      <c r="C25" s="11" t="s">
-        <v>37</v>
       </c>
       <c r="D25" s="13"/>
       <c r="E25" s="13"/>
       <c r="F25" s="11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1787,18 +1787,18 @@
         <v>22</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D26" s="13"/>
       <c r="E26" s="13"/>
       <c r="F26" s="14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G26" s="14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1806,18 +1806,18 @@
         <v>23</v>
       </c>
       <c r="B27" s="20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D27" s="13"/>
       <c r="E27" s="13"/>
       <c r="F27" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1825,18 +1825,18 @@
         <v>24</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D28" s="13"/>
       <c r="E28" s="13"/>
       <c r="F28" s="14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G28" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1844,18 +1844,18 @@
         <v>25</v>
       </c>
       <c r="B29" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="C29" s="11" t="s">
         <v>42</v>
-      </c>
-      <c r="C29" s="11" t="s">
-        <v>43</v>
       </c>
       <c r="D29" s="13"/>
       <c r="E29" s="13"/>
       <c r="F29" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="G29" s="11" t="s">
         <v>44</v>
-      </c>
-      <c r="G29" s="11" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1863,18 +1863,18 @@
         <v>26</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D30" s="13"/>
       <c r="E30" s="13"/>
       <c r="F30" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G30" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1882,18 +1882,18 @@
         <v>27</v>
       </c>
       <c r="B31" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="C31" s="11" t="s">
         <v>42</v>
-      </c>
-      <c r="C31" s="11" t="s">
-        <v>43</v>
       </c>
       <c r="D31" s="13"/>
       <c r="E31" s="13"/>
       <c r="F31" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1901,18 +1901,18 @@
         <v>28</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D32" s="13"/>
       <c r="E32" s="13"/>
       <c r="F32" s="14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G32" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1920,18 +1920,18 @@
         <v>29</v>
       </c>
       <c r="B33" s="22" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D33" s="13"/>
       <c r="E33" s="13"/>
       <c r="F33" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1939,18 +1939,18 @@
         <v>30</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D34" s="13"/>
       <c r="E34" s="13"/>
       <c r="F34" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G34" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1958,18 +1958,18 @@
         <v>31</v>
       </c>
       <c r="B35" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="C35" s="11" t="s">
         <v>49</v>
-      </c>
-      <c r="C35" s="11" t="s">
-        <v>50</v>
       </c>
       <c r="D35" s="13"/>
       <c r="E35" s="13"/>
       <c r="F35" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1977,18 +1977,18 @@
         <v>32</v>
       </c>
       <c r="B36" s="25" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D36" s="13"/>
       <c r="E36" s="13"/>
       <c r="F36" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G36" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1996,18 +1996,18 @@
         <v>33</v>
       </c>
       <c r="B37" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="C37" s="11" t="s">
         <v>49</v>
-      </c>
-      <c r="C37" s="11" t="s">
-        <v>50</v>
       </c>
       <c r="D37" s="13"/>
       <c r="E37" s="13"/>
       <c r="F37" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2015,18 +2015,18 @@
         <v>34</v>
       </c>
       <c r="B38" s="25" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D38" s="13"/>
       <c r="E38" s="13"/>
       <c r="F38" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G38" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2034,18 +2034,18 @@
         <v>35</v>
       </c>
       <c r="B39" s="24" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D39" s="13"/>
       <c r="E39" s="13"/>
       <c r="F39" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2053,18 +2053,18 @@
         <v>36</v>
       </c>
       <c r="B40" s="25" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D40" s="13"/>
       <c r="E40" s="13"/>
       <c r="F40" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2072,18 +2072,18 @@
         <v>37</v>
       </c>
       <c r="B41" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="C41" s="11" t="s">
         <v>54</v>
-      </c>
-      <c r="C41" s="11" t="s">
-        <v>55</v>
       </c>
       <c r="D41" s="13"/>
       <c r="E41" s="13"/>
       <c r="F41" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="G41" s="11" t="s">
         <v>56</v>
-      </c>
-      <c r="G41" s="11" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2091,18 +2091,18 @@
         <v>38</v>
       </c>
       <c r="B42" s="27" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D42" s="13"/>
       <c r="E42" s="13"/>
       <c r="F42" s="14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2110,18 +2110,18 @@
         <v>39</v>
       </c>
       <c r="B43" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="C43" s="11" t="s">
         <v>54</v>
-      </c>
-      <c r="C43" s="11" t="s">
-        <v>55</v>
       </c>
       <c r="D43" s="13"/>
       <c r="E43" s="13"/>
       <c r="F43" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G43" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2129,18 +2129,18 @@
         <v>40</v>
       </c>
       <c r="B44" s="27" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D44" s="13"/>
       <c r="E44" s="13"/>
       <c r="F44" s="14" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G44" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2148,18 +2148,18 @@
         <v>41</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D45" s="13"/>
       <c r="E45" s="13"/>
       <c r="F45" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G45" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2167,18 +2167,18 @@
         <v>42</v>
       </c>
       <c r="B46" s="27" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D46" s="13"/>
       <c r="E46" s="13"/>
       <c r="F46" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G46" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2186,18 +2186,18 @@
         <v>43</v>
       </c>
       <c r="B47" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="C47" s="11" t="s">
         <v>62</v>
-      </c>
-      <c r="C47" s="11" t="s">
-        <v>63</v>
       </c>
       <c r="D47" s="13"/>
       <c r="E47" s="13"/>
       <c r="F47" s="11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G47" s="11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2205,18 +2205,18 @@
         <v>44</v>
       </c>
       <c r="B48" s="29" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D48" s="13"/>
       <c r="E48" s="13"/>
       <c r="F48" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G48" s="14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2224,18 +2224,18 @@
         <v>45</v>
       </c>
       <c r="B49" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="C49" s="11" t="s">
         <v>62</v>
-      </c>
-      <c r="C49" s="11" t="s">
-        <v>63</v>
       </c>
       <c r="D49" s="13"/>
       <c r="E49" s="13"/>
       <c r="F49" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G49" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2243,18 +2243,18 @@
         <v>46</v>
       </c>
       <c r="B50" s="29" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D50" s="13"/>
       <c r="E50" s="13"/>
       <c r="F50" s="14" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G50" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2262,18 +2262,18 @@
         <v>47</v>
       </c>
       <c r="B51" s="28" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D51" s="13"/>
       <c r="E51" s="13"/>
       <c r="F51" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G51" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2281,18 +2281,18 @@
         <v>48</v>
       </c>
       <c r="B52" s="29" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D52" s="13"/>
       <c r="E52" s="13"/>
       <c r="F52" s="14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G52" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2300,18 +2300,18 @@
         <v>49</v>
       </c>
       <c r="B53" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="C53" s="11" t="s">
         <v>67</v>
-      </c>
-      <c r="C53" s="11" t="s">
-        <v>68</v>
       </c>
       <c r="D53" s="13"/>
       <c r="E53" s="13"/>
       <c r="F53" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="G53" s="11" t="s">
         <v>69</v>
-      </c>
-      <c r="G53" s="11" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2319,18 +2319,18 @@
         <v>50</v>
       </c>
       <c r="B54" s="31" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D54" s="13"/>
       <c r="E54" s="13"/>
       <c r="F54" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G54" s="14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2338,18 +2338,18 @@
         <v>51</v>
       </c>
       <c r="B55" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="C55" s="11" t="s">
         <v>67</v>
-      </c>
-      <c r="C55" s="11" t="s">
-        <v>68</v>
       </c>
       <c r="D55" s="13"/>
       <c r="E55" s="13"/>
       <c r="F55" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G55" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2357,18 +2357,18 @@
         <v>52</v>
       </c>
       <c r="B56" s="31" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D56" s="13"/>
       <c r="E56" s="13"/>
       <c r="F56" s="14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G56" s="14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2376,18 +2376,18 @@
         <v>53</v>
       </c>
       <c r="B57" s="30" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C57" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D57" s="13"/>
       <c r="E57" s="13"/>
       <c r="F57" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G57" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2395,18 +2395,18 @@
         <v>54</v>
       </c>
       <c r="B58" s="31" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D58" s="13"/>
       <c r="E58" s="13"/>
       <c r="F58" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G58" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2414,18 +2414,18 @@
         <v>55</v>
       </c>
       <c r="B59" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="C59" s="11" t="s">
         <v>74</v>
-      </c>
-      <c r="C59" s="11" t="s">
-        <v>75</v>
       </c>
       <c r="D59" s="13"/>
       <c r="E59" s="13"/>
       <c r="F59" s="11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G59" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2433,18 +2433,18 @@
         <v>56</v>
       </c>
       <c r="B60" s="33" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C60" s="14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D60" s="13"/>
       <c r="E60" s="13"/>
       <c r="F60" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G60" s="14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2452,18 +2452,18 @@
         <v>57</v>
       </c>
       <c r="B61" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="C61" s="11" t="s">
         <v>74</v>
-      </c>
-      <c r="C61" s="11" t="s">
-        <v>75</v>
       </c>
       <c r="D61" s="13"/>
       <c r="E61" s="13"/>
       <c r="F61" s="11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G61" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2471,18 +2471,18 @@
         <v>58</v>
       </c>
       <c r="B62" s="33" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C62" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D62" s="13"/>
       <c r="E62" s="13"/>
       <c r="F62" s="14" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G62" s="14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2490,18 +2490,18 @@
         <v>59</v>
       </c>
       <c r="B63" s="32" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C63" s="11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D63" s="13"/>
       <c r="E63" s="13"/>
       <c r="F63" s="11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G63" s="11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2509,18 +2509,18 @@
         <v>60</v>
       </c>
       <c r="B64" s="33" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C64" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D64" s="13"/>
       <c r="E64" s="13"/>
       <c r="F64" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G64" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2528,18 +2528,18 @@
         <v>61</v>
       </c>
       <c r="B65" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="C65" s="11" t="s">
         <v>80</v>
-      </c>
-      <c r="C65" s="11" t="s">
-        <v>81</v>
       </c>
       <c r="D65" s="13"/>
       <c r="E65" s="13"/>
       <c r="F65" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="G65" s="11" t="s">
         <v>82</v>
-      </c>
-      <c r="G65" s="11" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2547,18 +2547,18 @@
         <v>62</v>
       </c>
       <c r="B66" s="35" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D66" s="13"/>
       <c r="E66" s="13"/>
       <c r="F66" s="14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G66" s="14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2566,18 +2566,18 @@
         <v>63</v>
       </c>
       <c r="B67" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="C67" s="11" t="s">
         <v>80</v>
-      </c>
-      <c r="C67" s="11" t="s">
-        <v>81</v>
       </c>
       <c r="D67" s="13"/>
       <c r="E67" s="13"/>
       <c r="F67" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G67" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2585,18 +2585,18 @@
         <v>64</v>
       </c>
       <c r="B68" s="35" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C68" s="14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D68" s="13"/>
       <c r="E68" s="13"/>
       <c r="F68" s="14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G68" s="14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2604,18 +2604,18 @@
         <v>65</v>
       </c>
       <c r="B69" s="34" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C69" s="11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D69" s="13"/>
       <c r="E69" s="13"/>
       <c r="F69" s="11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G69" s="11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2623,18 +2623,18 @@
         <v>66</v>
       </c>
       <c r="B70" s="35" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C70" s="14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D70" s="13"/>
       <c r="E70" s="13"/>
       <c r="F70" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G70" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2642,18 +2642,18 @@
         <v>67</v>
       </c>
       <c r="B71" s="36" t="s">
+        <v>86</v>
+      </c>
+      <c r="C71" s="11" t="s">
         <v>87</v>
-      </c>
-      <c r="C71" s="11" t="s">
-        <v>88</v>
       </c>
       <c r="D71" s="13"/>
       <c r="E71" s="13"/>
       <c r="F71" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G71" s="11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2661,18 +2661,18 @@
         <v>68</v>
       </c>
       <c r="B72" s="37" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C72" s="14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D72" s="13"/>
       <c r="E72" s="13"/>
       <c r="F72" s="14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G72" s="14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="73" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2680,18 +2680,18 @@
         <v>69</v>
       </c>
       <c r="B73" s="36" t="s">
+        <v>86</v>
+      </c>
+      <c r="C73" s="11" t="s">
         <v>87</v>
-      </c>
-      <c r="C73" s="11" t="s">
-        <v>88</v>
       </c>
       <c r="D73" s="13"/>
       <c r="E73" s="13"/>
       <c r="F73" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G73" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="74" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2699,18 +2699,18 @@
         <v>70</v>
       </c>
       <c r="B74" s="37" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C74" s="14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D74" s="13"/>
       <c r="E74" s="13"/>
       <c r="F74" s="14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G74" s="14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2718,18 +2718,18 @@
         <v>71</v>
       </c>
       <c r="B75" s="36" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C75" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D75" s="13"/>
       <c r="E75" s="13"/>
       <c r="F75" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G75" s="11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2737,18 +2737,18 @@
         <v>72</v>
       </c>
       <c r="B76" s="37" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C76" s="14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D76" s="13"/>
       <c r="E76" s="13"/>
       <c r="F76" s="14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G76" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -2774,7 +2774,7 @@
   <sheetData>
     <row r="1" spans="1:33" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="46" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B1" s="46"/>
       <c r="C1" s="46"/>
@@ -2811,7 +2811,7 @@
     </row>
     <row r="2" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="45" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B2" s="45"/>
       <c r="C2" s="45"/>
@@ -2852,10 +2852,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="38" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" s="39" t="s">
         <v>94</v>
-      </c>
-      <c r="C4" s="39" t="s">
-        <v>95</v>
       </c>
       <c r="D4" s="47" t="str">
         <f>Participantes!B5</f>
@@ -2929,7 +2929,7 @@
       <c r="AE4" s="47"/>
       <c r="AF4" s="47" t="str">
         <f>Participantes!B19</f>
-        <v>Participante 15</v>
+        <v>Maria Camila</v>
       </c>
       <c r="AG4" s="47"/>
     </row>
@@ -2937,97 +2937,97 @@
       <c r="A5" s="40"/>
       <c r="B5" s="40"/>
       <c r="C5" s="41" t="s">
+        <v>95</v>
+      </c>
+      <c r="D5" s="42" t="s">
+        <v>86</v>
+      </c>
+      <c r="E5" s="42" t="s">
         <v>96</v>
       </c>
-      <c r="D5" s="42" t="s">
-        <v>87</v>
-      </c>
-      <c r="E5" s="42" t="s">
-        <v>97</v>
-      </c>
       <c r="F5" s="42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G5" s="42" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H5" s="42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I5" s="42" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J5" s="42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="K5" s="42" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L5" s="42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="M5" s="42" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="N5" s="42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O5" s="42" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="P5" s="42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Q5" s="42" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="R5" s="42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="S5" s="42" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="T5" s="42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="U5" s="42" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="V5" s="42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="W5" s="42" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="X5" s="42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Y5" s="42" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="Z5" s="42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA5" s="42" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="AB5" s="42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AC5" s="42" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="AD5" s="42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AE5" s="42" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="AF5" s="42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AG5" s="42" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" spans="1:33" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualizar - 07-05-dom 11:00
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_v2.xlsx
+++ b/Quiniela_Mundial_2026_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\MIOS\polla mundialista github\polla-mundialista-pocheche\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBDB6330-5876-4EA7-94E4-67DA0DECFDFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B0AD6A0-2B92-4A13-9497-62EDFF577F66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1125" yWindow="1125" windowWidth="21600" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -352,9 +352,6 @@
     <t xml:space="preserve">Juan David </t>
   </si>
   <si>
-    <t>María Trinidad</t>
-  </si>
-  <si>
     <t xml:space="preserve">María Gabriela </t>
   </si>
   <si>
@@ -377,6 +374,9 @@
   </si>
   <si>
     <t>Maria Camila</t>
+  </si>
+  <si>
+    <t>José David</t>
   </si>
 </sst>
 </file>
@@ -1183,7 +1183,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C11" s="4">
         <v>0</v>
@@ -1198,7 +1198,7 @@
         <v>8</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C12" s="8">
         <v>0</v>
@@ -1213,7 +1213,7 @@
         <v>9</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C13" s="4">
         <v>0</v>
@@ -1228,7 +1228,7 @@
         <v>10</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C14" s="8">
         <v>0</v>
@@ -1243,7 +1243,7 @@
         <v>11</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C15" s="4">
         <v>0</v>
@@ -1258,7 +1258,7 @@
         <v>12</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C16" s="8">
         <v>0</v>
@@ -1273,7 +1273,7 @@
         <v>13</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C17" s="4">
         <v>0</v>
@@ -1288,7 +1288,7 @@
         <v>14</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C18" s="8">
         <v>0</v>
@@ -1303,7 +1303,7 @@
         <v>15</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C19" s="4">
         <v>0</v>
@@ -2889,7 +2889,7 @@
       <c r="O4" s="47"/>
       <c r="P4" s="47" t="str">
         <f>Participantes!B11</f>
-        <v>María Trinidad</v>
+        <v>José David</v>
       </c>
       <c r="Q4" s="47"/>
       <c r="R4" s="47" t="str">
@@ -6224,11 +6224,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="X4:Y4"/>
-    <mergeCell ref="Z4:AA4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AD4:AE4"/>
-    <mergeCell ref="AF4:AG4"/>
     <mergeCell ref="A1:AG1"/>
     <mergeCell ref="A2:AG2"/>
     <mergeCell ref="D4:E4"/>
@@ -6241,6 +6236,11 @@
     <mergeCell ref="R4:S4"/>
     <mergeCell ref="T4:U4"/>
     <mergeCell ref="V4:W4"/>
+    <mergeCell ref="X4:Y4"/>
+    <mergeCell ref="Z4:AA4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AD4:AE4"/>
+    <mergeCell ref="AF4:AG4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>